<commit_message>
Actualización automática 2026-01-21 13:30:11
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R66"/>
+  <dimension ref="A1:R67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3354,10 +3354,10 @@
         <v>0</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>421.72</v>
+        <v>0</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>36.44</v>
+        <v>0</v>
       </c>
       <c r="N48" s="2" t="n">
         <v>0</v>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PAREDES POVEDA TATIANA VERONICA</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>0</v>
+        <v>421.72</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>0</v>
+        <v>36.44</v>
       </c>
       <c r="N49" s="2" t="n">
         <v>0</v>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PAREDES POVEDA TATIANA VERONICA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,14 +3683,14 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>679.55</v>
+        <v>0</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>0</v>
@@ -3743,14 +3743,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>0</v>
+        <v>679.55</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>0</v>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,137 +4343,197 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R65" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R65" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>0 de 64</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>2 de 64</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="inlineStr">
-        <is>
-          <t>0 de 64</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>0 de 64</t>
-        </is>
-      </c>
-      <c r="G66" s="3" t="inlineStr">
-        <is>
-          <t>0 de 64</t>
-        </is>
-      </c>
-      <c r="H66" s="3" t="inlineStr">
-        <is>
-          <t>1 de 64</t>
-        </is>
-      </c>
-      <c r="I66" s="3" t="inlineStr">
-        <is>
-          <t>1 de 64</t>
-        </is>
-      </c>
-      <c r="J66" s="3" t="inlineStr">
-        <is>
-          <t>0 de 64</t>
-        </is>
-      </c>
-      <c r="K66" s="3" t="inlineStr">
-        <is>
-          <t>0 de 64</t>
-        </is>
-      </c>
-      <c r="L66" s="3" t="inlineStr">
-        <is>
-          <t>2 de 64</t>
-        </is>
-      </c>
-      <c r="M66" s="3" t="inlineStr">
-        <is>
-          <t>3 de 64</t>
-        </is>
-      </c>
-      <c r="N66" s="3" t="inlineStr">
-        <is>
-          <t>0 de 64</t>
-        </is>
-      </c>
-      <c r="O66" s="3" t="inlineStr">
-        <is>
-          <t>0 de 64</t>
-        </is>
-      </c>
-      <c r="P66" s="3" t="inlineStr">
-        <is>
-          <t>1 de 64</t>
-        </is>
-      </c>
-      <c r="Q66" s="3" t="inlineStr">
-        <is>
-          <t>0 de 64</t>
-        </is>
-      </c>
-      <c r="R66" s="3" t="inlineStr">
-        <is>
-          <t>0 de 64</t>
+      <c r="C66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R66" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>0 de 65</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>2 de 65</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>0 de 65</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>0 de 65</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>0 de 65</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>1 de 65</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>1 de 65</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>0 de 65</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>0 de 65</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t>2 de 65</t>
+        </is>
+      </c>
+      <c r="M67" s="3" t="inlineStr">
+        <is>
+          <t>3 de 65</t>
+        </is>
+      </c>
+      <c r="N67" s="3" t="inlineStr">
+        <is>
+          <t>0 de 65</t>
+        </is>
+      </c>
+      <c r="O67" s="3" t="inlineStr">
+        <is>
+          <t>0 de 65</t>
+        </is>
+      </c>
+      <c r="P67" s="3" t="inlineStr">
+        <is>
+          <t>1 de 65</t>
+        </is>
+      </c>
+      <c r="Q67" s="3" t="inlineStr">
+        <is>
+          <t>0 de 65</t>
+        </is>
+      </c>
+      <c r="R67" s="3" t="inlineStr">
+        <is>
+          <t>0 de 65</t>
         </is>
       </c>
     </row>
@@ -4488,7 +4548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5760,14 +5820,14 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>450.22</v>
+        <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>0</v>
@@ -5787,20 +5847,20 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>179.12</v>
+        <v>0</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>517.0599999999999</v>
+        <v>450.22</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>408.89</v>
+        <v>0</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>458.16</v>
+        <v>0</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>0</v>
@@ -5814,20 +5874,20 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PAREDES POVEDA TATIANA VERONICA</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>0</v>
+        <v>179.12</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0</v>
+        <v>517.0599999999999</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0</v>
+        <v>408.89</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0</v>
+        <v>458.16</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>0</v>
@@ -5841,7 +5901,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PAREDES POVEDA TATIANA VERONICA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -5851,7 +5911,7 @@
         <v>0</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>137.52</v>
+        <v>0</v>
       </c>
       <c r="F50" s="2" t="n">
         <v>0</v>
@@ -5868,17 +5928,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>503.15</v>
+        <v>0</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>0</v>
+        <v>137.52</v>
       </c>
       <c r="F51" s="2" t="n">
         <v>0</v>
@@ -5895,14 +5955,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>0</v>
+        <v>503.15</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>0</v>
@@ -5922,7 +5982,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -5949,20 +6009,20 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>194.16</v>
+        <v>0</v>
       </c>
       <c r="D54" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>2857.01</v>
+        <v>0</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>679.55</v>
+        <v>0</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>0</v>
@@ -5976,20 +6036,20 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>0</v>
+        <v>194.16</v>
       </c>
       <c r="D55" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0</v>
+        <v>2857.01</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>0</v>
+        <v>679.55</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>0</v>
@@ -6003,7 +6063,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -6030,7 +6090,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -6057,11 +6117,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>334.37</v>
+        <v>0</v>
       </c>
       <c r="D58" s="2" t="n">
         <v>0</v>
@@ -6084,11 +6144,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>0</v>
+        <v>334.37</v>
       </c>
       <c r="D59" s="2" t="n">
         <v>0</v>
@@ -6111,7 +6171,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -6121,7 +6181,7 @@
         <v>0</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>1144.09</v>
+        <v>0</v>
       </c>
       <c r="F60" s="2" t="n">
         <v>0</v>
@@ -6138,17 +6198,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>944.42</v>
+        <v>0</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>537.98</v>
+        <v>1144.09</v>
       </c>
       <c r="F61" s="2" t="n">
         <v>0</v>
@@ -6165,17 +6225,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>0</v>
+        <v>944.42</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0</v>
+        <v>537.98</v>
       </c>
       <c r="F62" s="2" t="n">
         <v>0</v>
@@ -6192,7 +6252,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -6219,7 +6279,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -6229,7 +6289,7 @@
         <v>0</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>281.46</v>
+        <v>0</v>
       </c>
       <c r="F64" s="2" t="n">
         <v>0</v>
@@ -6246,39 +6306,66 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>281.46</v>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G65" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="C66" s="4" t="n">
+      <c r="C66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="C67" s="4" t="n">
         <v>574.9</v>
       </c>
-      <c r="D66" s="4" t="n">
+      <c r="D67" s="4" t="n">
         <v>6694.99</v>
       </c>
-      <c r="E66" s="4" t="n">
+      <c r="E67" s="4" t="n">
         <v>8555.65</v>
       </c>
-      <c r="F66" s="4" t="n">
+      <c r="F67" s="4" t="n">
         <v>7044.440000000001</v>
       </c>
-      <c r="G66" s="4" t="n">
+      <c r="G67" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-01-22 15:30:12
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -6462,10 +6462,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4807.71</v>
+        <v>5109.94</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-4807.71</v>
+        <v>-5109.94</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -6529,13 +6529,13 @@
         <v>20532.82</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7282.210000000001</v>
+        <v>7584.440000000001</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>13250.61</v>
+        <v>12948.38</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.3546619509643586</v>
+        <v>0.3693813124548893</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-01-27 17:30:13
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -6486,13 +6486,13 @@
         <v>20000</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2017.5</v>
+        <v>2665.51</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>17982.5</v>
+        <v>17334.49</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.100875</v>
+        <v>0.1332755</v>
       </c>
     </row>
     <row r="5">
@@ -6529,13 +6529,13 @@
         <v>20532.82</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7848.48</v>
+        <v>8496.49</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>12684.34</v>
+        <v>12036.33</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.3822407248492901</v>
+        <v>0.4138004424136578</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-06 11:30:12
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -6549,10 +6549,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>3053.06</v>
+        <v>3074.64</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-3053.06</v>
+        <v>-3074.64</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -6616,13 +6616,13 @@
         <v>15532.82</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>5725.299999999999</v>
+        <v>5746.879999999999</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>9807.52</v>
+        <v>9785.940000000001</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.3685937260587581</v>
+        <v>0.3699830423580521</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-13 17:30:20
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -6549,10 +6549,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>3907.16</v>
+        <v>3994.12</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-3907.16</v>
+        <v>-3994.12</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -6616,13 +6616,13 @@
         <v>15532.82</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>6579.4</v>
+        <v>6666.36</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>8953.42</v>
+        <v>8866.460000000001</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.4235805217597319</v>
+        <v>0.429178990035293</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-20 12:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R69"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,137 +4523,197 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R68" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R68" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="C69" s="3" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="E69" s="3" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="F69" s="3" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="G69" s="3" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="H69" s="3" t="inlineStr">
-        <is>
-          <t>1 de 67</t>
-        </is>
-      </c>
-      <c r="I69" s="3" t="inlineStr">
-        <is>
-          <t>1 de 67</t>
-        </is>
-      </c>
-      <c r="J69" s="3" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="K69" s="3" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="L69" s="3" t="inlineStr">
-        <is>
-          <t>2 de 67</t>
-        </is>
-      </c>
-      <c r="M69" s="3" t="inlineStr">
-        <is>
-          <t>1 de 67</t>
-        </is>
-      </c>
-      <c r="N69" s="3" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="O69" s="3" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="P69" s="3" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="Q69" s="3" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="R69" s="3" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
+      <c r="C69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R69" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>0 de 68</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>0 de 68</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>0 de 68</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>0 de 68</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>0 de 68</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>1 de 68</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>1 de 68</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>0 de 68</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>0 de 68</t>
+        </is>
+      </c>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t>2 de 68</t>
+        </is>
+      </c>
+      <c r="M70" s="3" t="inlineStr">
+        <is>
+          <t>1 de 68</t>
+        </is>
+      </c>
+      <c r="N70" s="3" t="inlineStr">
+        <is>
+          <t>0 de 68</t>
+        </is>
+      </c>
+      <c r="O70" s="3" t="inlineStr">
+        <is>
+          <t>0 de 68</t>
+        </is>
+      </c>
+      <c r="P70" s="3" t="inlineStr">
+        <is>
+          <t>0 de 68</t>
+        </is>
+      </c>
+      <c r="Q70" s="3" t="inlineStr">
+        <is>
+          <t>0 de 68</t>
+        </is>
+      </c>
+      <c r="R70" s="3" t="inlineStr">
+        <is>
+          <t>0 de 68</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6318,7 +6378,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -6345,7 +6405,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -6372,14 +6432,14 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>1144.09</v>
+        <v>0</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>0</v>
@@ -6399,14 +6459,14 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>944.42</v>
+        <v>0</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>537.98</v>
+        <v>1144.09</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>0</v>
@@ -6426,14 +6486,14 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>0</v>
+        <v>944.42</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0</v>
+        <v>537.98</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>0</v>
@@ -6453,7 +6513,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -6480,14 +6540,14 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>281.46</v>
+        <v>0</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>0</v>
@@ -6507,39 +6567,66 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>281.46</v>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G68" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="C69" s="4" t="n">
+      <c r="C69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="C70" s="4" t="n">
         <v>6694.99</v>
       </c>
-      <c r="D69" s="4" t="n">
+      <c r="D70" s="4" t="n">
         <v>8555.65</v>
       </c>
-      <c r="E69" s="4" t="n">
+      <c r="E70" s="4" t="n">
         <v>8147.21</v>
       </c>
-      <c r="F69" s="4" t="n">
+      <c r="F70" s="4" t="n">
         <v>1608.51</v>
       </c>
-      <c r="G69" s="4" t="n">
+      <c r="G70" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-02-23 12:30:22
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -6723,10 +6723,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4927.05</v>
+        <v>4961.61</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-4927.05</v>
+        <v>-4961.61</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -6790,13 +6790,13 @@
         <v>15532.82</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7918.08</v>
+        <v>7952.639999999999</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>7614.739999999999</v>
+        <v>7580.179999999999</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.5097644857791438</v>
+        <v>0.5119894520119335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-25 15:30:22
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
+          <t>BURGOS OLVERA VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1554,7 +1554,7 @@
         <v>0</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>84.75</v>
+        <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
         <v>0</v>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1614,7 +1614,7 @@
         <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>0</v>
+        <v>84.75</v>
       </c>
       <c r="M19" s="2" t="n">
         <v>0</v>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CORONADO MONTERO LIDA VERONICA</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CORREA IGLESIAS RAMIRO MARCELO</t>
+          <t>CORONADO MONTERO LIDA VERONICA</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>CORREA IGLESIAS RAMIRO MARCELO</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1842,10 +1842,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>497.7</v>
+        <v>0</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>207.42</v>
+        <v>0</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0</v>
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>-23.01</v>
+        <v>0</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1902,10 +1902,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>0</v>
+        <v>497.7</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0</v>
+        <v>207.42</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0</v>
@@ -1917,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>-23.01</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GARCIA BRAVO JOSE LUIS</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>GAVILANES VELEZ MARIA VALERIA</t>
+          <t>GARCIA BRAVO JOSE LUIS</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GRANJA VANEGAS MARCELA</t>
+          <t>GAVILANES VELEZ MARIA VALERIA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GRANJA VANEGAS MARCELA</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>IDEARQ ESTUDIO S.A.S.</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>IDEARQ ESTUDIO S.A.S.</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>KITCHENSCO S.A.</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
+          <t>KITCHENSCO S.A.</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PAREDES POVEDA TATIANA VERONICA</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PAREDES POVEDA TATIANA VERONICA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,137 +4583,197 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R69" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R69" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="C70" s="3" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="E70" s="3" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="F70" s="3" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="G70" s="3" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="H70" s="3" t="inlineStr">
-        <is>
-          <t>1 de 68</t>
-        </is>
-      </c>
-      <c r="I70" s="3" t="inlineStr">
-        <is>
-          <t>1 de 68</t>
-        </is>
-      </c>
-      <c r="J70" s="3" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="K70" s="3" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="L70" s="3" t="inlineStr">
-        <is>
-          <t>2 de 68</t>
-        </is>
-      </c>
-      <c r="M70" s="3" t="inlineStr">
-        <is>
-          <t>1 de 68</t>
-        </is>
-      </c>
-      <c r="N70" s="3" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="O70" s="3" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="P70" s="3" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="Q70" s="3" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="R70" s="3" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
+      <c r="C70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R70" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>0 de 69</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>0 de 69</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>0 de 69</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>0 de 69</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>0 de 69</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>1 de 69</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>1 de 69</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>0 de 69</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>0 de 69</t>
+        </is>
+      </c>
+      <c r="L71" s="3" t="inlineStr">
+        <is>
+          <t>2 de 69</t>
+        </is>
+      </c>
+      <c r="M71" s="3" t="inlineStr">
+        <is>
+          <t>1 de 69</t>
+        </is>
+      </c>
+      <c r="N71" s="3" t="inlineStr">
+        <is>
+          <t>0 de 69</t>
+        </is>
+      </c>
+      <c r="O71" s="3" t="inlineStr">
+        <is>
+          <t>0 de 69</t>
+        </is>
+      </c>
+      <c r="P71" s="3" t="inlineStr">
+        <is>
+          <t>0 de 69</t>
+        </is>
+      </c>
+      <c r="Q71" s="3" t="inlineStr">
+        <is>
+          <t>0 de 69</t>
+        </is>
+      </c>
+      <c r="R71" s="3" t="inlineStr">
+        <is>
+          <t>0 de 69</t>
         </is>
       </c>
     </row>
@@ -4728,7 +4788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5163,7 +5223,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
+          <t>BURGOS OLVERA VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -5190,7 +5250,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -5217,7 +5277,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -5227,10 +5287,10 @@
         <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>381.36</v>
+        <v>0</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>84.75</v>
+        <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>0</v>
@@ -5244,7 +5304,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -5254,10 +5314,10 @@
         <v>0</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0</v>
+        <v>381.36</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0</v>
+        <v>84.75</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>0</v>
@@ -5271,7 +5331,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CORONADO MONTERO LIDA VERONICA</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -5298,7 +5358,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CORREA IGLESIAS RAMIRO MARCELO</t>
+          <t>CORONADO MONTERO LIDA VERONICA</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -5325,7 +5385,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>CORREA IGLESIAS RAMIRO MARCELO</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -5352,20 +5412,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>3669.5</v>
+        <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>968.04</v>
+        <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>5185.61</v>
+        <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>682.11</v>
+        <v>0</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -5379,20 +5439,20 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0</v>
+        <v>3669.5</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0</v>
+        <v>968.04</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0</v>
+        <v>5185.61</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0</v>
+        <v>682.11</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>0</v>
@@ -5406,7 +5466,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -5416,7 +5476,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>67.03</v>
+        <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>0</v>
@@ -5433,7 +5493,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -5443,7 +5503,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>17.26</v>
+        <v>67.03</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>0</v>
@@ -5460,7 +5520,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -5470,7 +5530,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0</v>
+        <v>17.26</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>0</v>
@@ -5487,7 +5547,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -5514,7 +5574,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GARCIA BRAVO JOSE LUIS</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -5541,7 +5601,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>GAVILANES VELEZ MARIA VALERIA</t>
+          <t>GARCIA BRAVO JOSE LUIS</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -5568,7 +5628,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GRANJA VANEGAS MARCELA</t>
+          <t>GAVILANES VELEZ MARIA VALERIA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -5595,14 +5655,14 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GRANJA VANEGAS MARCELA</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>393.88</v>
+        <v>0</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>65.66</v>
+        <v>0</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>0</v>
@@ -5622,14 +5682,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>IDEARQ ESTUDIO S.A.S.</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0</v>
+        <v>393.88</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0</v>
+        <v>65.66</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>0</v>
@@ -5649,7 +5709,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>IDEARQ ESTUDIO S.A.S.</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -5676,7 +5736,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -5703,7 +5763,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -5730,7 +5790,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>KITCHENSCO S.A.</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -5757,7 +5817,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
+          <t>KITCHENSCO S.A.</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -5784,11 +5844,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>216.76</v>
+        <v>0</v>
       </c>
       <c r="D39" s="2" t="n">
         <v>0</v>
@@ -5811,11 +5871,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>0</v>
+        <v>216.76</v>
       </c>
       <c r="D40" s="2" t="n">
         <v>0</v>
@@ -5838,7 +5898,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -5848,7 +5908,7 @@
         <v>0</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>369.48</v>
+        <v>0</v>
       </c>
       <c r="F41" s="2" t="n">
         <v>0</v>
@@ -5865,7 +5925,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -5875,7 +5935,7 @@
         <v>0</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0</v>
+        <v>369.48</v>
       </c>
       <c r="F42" s="2" t="n">
         <v>0</v>
@@ -5892,7 +5952,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -5919,7 +5979,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -5946,7 +6006,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -5973,7 +6033,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -6000,7 +6060,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -6027,7 +6087,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -6054,7 +6114,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -6064,7 +6124,7 @@
         <v>0</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>210.03</v>
+        <v>0</v>
       </c>
       <c r="F49" s="2" t="n">
         <v>0</v>
@@ -6081,17 +6141,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>450.22</v>
+        <v>0</v>
       </c>
       <c r="D50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>0</v>
+        <v>210.03</v>
       </c>
       <c r="F50" s="2" t="n">
         <v>0</v>
@@ -6108,17 +6168,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>517.0599999999999</v>
+        <v>450.22</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>408.89</v>
+        <v>0</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>553.5</v>
+        <v>0</v>
       </c>
       <c r="F51" s="2" t="n">
         <v>0</v>
@@ -6135,17 +6195,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PAREDES POVEDA TATIANA VERONICA</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>0</v>
+        <v>517.0599999999999</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>0</v>
+        <v>408.89</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0</v>
+        <v>553.5</v>
       </c>
       <c r="F52" s="2" t="n">
         <v>0</v>
@@ -6162,14 +6222,14 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PAREDES POVEDA TATIANA VERONICA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>137.52</v>
+        <v>0</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>0</v>
@@ -6189,14 +6249,14 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>503.15</v>
+        <v>0</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>0</v>
+        <v>137.52</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>0</v>
@@ -6216,11 +6276,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>0</v>
+        <v>503.15</v>
       </c>
       <c r="D55" s="2" t="n">
         <v>0</v>
@@ -6243,7 +6303,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -6270,17 +6330,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>2857.01</v>
+        <v>0</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>679.55</v>
+        <v>0</v>
       </c>
       <c r="F57" s="2" t="n">
         <v>0</v>
@@ -6297,17 +6357,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>0</v>
+        <v>2857.01</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0</v>
+        <v>679.55</v>
       </c>
       <c r="F58" s="2" t="n">
         <v>0</v>
@@ -6324,7 +6384,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -6351,7 +6411,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -6378,7 +6438,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -6405,7 +6465,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -6432,7 +6492,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -6459,14 +6519,14 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>1144.09</v>
+        <v>0</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>0</v>
@@ -6486,14 +6546,14 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>944.42</v>
+        <v>0</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>537.98</v>
+        <v>1144.09</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>0</v>
@@ -6513,14 +6573,14 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>0</v>
+        <v>944.42</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>0</v>
+        <v>537.98</v>
       </c>
       <c r="E66" s="2" t="n">
         <v>0</v>
@@ -6540,7 +6600,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -6567,14 +6627,14 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>281.46</v>
+        <v>0</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>0</v>
@@ -6594,39 +6654,66 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>281.46</v>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G69" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="C70" s="4" t="n">
+      <c r="C70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="C71" s="4" t="n">
         <v>6694.99</v>
       </c>
-      <c r="D70" s="4" t="n">
+      <c r="D71" s="4" t="n">
         <v>8555.65</v>
       </c>
-      <c r="E70" s="4" t="n">
+      <c r="E71" s="4" t="n">
         <v>8147.21</v>
       </c>
-      <c r="F70" s="4" t="n">
+      <c r="F71" s="4" t="n">
         <v>1608.51</v>
       </c>
-      <c r="G70" s="4" t="n">
+      <c r="G71" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-03-09 12:30:23
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R71"/>
+  <dimension ref="A1:R72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>GARCIA BRAVO JOSE LUIS</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GAVILANES VELEZ MARIA VALERIA</t>
+          <t>GARCIA BRAVO JOSE LUIS</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GRANJA VANEGAS MARCELA</t>
+          <t>GAVILANES VELEZ MARIA VALERIA</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GRANJA VANEGAS MARCELA</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>IDEARQ ESTUDIO S.A.S.</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>IDEARQ ESTUDIO S.A.S.</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KITCHENSCO S.A.</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
+          <t>KITCHENSCO S.A.</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PAREDES POVEDA TATIANA VERONICA</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PAREDES POVEDA TATIANA VERONICA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,137 +4643,197 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R70" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R70" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="C71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="E71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="F71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="G71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="H71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="I71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="J71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="K71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="L71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="M71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="N71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="O71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="P71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="Q71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
-        </is>
-      </c>
-      <c r="R71" s="3" t="inlineStr">
-        <is>
-          <t>0 de 69</t>
+      <c r="C71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R71" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="K72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="L72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="M72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="N72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="O72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="P72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="Q72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
+        </is>
+      </c>
+      <c r="R72" s="3" t="inlineStr">
+        <is>
+          <t>0 de 70</t>
         </is>
       </c>
     </row>
@@ -4788,7 +4848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5412,7 +5472,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -5439,17 +5499,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>968.04</v>
+        <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>5185.61</v>
+        <v>0</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>682.11</v>
+        <v>0</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>0</v>
@@ -5466,17 +5526,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0</v>
+        <v>968.04</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0</v>
+        <v>5185.61</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0</v>
+        <v>682.11</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>0</v>
@@ -5493,14 +5553,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>67.03</v>
+        <v>0</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>0</v>
@@ -5520,14 +5580,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>17.26</v>
+        <v>67.03</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>0</v>
@@ -5547,14 +5607,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0</v>
+        <v>17.26</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>0</v>
@@ -5574,7 +5634,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -5601,7 +5661,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>GARCIA BRAVO JOSE LUIS</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -5628,7 +5688,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GAVILANES VELEZ MARIA VALERIA</t>
+          <t>GARCIA BRAVO JOSE LUIS</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -5655,7 +5715,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GRANJA VANEGAS MARCELA</t>
+          <t>GAVILANES VELEZ MARIA VALERIA</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -5682,11 +5742,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GRANJA VANEGAS MARCELA</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>65.66</v>
+        <v>0</v>
       </c>
       <c r="D33" s="2" t="n">
         <v>0</v>
@@ -5709,11 +5769,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>IDEARQ ESTUDIO S.A.S.</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0</v>
+        <v>65.66</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>0</v>
@@ -5736,7 +5796,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>IDEARQ ESTUDIO S.A.S.</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -5763,7 +5823,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -5790,7 +5850,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -5817,7 +5877,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KITCHENSCO S.A.</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -5844,7 +5904,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
+          <t>KITCHENSCO S.A.</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -5871,7 +5931,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -5898,7 +5958,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -5925,14 +5985,14 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>369.48</v>
+        <v>0</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>0</v>
@@ -5952,14 +6012,14 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0</v>
+        <v>369.48</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>0</v>
@@ -5979,7 +6039,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -6006,7 +6066,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -6033,7 +6093,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -6060,7 +6120,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -6087,7 +6147,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -6114,7 +6174,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -6141,14 +6201,14 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>210.03</v>
+        <v>0</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>0</v>
@@ -6168,14 +6228,14 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>0</v>
+        <v>210.03</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>0</v>
@@ -6195,14 +6255,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>408.89</v>
+        <v>0</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>553.5</v>
+        <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>0</v>
@@ -6222,14 +6282,14 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PAREDES POVEDA TATIANA VERONICA</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>0</v>
+        <v>408.89</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>0</v>
+        <v>553.5</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>0</v>
@@ -6249,11 +6309,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PAREDES POVEDA TATIANA VERONICA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>137.52</v>
+        <v>0</v>
       </c>
       <c r="D54" s="2" t="n">
         <v>0</v>
@@ -6276,11 +6336,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>0</v>
+        <v>137.52</v>
       </c>
       <c r="D55" s="2" t="n">
         <v>0</v>
@@ -6303,7 +6363,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -6330,7 +6390,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -6357,14 +6417,14 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>2857.01</v>
+        <v>0</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>679.55</v>
+        <v>0</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>0</v>
@@ -6384,14 +6444,14 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>0</v>
+        <v>2857.01</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>0</v>
+        <v>679.55</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>0</v>
@@ -6411,7 +6471,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -6438,7 +6498,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -6465,7 +6525,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -6475,7 +6535,7 @@
         <v>0</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>719.26</v>
+        <v>0</v>
       </c>
       <c r="F62" s="2" t="n">
         <v>0</v>
@@ -6492,7 +6552,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -6502,7 +6562,7 @@
         <v>0</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>0</v>
+        <v>719.26</v>
       </c>
       <c r="F63" s="2" t="n">
         <v>0</v>
@@ -6519,7 +6579,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -6546,11 +6606,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>1144.09</v>
+        <v>0</v>
       </c>
       <c r="D65" s="2" t="n">
         <v>0</v>
@@ -6573,11 +6633,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>537.98</v>
+        <v>1144.09</v>
       </c>
       <c r="D66" s="2" t="n">
         <v>0</v>
@@ -6600,11 +6660,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
-        <v>0</v>
+        <v>537.98</v>
       </c>
       <c r="D67" s="2" t="n">
         <v>0</v>
@@ -6627,7 +6687,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -6654,11 +6714,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
-        <v>281.46</v>
+        <v>0</v>
       </c>
       <c r="D69" s="2" t="n">
         <v>0</v>
@@ -6681,39 +6741,66 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>281.46</v>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G70" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="C71" s="4" t="n">
+      <c r="C71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="C72" s="4" t="n">
         <v>8555.65</v>
       </c>
-      <c r="D71" s="4" t="n">
+      <c r="D72" s="4" t="n">
         <v>8147.21</v>
       </c>
-      <c r="E71" s="4" t="n">
+      <c r="E72" s="4" t="n">
         <v>2478.5</v>
       </c>
-      <c r="F71" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G71" s="4" t="n">
+      <c r="F72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-03-10 17:30:23
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -6921,10 +6921,10 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1007.84</v>
+        <v>1486.84</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-1007.84</v>
+        <v>-1486.84</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>0</v>
@@ -6964,13 +6964,13 @@
         <v>15412.82</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2317.55</v>
+        <v>2796.55</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>13095.27</v>
+        <v>12616.27</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.1503650856884075</v>
+        <v>0.181443110345803</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-11 11:30:19
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0</v>
+        <v>11.45</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -4808,7 +4808,7 @@
       </c>
       <c r="M72" s="3" t="inlineStr">
         <is>
-          <t>1 de 70</t>
+          <t>2 de 70</t>
         </is>
       </c>
       <c r="N72" s="3" t="inlineStr">
@@ -5485,7 +5485,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>11.45</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -6798,7 +6798,7 @@
         <v>2478.5</v>
       </c>
       <c r="F72" s="4" t="n">
-        <v>200.78</v>
+        <v>212.23</v>
       </c>
       <c r="G72" s="4" t="n">
         <v>0</v>
@@ -6823,7 +6823,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6945,13 +6945,13 @@
         <v>15000</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1309.71</v>
+        <v>1321.16</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>13690.29</v>
+        <v>13678.84</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.087314</v>
+        <v>0.08807733333333334</v>
       </c>
     </row>
     <row r="6">
@@ -6964,13 +6964,13 @@
         <v>15412.82</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2796.55</v>
+        <v>2808</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>12616.27</v>
+        <v>12604.82</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.181443110345803</v>
+        <v>0.1821859984091166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-16 10:30:23
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -1962,10 +1962,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>0</v>
+        <v>289.8</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0</v>
+        <v>175.5</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0</v>
@@ -4843,12 +4843,12 @@
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>0 de 71</t>
+          <t>1 de 71</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>0 de 71</t>
+          <t>1 de 71</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
@@ -5599,7 +5599,7 @@
         <v>682.11</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0</v>
+        <v>465.3</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>0</v>
@@ -6885,7 +6885,7 @@
         <v>2478.5</v>
       </c>
       <c r="F73" s="4" t="n">
-        <v>1323.22</v>
+        <v>1788.52</v>
       </c>
       <c r="G73" s="4" t="n">
         <v>0</v>
@@ -6909,7 +6909,7 @@
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -6984,13 +6984,13 @@
         <v>240</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>289.8</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>240</v>
+        <v>-49.80000000000001</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0</v>
+        <v>1.2075</v>
       </c>
     </row>
     <row r="4">
@@ -7008,10 +7008,10 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2768.39</v>
+        <v>2943.89</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-2768.39</v>
+        <v>-2943.89</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>0</v>
@@ -7051,13 +7051,13 @@
         <v>15412.82</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>5135.639999999999</v>
+        <v>5600.940000000001</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>10277.18</v>
+        <v>9811.880000000001</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.3332057339279898</v>
+        <v>0.3633948881515518</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-19 15:30:24
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -6997,7 +6997,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7119,13 +7119,13 @@
         <v>15000</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2511.81</v>
+        <v>2523.64</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>12488.19</v>
+        <v>12476.36</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.167454</v>
+        <v>0.1682426666666667</v>
       </c>
     </row>
     <row r="6">
@@ -7138,13 +7138,13 @@
         <v>15412.82</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>6062.3</v>
+        <v>6074.13</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>9350.52</v>
+        <v>9338.690000000001</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.3933284110240696</v>
+        <v>0.3940959538877376</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-23 17:30:24
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -6997,7 +6997,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7095,10 +7095,10 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>3889.95</v>
+        <v>4224.48</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-3889.95</v>
+        <v>-4224.48</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>0</v>
@@ -7119,13 +7119,13 @@
         <v>15000</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2930.7</v>
+        <v>5740.28</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>12069.3</v>
+        <v>9259.720000000001</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.19538</v>
+        <v>0.3826853333333333</v>
       </c>
     </row>
     <row r="6">
@@ -7138,13 +7138,13 @@
         <v>15412.82</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7110.45</v>
+        <v>10254.56</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>8302.369999999999</v>
+        <v>5158.260000000002</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.4613334873177005</v>
+        <v>0.6653266566403812</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-26 11:30:19
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R74"/>
+  <dimension ref="A1:R75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CORONADO MONTERO LIDA VERONICA</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CORREA IGLESIAS RAMIRO MARCELO</t>
+          <t>CORONADO MONTERO LIDA VERONICA</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Carlos Meza Peña</t>
+          <t>CORREA IGLESIAS RAMIRO MARCELO</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>11.45</v>
+        <v>0</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1917,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>11.45</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -1962,10 +1962,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>289.8</v>
+        <v>0</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>175.5</v>
+        <v>0</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0</v>
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>2209.05</v>
+        <v>0</v>
       </c>
       <c r="N25" s="2" t="n">
         <v>0</v>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2022,10 +2022,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>0</v>
+        <v>289.8</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>0</v>
+        <v>175.5</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0</v>
@@ -2034,10 +2034,10 @@
         <v>0</v>
       </c>
       <c r="L26" s="2" t="n">
-        <v>1110.99</v>
+        <v>0</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>0</v>
+        <v>2209.05</v>
       </c>
       <c r="N26" s="2" t="n">
         <v>0</v>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2094,7 +2094,7 @@
         <v>0</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0</v>
+        <v>1110.99</v>
       </c>
       <c r="M27" s="2" t="n">
         <v>0</v>
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GARCIA BRAVO JOSE LUIS</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GAVILANES VELEZ MARIA VALERIA</t>
+          <t>GARCIA BRAVO JOSE LUIS</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>GRANJA VANEGAS MARCELA</t>
+          <t>GAVILANES VELEZ MARIA VALERIA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GRANJA VANEGAS MARCELA</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>IDEARQ ESTUDIO S.A.S.</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>IDEARQ ESTUDIO S.A.S.</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>KITCHENSCO S.A.</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
+          <t>KITCHENSCO S.A.</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PAREDES POVEDA TATIANA VERONICA</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PAREDES POVEDA TATIANA VERONICA</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4191,7 +4191,7 @@
         <v>0</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>0</v>
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4251,7 +4251,7 @@
         <v>0</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,137 +4823,197 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R73" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R73" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="C74" s="3" t="inlineStr">
-        <is>
-          <t>0 de 72</t>
-        </is>
-      </c>
-      <c r="D74" s="3" t="inlineStr">
-        <is>
-          <t>1 de 72</t>
-        </is>
-      </c>
-      <c r="E74" s="3" t="inlineStr">
-        <is>
-          <t>0 de 72</t>
-        </is>
-      </c>
-      <c r="F74" s="3" t="inlineStr">
-        <is>
-          <t>0 de 72</t>
-        </is>
-      </c>
-      <c r="G74" s="3" t="inlineStr">
-        <is>
-          <t>0 de 72</t>
-        </is>
-      </c>
-      <c r="H74" s="3" t="inlineStr">
-        <is>
-          <t>1 de 72</t>
-        </is>
-      </c>
-      <c r="I74" s="3" t="inlineStr">
-        <is>
-          <t>1 de 72</t>
-        </is>
-      </c>
-      <c r="J74" s="3" t="inlineStr">
-        <is>
-          <t>0 de 72</t>
-        </is>
-      </c>
-      <c r="K74" s="3" t="inlineStr">
-        <is>
-          <t>1 de 72</t>
-        </is>
-      </c>
-      <c r="L74" s="3" t="inlineStr">
-        <is>
-          <t>1 de 72</t>
-        </is>
-      </c>
-      <c r="M74" s="3" t="inlineStr">
-        <is>
-          <t>3 de 72</t>
-        </is>
-      </c>
-      <c r="N74" s="3" t="inlineStr">
-        <is>
-          <t>0 de 72</t>
-        </is>
-      </c>
-      <c r="O74" s="3" t="inlineStr">
-        <is>
-          <t>0 de 72</t>
-        </is>
-      </c>
-      <c r="P74" s="3" t="inlineStr">
-        <is>
-          <t>0 de 72</t>
-        </is>
-      </c>
-      <c r="Q74" s="3" t="inlineStr">
-        <is>
-          <t>0 de 72</t>
-        </is>
-      </c>
-      <c r="R74" s="3" t="inlineStr">
-        <is>
-          <t>0 de 72</t>
+      <c r="C74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R74" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>0 de 73</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>1 de 73</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>0 de 73</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>0 de 73</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>0 de 73</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>1 de 73</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>1 de 73</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>0 de 73</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t>1 de 73</t>
+        </is>
+      </c>
+      <c r="L75" s="3" t="inlineStr">
+        <is>
+          <t>1 de 73</t>
+        </is>
+      </c>
+      <c r="M75" s="3" t="inlineStr">
+        <is>
+          <t>3 de 73</t>
+        </is>
+      </c>
+      <c r="N75" s="3" t="inlineStr">
+        <is>
+          <t>0 de 73</t>
+        </is>
+      </c>
+      <c r="O75" s="3" t="inlineStr">
+        <is>
+          <t>0 de 73</t>
+        </is>
+      </c>
+      <c r="P75" s="3" t="inlineStr">
+        <is>
+          <t>0 de 73</t>
+        </is>
+      </c>
+      <c r="Q75" s="3" t="inlineStr">
+        <is>
+          <t>0 de 73</t>
+        </is>
+      </c>
+      <c r="R75" s="3" t="inlineStr">
+        <is>
+          <t>0 de 73</t>
         </is>
       </c>
     </row>
@@ -4968,7 +5028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5511,7 +5571,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -5538,7 +5598,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CORONADO MONTERO LIDA VERONICA</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -5565,7 +5625,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CORREA IGLESIAS RAMIRO MARCELO</t>
+          <t>CORONADO MONTERO LIDA VERONICA</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -5592,7 +5652,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Carlos Meza Peña</t>
+          <t>CORREA IGLESIAS RAMIRO MARCELO</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -5605,7 +5665,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>11.45</v>
+        <v>0</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -5619,7 +5679,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -5632,7 +5692,7 @@
         <v>0</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0</v>
+        <v>11.45</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>0</v>
@@ -5646,20 +5706,20 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>968.04</v>
+        <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>5185.61</v>
+        <v>0</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>682.11</v>
+        <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>2674.35</v>
+        <v>0</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>0</v>
@@ -5673,20 +5733,20 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0</v>
+        <v>968.04</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0</v>
+        <v>5185.61</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0</v>
+        <v>682.11</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>1110.99</v>
+        <v>2674.35</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>0</v>
@@ -5700,7 +5760,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -5713,7 +5773,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>1110.99</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -5727,14 +5787,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>67.03</v>
+        <v>0</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>0</v>
@@ -5754,14 +5814,14 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>17.26</v>
+        <v>67.03</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>0</v>
@@ -5781,14 +5841,14 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0</v>
+        <v>17.26</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>0</v>
@@ -5808,7 +5868,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -5835,7 +5895,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GARCIA BRAVO JOSE LUIS</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -5862,7 +5922,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GAVILANES VELEZ MARIA VALERIA</t>
+          <t>GARCIA BRAVO JOSE LUIS</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -5889,7 +5949,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>GRANJA VANEGAS MARCELA</t>
+          <t>GAVILANES VELEZ MARIA VALERIA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -5916,11 +5976,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GRANJA VANEGAS MARCELA</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>65.66</v>
+        <v>0</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>0</v>
@@ -5943,11 +6003,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>IDEARQ ESTUDIO S.A.S.</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0</v>
+        <v>65.66</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>0</v>
@@ -5970,7 +6030,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>IDEARQ ESTUDIO S.A.S.</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -5997,7 +6057,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -6024,7 +6084,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -6051,7 +6111,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>KITCHENSCO S.A.</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -6078,7 +6138,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
+          <t>KITCHENSCO S.A.</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -6105,7 +6165,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -6132,7 +6192,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -6159,14 +6219,14 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>369.48</v>
+        <v>0</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>0</v>
@@ -6186,14 +6246,14 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0</v>
+        <v>369.48</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>0</v>
@@ -6213,7 +6273,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -6240,7 +6300,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -6267,7 +6327,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -6294,7 +6354,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -6321,7 +6381,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -6348,7 +6408,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -6375,14 +6435,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>210.03</v>
+        <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>0</v>
@@ -6402,14 +6462,14 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>0</v>
+        <v>210.03</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>0</v>
@@ -6429,14 +6489,14 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>408.89</v>
+        <v>0</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>553.5</v>
+        <v>0</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>0</v>
@@ -6456,14 +6516,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PAREDES POVEDA TATIANA VERONICA</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>0</v>
+        <v>408.89</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>0</v>
+        <v>553.5</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>0</v>
@@ -6483,11 +6543,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PAREDES POVEDA TATIANA VERONICA</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>137.52</v>
+        <v>0</v>
       </c>
       <c r="D56" s="2" t="n">
         <v>0</v>
@@ -6510,11 +6570,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>0</v>
+        <v>137.52</v>
       </c>
       <c r="D57" s="2" t="n">
         <v>0</v>
@@ -6537,7 +6597,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -6564,7 +6624,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -6591,14 +6651,14 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>2857.01</v>
+        <v>0</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>679.55</v>
+        <v>0</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>0</v>
@@ -6618,14 +6678,14 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
-        <v>0</v>
+        <v>2857.01</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>0</v>
+        <v>679.55</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>0</v>
@@ -6645,7 +6705,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -6658,7 +6718,7 @@
         <v>0</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="G62" s="2" t="n">
         <v>0</v>
@@ -6672,7 +6732,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -6685,7 +6745,7 @@
         <v>0</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>0</v>
@@ -6699,7 +6759,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -6726,7 +6786,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -6736,7 +6796,7 @@
         <v>0</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>719.26</v>
+        <v>0</v>
       </c>
       <c r="F65" s="2" t="n">
         <v>0</v>
@@ -6753,7 +6813,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -6763,7 +6823,7 @@
         <v>0</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>0</v>
+        <v>719.26</v>
       </c>
       <c r="F66" s="2" t="n">
         <v>0</v>
@@ -6780,7 +6840,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -6807,11 +6867,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
-        <v>1144.09</v>
+        <v>0</v>
       </c>
       <c r="D68" s="2" t="n">
         <v>0</v>
@@ -6834,11 +6894,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
-        <v>537.98</v>
+        <v>1144.09</v>
       </c>
       <c r="D69" s="2" t="n">
         <v>0</v>
@@ -6861,11 +6921,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
-        <v>0</v>
+        <v>537.98</v>
       </c>
       <c r="D70" s="2" t="n">
         <v>0</v>
@@ -6888,7 +6948,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -6915,11 +6975,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
-        <v>281.46</v>
+        <v>0</v>
       </c>
       <c r="D72" s="2" t="n">
         <v>0</v>
@@ -6942,39 +7002,66 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>281.46</v>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G73" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="C74" s="4" t="n">
+      <c r="C74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="C75" s="4" t="n">
         <v>8555.65</v>
       </c>
-      <c r="D74" s="4" t="n">
+      <c r="D75" s="4" t="n">
         <v>8147.21</v>
       </c>
-      <c r="E74" s="4" t="n">
+      <c r="E75" s="4" t="n">
         <v>2478.5</v>
       </c>
-      <c r="F74" s="4" t="n">
+      <c r="F75" s="4" t="n">
         <v>4128.49</v>
       </c>
-      <c r="G74" s="4" t="n">
+      <c r="G75" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-03-27 14:30:24
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -7269,10 +7269,10 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>6025.86</v>
+        <v>6342.66</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-6025.86</v>
+        <v>-6342.66</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>0</v>
@@ -7312,13 +7312,13 @@
         <v>15412.82</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>14408.07</v>
+        <v>14724.87</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1004.750000000001</v>
+        <v>687.9500000000007</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.9348107614310684</v>
+        <v>0.955365079200302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-08 17:30:21
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R76"/>
+  <dimension ref="A1:R77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PAREDES POVEDA TATIANA VERONICA</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PAREDES POVEDA TATIANA VERONICA</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4311,7 +4311,7 @@
         <v>0</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="L64" s="2" t="n">
         <v>0</v>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4371,7 +4371,7 @@
         <v>0</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="L65" s="2" t="n">
         <v>0</v>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,137 +4943,197 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R75" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R75" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="C76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="D76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="E76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="F76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="G76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="H76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="I76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="J76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="K76" s="3" t="inlineStr">
-        <is>
-          <t>1 de 74</t>
-        </is>
-      </c>
-      <c r="L76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="M76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="N76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="O76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="P76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="Q76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
-        </is>
-      </c>
-      <c r="R76" s="3" t="inlineStr">
-        <is>
-          <t>0 de 74</t>
+      <c r="C76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R76" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>1 de 75</t>
+        </is>
+      </c>
+      <c r="L77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="M77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="N77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="O77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="P77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="Q77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
+        </is>
+      </c>
+      <c r="R77" s="3" t="inlineStr">
+        <is>
+          <t>0 de 75</t>
         </is>
       </c>
     </row>
@@ -5088,7 +5148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6603,17 +6663,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>553.5</v>
+        <v>0</v>
       </c>
       <c r="D56" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>198.03</v>
+        <v>0</v>
       </c>
       <c r="F56" s="2" t="n">
         <v>0</v>
@@ -6630,17 +6690,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PAREDES POVEDA TATIANA VERONICA</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>0</v>
+        <v>553.5</v>
       </c>
       <c r="D57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0</v>
+        <v>198.03</v>
       </c>
       <c r="F57" s="2" t="n">
         <v>0</v>
@@ -6657,7 +6717,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PAREDES POVEDA TATIANA VERONICA</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -6684,7 +6744,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -6711,7 +6771,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -6738,7 +6798,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -6765,11 +6825,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
-        <v>679.55</v>
+        <v>0</v>
       </c>
       <c r="D62" s="2" t="n">
         <v>0</v>
@@ -6792,11 +6852,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>0</v>
+        <v>679.55</v>
       </c>
       <c r="D63" s="2" t="n">
         <v>0</v>
@@ -6819,7 +6879,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -6829,10 +6889,10 @@
         <v>0</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="G64" s="2" t="n">
         <v>0</v>
@@ -6846,7 +6906,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -6856,10 +6916,10 @@
         <v>0</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="G65" s="2" t="n">
         <v>0</v>
@@ -6873,7 +6933,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -6900,14 +6960,14 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>719.26</v>
+        <v>0</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>0</v>
@@ -6927,14 +6987,14 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>0</v>
+        <v>719.26</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>0</v>
@@ -6954,7 +7014,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -6981,7 +7041,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -7008,7 +7068,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -7035,7 +7095,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -7062,7 +7122,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -7089,7 +7149,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -7116,39 +7176,66 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F75" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G75" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="C76" s="4" t="n">
+      <c r="C76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="C77" s="4" t="n">
         <v>8147.21</v>
       </c>
-      <c r="D76" s="4" t="n">
+      <c r="D77" s="4" t="n">
         <v>2478.5</v>
       </c>
-      <c r="E76" s="4" t="n">
+      <c r="E77" s="4" t="n">
         <v>4437.4</v>
       </c>
-      <c r="F76" s="4" t="n">
+      <c r="F77" s="4" t="n">
         <v>130.92</v>
       </c>
-      <c r="G76" s="4" t="n">
+      <c r="G77" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-04-15 11:30:21
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R77"/>
+  <dimension ref="A1:R78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,137 +5003,197 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R76" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R76" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="C77" s="3" t="inlineStr">
-        <is>
-          <t>0 de 75</t>
-        </is>
-      </c>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>0 de 75</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="inlineStr">
-        <is>
-          <t>0 de 75</t>
-        </is>
-      </c>
-      <c r="F77" s="3" t="inlineStr">
-        <is>
-          <t>0 de 75</t>
-        </is>
-      </c>
-      <c r="G77" s="3" t="inlineStr">
-        <is>
-          <t>0 de 75</t>
-        </is>
-      </c>
-      <c r="H77" s="3" t="inlineStr">
-        <is>
-          <t>1 de 75</t>
-        </is>
-      </c>
-      <c r="I77" s="3" t="inlineStr">
-        <is>
-          <t>1 de 75</t>
-        </is>
-      </c>
-      <c r="J77" s="3" t="inlineStr">
-        <is>
-          <t>0 de 75</t>
-        </is>
-      </c>
-      <c r="K77" s="3" t="inlineStr">
-        <is>
-          <t>1 de 75</t>
-        </is>
-      </c>
-      <c r="L77" s="3" t="inlineStr">
-        <is>
-          <t>1 de 75</t>
-        </is>
-      </c>
-      <c r="M77" s="3" t="inlineStr">
-        <is>
-          <t>0 de 75</t>
-        </is>
-      </c>
-      <c r="N77" s="3" t="inlineStr">
-        <is>
-          <t>0 de 75</t>
-        </is>
-      </c>
-      <c r="O77" s="3" t="inlineStr">
-        <is>
-          <t>0 de 75</t>
-        </is>
-      </c>
-      <c r="P77" s="3" t="inlineStr">
-        <is>
-          <t>0 de 75</t>
-        </is>
-      </c>
-      <c r="Q77" s="3" t="inlineStr">
-        <is>
-          <t>0 de 75</t>
-        </is>
-      </c>
-      <c r="R77" s="3" t="inlineStr">
-        <is>
-          <t>0 de 75</t>
+      <c r="C77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R77" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>0 de 76</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>0 de 76</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>0 de 76</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>0 de 76</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>0 de 76</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>1 de 76</t>
+        </is>
+      </c>
+      <c r="I78" s="3" t="inlineStr">
+        <is>
+          <t>1 de 76</t>
+        </is>
+      </c>
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t>0 de 76</t>
+        </is>
+      </c>
+      <c r="K78" s="3" t="inlineStr">
+        <is>
+          <t>1 de 76</t>
+        </is>
+      </c>
+      <c r="L78" s="3" t="inlineStr">
+        <is>
+          <t>1 de 76</t>
+        </is>
+      </c>
+      <c r="M78" s="3" t="inlineStr">
+        <is>
+          <t>0 de 76</t>
+        </is>
+      </c>
+      <c r="N78" s="3" t="inlineStr">
+        <is>
+          <t>0 de 76</t>
+        </is>
+      </c>
+      <c r="O78" s="3" t="inlineStr">
+        <is>
+          <t>0 de 76</t>
+        </is>
+      </c>
+      <c r="P78" s="3" t="inlineStr">
+        <is>
+          <t>0 de 76</t>
+        </is>
+      </c>
+      <c r="Q78" s="3" t="inlineStr">
+        <is>
+          <t>0 de 76</t>
+        </is>
+      </c>
+      <c r="R78" s="3" t="inlineStr">
+        <is>
+          <t>0 de 76</t>
         </is>
       </c>
     </row>
@@ -5148,7 +5208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7068,7 +7128,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -7095,7 +7155,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -7122,7 +7182,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -7149,7 +7209,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -7176,7 +7236,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -7203,39 +7263,66 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F76" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G76" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="C77" s="4" t="n">
+      <c r="C77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="C78" s="4" t="n">
         <v>8147.21</v>
       </c>
-      <c r="D77" s="4" t="n">
+      <c r="D78" s="4" t="n">
         <v>2478.5</v>
       </c>
-      <c r="E77" s="4" t="n">
+      <c r="E78" s="4" t="n">
         <v>4437.4</v>
       </c>
-      <c r="F77" s="4" t="n">
+      <c r="F78" s="4" t="n">
         <v>566.61</v>
       </c>
-      <c r="G77" s="4" t="n">
+      <c r="G78" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-04-16 11:30:17
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R78"/>
+  <dimension ref="A1:R79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4533,7 +4533,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="F68" s="2" t="n">
         <v>0</v>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,137 +5063,197 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R77" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R77" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="C78" s="3" t="inlineStr">
-        <is>
-          <t>0 de 76</t>
-        </is>
-      </c>
-      <c r="D78" s="3" t="inlineStr">
-        <is>
-          <t>0 de 76</t>
-        </is>
-      </c>
-      <c r="E78" s="3" t="inlineStr">
-        <is>
-          <t>0 de 76</t>
-        </is>
-      </c>
-      <c r="F78" s="3" t="inlineStr">
-        <is>
-          <t>0 de 76</t>
-        </is>
-      </c>
-      <c r="G78" s="3" t="inlineStr">
-        <is>
-          <t>0 de 76</t>
-        </is>
-      </c>
-      <c r="H78" s="3" t="inlineStr">
-        <is>
-          <t>1 de 76</t>
-        </is>
-      </c>
-      <c r="I78" s="3" t="inlineStr">
-        <is>
-          <t>1 de 76</t>
-        </is>
-      </c>
-      <c r="J78" s="3" t="inlineStr">
-        <is>
-          <t>0 de 76</t>
-        </is>
-      </c>
-      <c r="K78" s="3" t="inlineStr">
-        <is>
-          <t>1 de 76</t>
-        </is>
-      </c>
-      <c r="L78" s="3" t="inlineStr">
-        <is>
-          <t>1 de 76</t>
-        </is>
-      </c>
-      <c r="M78" s="3" t="inlineStr">
-        <is>
-          <t>0 de 76</t>
-        </is>
-      </c>
-      <c r="N78" s="3" t="inlineStr">
-        <is>
-          <t>0 de 76</t>
-        </is>
-      </c>
-      <c r="O78" s="3" t="inlineStr">
-        <is>
-          <t>0 de 76</t>
-        </is>
-      </c>
-      <c r="P78" s="3" t="inlineStr">
-        <is>
-          <t>0 de 76</t>
-        </is>
-      </c>
-      <c r="Q78" s="3" t="inlineStr">
-        <is>
-          <t>0 de 76</t>
-        </is>
-      </c>
-      <c r="R78" s="3" t="inlineStr">
-        <is>
-          <t>0 de 76</t>
+      <c r="C78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R78" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>0 de 77</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>0 de 77</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>1 de 77</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>0 de 77</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>0 de 77</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>1 de 77</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>1 de 77</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>0 de 77</t>
+        </is>
+      </c>
+      <c r="K79" s="3" t="inlineStr">
+        <is>
+          <t>1 de 77</t>
+        </is>
+      </c>
+      <c r="L79" s="3" t="inlineStr">
+        <is>
+          <t>1 de 77</t>
+        </is>
+      </c>
+      <c r="M79" s="3" t="inlineStr">
+        <is>
+          <t>0 de 77</t>
+        </is>
+      </c>
+      <c r="N79" s="3" t="inlineStr">
+        <is>
+          <t>0 de 77</t>
+        </is>
+      </c>
+      <c r="O79" s="3" t="inlineStr">
+        <is>
+          <t>0 de 77</t>
+        </is>
+      </c>
+      <c r="P79" s="3" t="inlineStr">
+        <is>
+          <t>0 de 77</t>
+        </is>
+      </c>
+      <c r="Q79" s="3" t="inlineStr">
+        <is>
+          <t>0 de 77</t>
+        </is>
+      </c>
+      <c r="R79" s="3" t="inlineStr">
+        <is>
+          <t>0 de 77</t>
         </is>
       </c>
     </row>
@@ -5208,7 +5268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7047,20 +7107,20 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>719.26</v>
+        <v>0</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="G68" s="2" t="n">
         <v>0</v>
@@ -7074,14 +7134,14 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>0</v>
+        <v>719.26</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>0</v>
@@ -7101,7 +7161,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -7128,7 +7188,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -7155,7 +7215,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -7182,7 +7242,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -7209,7 +7269,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -7236,7 +7296,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -7263,7 +7323,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -7290,39 +7350,66 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G77" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="C78" s="4" t="n">
+      <c r="C78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="C79" s="4" t="n">
         <v>8147.21</v>
       </c>
-      <c r="D78" s="4" t="n">
+      <c r="D79" s="4" t="n">
         <v>2478.5</v>
       </c>
-      <c r="E78" s="4" t="n">
+      <c r="E79" s="4" t="n">
         <v>4437.4</v>
       </c>
-      <c r="F78" s="4" t="n">
-        <v>566.61</v>
-      </c>
-      <c r="G78" s="4" t="n">
+      <c r="F79" s="4" t="n">
+        <v>674.0699999999999</v>
+      </c>
+      <c r="G79" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7419,13 +7506,13 @@
         <v>199.5</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>199.5</v>
+        <v>92.04000000000001</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0</v>
+        <v>0.5386466165413534</v>
       </c>
     </row>
     <row r="4">
@@ -7534,13 +7621,13 @@
         <v>15372.32</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>3875.19</v>
+        <v>3982.65</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>11497.13</v>
+        <v>11389.67</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.252088819384452</v>
+        <v>0.2590793061815003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-16 17:30:22
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -7554,10 +7554,10 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1944.5</v>
+        <v>2788.1</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-1944.5</v>
+        <v>-2788.1</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0</v>
@@ -7621,13 +7621,13 @@
         <v>15372.32</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>3986.7</v>
+        <v>4830.3</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>11385.62</v>
+        <v>10542.02</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.259342766739178</v>
+        <v>0.3142206251235988</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-20 17:30:20
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -1707,7 +1707,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0</v>
+        <v>110.59</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>0</v>
@@ -5178,7 +5178,7 @@
     <row r="79">
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>0 de 77</t>
+          <t>1 de 77</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -5276,7 +5276,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -5851,7 +5851,7 @@
         <v>110.88</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>-110.88</v>
+        <v>-0.29</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>0</v>
@@ -7407,7 +7407,7 @@
         <v>4437.4</v>
       </c>
       <c r="F79" s="4" t="n">
-        <v>789.9499999999999</v>
+        <v>900.54</v>
       </c>
       <c r="G79" s="4" t="n">
         <v>0</v>
@@ -7482,10 +7482,10 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>110.59</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0</v>
+        <v>-110.59</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>0</v>
@@ -7621,13 +7621,13 @@
         <v>15372.32</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>5184.370000000001</v>
+        <v>5294.96</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>10187.95</v>
+        <v>10077.36</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.3372535830635845</v>
+        <v>0.3444476825879243</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-24 16:30:23
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -7517,7 +7517,7 @@
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -7641,10 +7641,10 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>4415.7</v>
+        <v>4621.45</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-4415.7</v>
+        <v>-4621.45</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0</v>
@@ -7708,13 +7708,13 @@
         <v>15372.32</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>8215.790000000001</v>
+        <v>8421.540000000001</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>7156.530000000001</v>
+        <v>6950.780000000001</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.5344534852253922</v>
+        <v>0.5478379320753146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-27 11:30:22
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -7641,10 +7641,10 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>4621.45</v>
+        <v>4728.45</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-4621.45</v>
+        <v>-4728.45</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0</v>
@@ -7708,13 +7708,13 @@
         <v>15372.32</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>8421.540000000001</v>
+        <v>8528.540000000001</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>6950.780000000001</v>
+        <v>6843.780000000001</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.5478379320753146</v>
+        <v>0.5547984949571698</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-27 12:30:25
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R80"/>
+  <dimension ref="A1:R81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>GRANJA VANEGAS MARCELA</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GRANJA VANEGAS MARCELA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>IDEARQ ESTUDIO S.A.S.</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>IDEARQ ESTUDIO S.A.S.</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>KITCHENSCO S.A.</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
+          <t>KITCHENSCO S.A.</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3834,7 +3834,7 @@
         <v>0</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>167.75</v>
+        <v>0</v>
       </c>
       <c r="M56" s="2" t="n">
         <v>0</v>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3894,7 +3894,7 @@
         <v>0</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>102.69</v>
+        <v>167.75</v>
       </c>
       <c r="M57" s="2" t="n">
         <v>0</v>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PAREDES POVEDA TATIANA VERONICA</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3954,7 +3954,7 @@
         <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>0</v>
+        <v>102.69</v>
       </c>
       <c r="M58" s="2" t="n">
         <v>0</v>
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PAREDES POVEDA TATIANA VERONICA</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4371,7 +4371,7 @@
         <v>0</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="L65" s="2" t="n">
         <v>0</v>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4431,7 +4431,7 @@
         <v>0</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="L66" s="2" t="n">
         <v>0</v>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4533,7 +4533,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>107.46</v>
+        <v>0</v>
       </c>
       <c r="F68" s="2" t="n">
         <v>0</v>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4593,7 +4593,7 @@
         <v>0</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="F69" s="2" t="n">
         <v>0</v>
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4797,7 +4797,7 @@
         <v>0</v>
       </c>
       <c r="M72" s="2" t="n">
-        <v>50.16</v>
+        <v>0</v>
       </c>
       <c r="N72" s="2" t="n">
         <v>0</v>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4857,7 +4857,7 @@
         <v>0</v>
       </c>
       <c r="M73" s="2" t="n">
-        <v>0</v>
+        <v>50.16</v>
       </c>
       <c r="N73" s="2" t="n">
         <v>0</v>
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4893,7 +4893,7 @@
         <v>0</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>176.6</v>
+        <v>0</v>
       </c>
       <c r="F74" s="2" t="n">
         <v>0</v>
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -4953,7 +4953,7 @@
         <v>0</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>0</v>
+        <v>176.6</v>
       </c>
       <c r="F75" s="2" t="n">
         <v>0</v>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5157,7 +5157,7 @@
         <v>0</v>
       </c>
       <c r="M78" s="2" t="n">
-        <v>3.94</v>
+        <v>0</v>
       </c>
       <c r="N78" s="2" t="n">
         <v>0</v>
@@ -5183,137 +5183,197 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" s="2" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="N79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R79" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R79" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="C80" s="3" t="inlineStr">
-        <is>
-          <t>1 de 78</t>
-        </is>
-      </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>0 de 78</t>
-        </is>
-      </c>
-      <c r="E80" s="3" t="inlineStr">
-        <is>
-          <t>2 de 78</t>
-        </is>
-      </c>
-      <c r="F80" s="3" t="inlineStr">
-        <is>
-          <t>0 de 78</t>
-        </is>
-      </c>
-      <c r="G80" s="3" t="inlineStr">
-        <is>
-          <t>0 de 78</t>
-        </is>
-      </c>
-      <c r="H80" s="3" t="inlineStr">
-        <is>
-          <t>1 de 78</t>
-        </is>
-      </c>
-      <c r="I80" s="3" t="inlineStr">
-        <is>
-          <t>1 de 78</t>
-        </is>
-      </c>
-      <c r="J80" s="3" t="inlineStr">
-        <is>
-          <t>0 de 78</t>
-        </is>
-      </c>
-      <c r="K80" s="3" t="inlineStr">
-        <is>
-          <t>1 de 78</t>
-        </is>
-      </c>
-      <c r="L80" s="3" t="inlineStr">
-        <is>
-          <t>2 de 78</t>
-        </is>
-      </c>
-      <c r="M80" s="3" t="inlineStr">
-        <is>
-          <t>2 de 78</t>
-        </is>
-      </c>
-      <c r="N80" s="3" t="inlineStr">
-        <is>
-          <t>0 de 78</t>
-        </is>
-      </c>
-      <c r="O80" s="3" t="inlineStr">
-        <is>
-          <t>0 de 78</t>
-        </is>
-      </c>
-      <c r="P80" s="3" t="inlineStr">
-        <is>
-          <t>0 de 78</t>
-        </is>
-      </c>
-      <c r="Q80" s="3" t="inlineStr">
-        <is>
-          <t>0 de 78</t>
-        </is>
-      </c>
-      <c r="R80" s="3" t="inlineStr">
-        <is>
-          <t>0 de 78</t>
+      <c r="C80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R80" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>1 de 79</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>0 de 79</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>2 de 79</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>0 de 79</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>0 de 79</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>1 de 79</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>1 de 79</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>0 de 79</t>
+        </is>
+      </c>
+      <c r="K81" s="3" t="inlineStr">
+        <is>
+          <t>1 de 79</t>
+        </is>
+      </c>
+      <c r="L81" s="3" t="inlineStr">
+        <is>
+          <t>2 de 79</t>
+        </is>
+      </c>
+      <c r="M81" s="3" t="inlineStr">
+        <is>
+          <t>2 de 79</t>
+        </is>
+      </c>
+      <c r="N81" s="3" t="inlineStr">
+        <is>
+          <t>0 de 79</t>
+        </is>
+      </c>
+      <c r="O81" s="3" t="inlineStr">
+        <is>
+          <t>0 de 79</t>
+        </is>
+      </c>
+      <c r="P81" s="3" t="inlineStr">
+        <is>
+          <t>0 de 79</t>
+        </is>
+      </c>
+      <c r="Q81" s="3" t="inlineStr">
+        <is>
+          <t>0 de 79</t>
+        </is>
+      </c>
+      <c r="R81" s="3" t="inlineStr">
+        <is>
+          <t>0 de 79</t>
         </is>
       </c>
     </row>
@@ -5328,7 +5388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6303,7 +6363,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>GRANJA VANEGAS MARCELA</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -6330,7 +6390,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GRANJA VANEGAS MARCELA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -6357,7 +6417,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>IDEARQ ESTUDIO S.A.S.</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -6384,7 +6444,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>IDEARQ ESTUDIO S.A.S.</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -6411,7 +6471,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -6438,7 +6498,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -6465,7 +6525,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>KITCHENSCO S.A.</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -6492,7 +6552,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
+          <t>KITCHENSCO S.A.</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -6519,7 +6579,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LINCANGO LUGMANIA SANDY LIZETH</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -6546,7 +6606,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -6573,11 +6633,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>369.48</v>
+        <v>0</v>
       </c>
       <c r="D46" s="2" t="n">
         <v>0</v>
@@ -6600,11 +6660,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>0</v>
+        <v>369.48</v>
       </c>
       <c r="D47" s="2" t="n">
         <v>0</v>
@@ -6627,7 +6687,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -6654,7 +6714,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -6681,7 +6741,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -6708,7 +6768,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -6735,7 +6795,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -6762,7 +6822,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -6789,11 +6849,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>210.03</v>
+        <v>0</v>
       </c>
       <c r="D54" s="2" t="n">
         <v>0</v>
@@ -6816,11 +6876,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>0</v>
+        <v>210.03</v>
       </c>
       <c r="D55" s="2" t="n">
         <v>0</v>
@@ -6843,7 +6903,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -6856,7 +6916,7 @@
         <v>0</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>167.75</v>
+        <v>0</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>0</v>
@@ -6870,20 +6930,20 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>553.5</v>
+        <v>0</v>
       </c>
       <c r="D57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>198.03</v>
+        <v>0</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>102.69</v>
+        <v>167.75</v>
       </c>
       <c r="G57" s="2" t="n">
         <v>0</v>
@@ -6897,20 +6957,20 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PAREDES POVEDA TATIANA VERONICA</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>0</v>
+        <v>553.5</v>
       </c>
       <c r="D58" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0</v>
+        <v>198.03</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>0</v>
+        <v>102.69</v>
       </c>
       <c r="G58" s="2" t="n">
         <v>0</v>
@@ -6924,7 +6984,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PAREDES POVEDA TATIANA VERONICA</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -6951,7 +7011,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -6978,7 +7038,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -7005,7 +7065,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -7032,11 +7092,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>679.55</v>
+        <v>0</v>
       </c>
       <c r="D63" s="2" t="n">
         <v>0</v>
@@ -7059,11 +7119,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>0</v>
+        <v>679.55</v>
       </c>
       <c r="D64" s="2" t="n">
         <v>0</v>
@@ -7086,7 +7146,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SALAZAR VERA ENRIQUE WILLIAM</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -7096,10 +7156,10 @@
         <v>0</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="G65" s="2" t="n">
         <v>0</v>
@@ -7113,7 +7173,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -7123,10 +7183,10 @@
         <v>0</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>0</v>
@@ -7140,7 +7200,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -7167,7 +7227,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -7180,7 +7240,7 @@
         <v>0</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>107.46</v>
+        <v>0</v>
       </c>
       <c r="G68" s="2" t="n">
         <v>0</v>
@@ -7194,20 +7254,20 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>719.26</v>
+        <v>0</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="G69" s="2" t="n">
         <v>0</v>
@@ -7221,14 +7281,14 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D70" s="2" t="n">
-        <v>0</v>
+        <v>719.26</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>0</v>
@@ -7248,7 +7308,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -7275,7 +7335,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -7288,7 +7348,7 @@
         <v>0</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>50.16</v>
+        <v>0</v>
       </c>
       <c r="G72" s="2" t="n">
         <v>0</v>
@@ -7302,7 +7362,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -7315,7 +7375,7 @@
         <v>0</v>
       </c>
       <c r="F73" s="2" t="n">
-        <v>0</v>
+        <v>50.16</v>
       </c>
       <c r="G73" s="2" t="n">
         <v>0</v>
@@ -7329,7 +7389,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -7342,7 +7402,7 @@
         <v>0</v>
       </c>
       <c r="F74" s="2" t="n">
-        <v>176.6</v>
+        <v>0</v>
       </c>
       <c r="G74" s="2" t="n">
         <v>0</v>
@@ -7356,7 +7416,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -7369,7 +7429,7 @@
         <v>0</v>
       </c>
       <c r="F75" s="2" t="n">
-        <v>0</v>
+        <v>176.6</v>
       </c>
       <c r="G75" s="2" t="n">
         <v>0</v>
@@ -7383,7 +7443,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -7410,7 +7470,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>VIZUETE GALARZA EDWIN RODRIGO</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -7437,7 +7497,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -7450,7 +7510,7 @@
         <v>0</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>3.94</v>
+        <v>0</v>
       </c>
       <c r="G78" s="2" t="n">
         <v>0</v>
@@ -7464,39 +7524,66 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
           <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
-      <c r="C79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G79" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="C80" s="4" t="n">
+      <c r="C80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="C81" s="4" t="n">
         <v>8147.21</v>
       </c>
-      <c r="D80" s="4" t="n">
+      <c r="D81" s="4" t="n">
         <v>2478.5</v>
       </c>
-      <c r="E80" s="4" t="n">
+      <c r="E81" s="4" t="n">
         <v>4437.4</v>
       </c>
-      <c r="F80" s="4" t="n">
+      <c r="F81" s="4" t="n">
         <v>1072.23</v>
       </c>
-      <c r="G80" s="4" t="n">
+      <c r="G81" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-04-28 17:30:21
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -3894,7 +3894,7 @@
         <v>0</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>167.75</v>
+        <v>346.79</v>
       </c>
       <c r="M57" s="2" t="n">
         <v>0</v>
@@ -6943,7 +6943,7 @@
         <v>0</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>167.75</v>
+        <v>346.79</v>
       </c>
       <c r="G57" s="2" t="n">
         <v>0</v>
@@ -7581,7 +7581,7 @@
         <v>4437.4</v>
       </c>
       <c r="F81" s="4" t="n">
-        <v>1905.26</v>
+        <v>2084.3</v>
       </c>
       <c r="G81" s="4" t="n">
         <v>0</v>
@@ -7728,10 +7728,10 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>5561.48</v>
+        <v>5740.52</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-5561.48</v>
+        <v>-5740.52</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0</v>
@@ -7795,13 +7795,13 @@
         <v>15372.32</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>9361.57</v>
+        <v>9540.610000000001</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>6010.750000000001</v>
+        <v>5831.71</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.6089887538120465</v>
+        <v>0.6206356620210873</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-05-11 08:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R117"/>
+  <dimension ref="A1:R116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LAM WONG NELLY ANGELA</t>
+          <t>LEM S.A.</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LEM S.A.</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -4977,7 +4977,7 @@
         <v>0</v>
       </c>
       <c r="M75" s="2" t="n">
-        <v>0</v>
+        <v>347.34</v>
       </c>
       <c r="N75" s="2" t="n">
         <v>0</v>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5037,7 +5037,7 @@
         <v>0</v>
       </c>
       <c r="M76" s="2" t="n">
-        <v>347.34</v>
+        <v>0</v>
       </c>
       <c r="N76" s="2" t="n">
         <v>0</v>
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6837,7 +6837,7 @@
         <v>0</v>
       </c>
       <c r="M106" s="2" t="n">
-        <v>0</v>
+        <v>217.99</v>
       </c>
       <c r="N106" s="2" t="n">
         <v>0</v>
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -6897,7 +6897,7 @@
         <v>0</v>
       </c>
       <c r="M107" s="2" t="n">
-        <v>217.99</v>
+        <v>0</v>
       </c>
       <c r="N107" s="2" t="n">
         <v>0</v>
@@ -6923,7 +6923,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -7043,7 +7043,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -7103,7 +7103,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
@@ -7163,7 +7163,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
@@ -7223,7 +7223,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
@@ -7396,144 +7396,84 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R116" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="C117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
-        </is>
-      </c>
-      <c r="D117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
-        </is>
-      </c>
-      <c r="E117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
-        </is>
-      </c>
-      <c r="F117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
-        </is>
-      </c>
-      <c r="G117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
-        </is>
-      </c>
-      <c r="H117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
-        </is>
-      </c>
-      <c r="I117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
-        </is>
-      </c>
-      <c r="J117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
-        </is>
-      </c>
-      <c r="K117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
-        </is>
-      </c>
-      <c r="L117" s="3" t="inlineStr">
-        <is>
-          <t>2 de 115</t>
-        </is>
-      </c>
-      <c r="M117" s="3" t="inlineStr">
-        <is>
-          <t>4 de 115</t>
-        </is>
-      </c>
-      <c r="N117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
-        </is>
-      </c>
-      <c r="O117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
-        </is>
-      </c>
-      <c r="P117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
-        </is>
-      </c>
-      <c r="Q117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
-        </is>
-      </c>
-      <c r="R117" s="3" t="inlineStr">
-        <is>
-          <t>0 de 115</t>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
+        </is>
+      </c>
+      <c r="H116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
+        </is>
+      </c>
+      <c r="I116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
+        </is>
+      </c>
+      <c r="J116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
+        </is>
+      </c>
+      <c r="K116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
+        </is>
+      </c>
+      <c r="L116" s="3" t="inlineStr">
+        <is>
+          <t>2 de 114</t>
+        </is>
+      </c>
+      <c r="M116" s="3" t="inlineStr">
+        <is>
+          <t>4 de 114</t>
+        </is>
+      </c>
+      <c r="N116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
+        </is>
+      </c>
+      <c r="O116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
+        </is>
+      </c>
+      <c r="P116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
+        </is>
+      </c>
+      <c r="Q116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
+        </is>
+      </c>
+      <c r="R116" s="3" t="inlineStr">
+        <is>
+          <t>0 de 114</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-05-12 08:30:21
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R116"/>
+  <dimension ref="A1:R117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -863,7 +863,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ALCIVAR BUSTAMANTE ERNESTO EDUARDO</t>
+          <t>ALAVA PACHAY TEDDY ALBERTO</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -897,7 +897,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0</v>
+        <v>196.19</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -923,7 +923,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ALMEIDA CUATIN JHONATANN CARLOS</t>
+          <t>ALCIVAR BUSTAMANTE ERNESTO EDUARDO</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ANALUISA BELTRAN FABIAN OSWALDO</t>
+          <t>ALMEIDA CUATIN JHONATANN CARLOS</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ANGULO PARRALES CARMEN</t>
+          <t>ANALUISA BELTRAN FABIAN OSWALDO</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ARCE CANDO DENISSE YAJAIRA</t>
+          <t>ANGULO PARRALES CARMEN</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ARMIJO AGUILAR ROBERT LENIN</t>
+          <t>ARCE CANDO DENISSE YAJAIRA</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ARQUITECKSA S.A.</t>
+          <t>ARMIJO AGUILAR ROBERT LENIN</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AVILA TORRES RAFAEL ALEJANDRO</t>
+          <t>ARQUITECKSA S.A.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BRAVO MANZABA MARIA CECILIA</t>
+          <t>AVILA TORRES RAFAEL ALEJANDRO</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BRIONES GOMEZ ASLEY YAMILEXY</t>
+          <t>BRAVO MANZABA MARIA CECILIA</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BRITO MORALES MARIA SOLEDAD</t>
+          <t>BRIONES GOMEZ ASLEY YAMILEXY</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>BURGOS OLVERA VICENTE JAVIER</t>
+          <t>BRITO MORALES MARIA SOLEDAD</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
+          <t>BURGOS OLVERA VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
+          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1674,7 +1674,7 @@
         <v>0</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>-861.02</v>
+        <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
         <v>0</v>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
+          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1734,7 +1734,7 @@
         <v>0</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>0</v>
+        <v>-861.02</v>
       </c>
       <c r="M21" s="2" t="n">
         <v>0</v>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
+          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CARRANZA AVILEZ WILSON</t>
+          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CARRANZA AVILEZ WILSON</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CATAECSA S.A.</t>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CERAMICASAECUADOR S.A.</t>
+          <t>CATAECSA S.A.</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2154,7 +2154,7 @@
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>1561.97</v>
+        <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
         <v>0</v>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
+          <t>CERAMICASAECUADOR S.A.</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2214,10 +2214,10 @@
         <v>0</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>0</v>
+        <v>1561.97</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>314.51</v>
+        <v>0</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CHICA ALBAN GILMERTH HOMERO</t>
+          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2277,7 +2277,7 @@
         <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>0</v>
+        <v>314.51</v>
       </c>
       <c r="N30" s="2" t="n">
         <v>0</v>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>CHICA ALBAN GILMERTH HOMERO</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
+          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
+          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Carlos Meza Peña</t>
+          <t>CONSTRUMERCADO S.A.</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ECUARECYCLING S.A.</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>ECUARECYCLING S.A.</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3234,7 +3234,7 @@
         <v>0</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>293.94</v>
+        <v>0</v>
       </c>
       <c r="M46" s="2" t="n">
         <v>0</v>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3294,7 +3294,7 @@
         <v>0</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>0</v>
+        <v>293.94</v>
       </c>
       <c r="M47" s="2" t="n">
         <v>0</v>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3717,7 +3717,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>116.77</v>
+        <v>0</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3777,7 +3777,7 @@
         <v>0</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>0</v>
+        <v>116.77</v>
       </c>
       <c r="N55" s="2" t="n">
         <v>0</v>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LEM S.A.</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LEM S.A.</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -4977,7 +4977,7 @@
         <v>0</v>
       </c>
       <c r="M75" s="2" t="n">
-        <v>347.34</v>
+        <v>0</v>
       </c>
       <c r="N75" s="2" t="n">
         <v>0</v>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5037,7 +5037,7 @@
         <v>0</v>
       </c>
       <c r="M76" s="2" t="n">
-        <v>0</v>
+        <v>347.34</v>
       </c>
       <c r="N76" s="2" t="n">
         <v>0</v>
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6837,7 +6837,7 @@
         <v>0</v>
       </c>
       <c r="M106" s="2" t="n">
-        <v>217.99</v>
+        <v>0</v>
       </c>
       <c r="N106" s="2" t="n">
         <v>0</v>
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -6897,7 +6897,7 @@
         <v>0</v>
       </c>
       <c r="M107" s="2" t="n">
-        <v>0</v>
+        <v>217.99</v>
       </c>
       <c r="N107" s="2" t="n">
         <v>0</v>
@@ -6923,7 +6923,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -7043,7 +7043,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -7103,7 +7103,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
@@ -7163,7 +7163,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
@@ -7223,7 +7223,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
@@ -7343,137 +7343,197 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
+          <t>ZAZACORP S.A.</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R115" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
           <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
-      <c r="C115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R115" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="116">
-      <c r="C116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
-        </is>
-      </c>
-      <c r="D116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
-        </is>
-      </c>
-      <c r="E116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
-        </is>
-      </c>
-      <c r="F116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
-        </is>
-      </c>
-      <c r="G116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
-        </is>
-      </c>
-      <c r="H116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
-        </is>
-      </c>
-      <c r="I116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
-        </is>
-      </c>
-      <c r="J116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
-        </is>
-      </c>
-      <c r="K116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
-        </is>
-      </c>
-      <c r="L116" s="3" t="inlineStr">
-        <is>
-          <t>2 de 114</t>
-        </is>
-      </c>
-      <c r="M116" s="3" t="inlineStr">
-        <is>
-          <t>4 de 114</t>
-        </is>
-      </c>
-      <c r="N116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
-        </is>
-      </c>
-      <c r="O116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
-        </is>
-      </c>
-      <c r="P116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
-        </is>
-      </c>
-      <c r="Q116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
-        </is>
-      </c>
-      <c r="R116" s="3" t="inlineStr">
-        <is>
-          <t>0 de 114</t>
+      <c r="C116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R116" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
+        </is>
+      </c>
+      <c r="G117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
+        </is>
+      </c>
+      <c r="H117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
+        </is>
+      </c>
+      <c r="I117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
+        </is>
+      </c>
+      <c r="J117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
+        </is>
+      </c>
+      <c r="K117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
+        </is>
+      </c>
+      <c r="L117" s="3" t="inlineStr">
+        <is>
+          <t>2 de 115</t>
+        </is>
+      </c>
+      <c r="M117" s="3" t="inlineStr">
+        <is>
+          <t>5 de 115</t>
+        </is>
+      </c>
+      <c r="N117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
+        </is>
+      </c>
+      <c r="O117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
+        </is>
+      </c>
+      <c r="P117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
+        </is>
+      </c>
+      <c r="Q117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
+        </is>
+      </c>
+      <c r="R117" s="3" t="inlineStr">
+        <is>
+          <t>0 de 115</t>
         </is>
       </c>
     </row>
@@ -7488,7 +7548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G158"/>
+  <dimension ref="A1:G159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7680,7 +7740,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ALAY BELTRAN JOFRE IVAN</t>
+          <t>ALAVA PACHAY TEDDY ALBERTO</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -7693,7 +7753,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0</v>
+        <v>196.19</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>0</v>
@@ -7707,7 +7767,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ALCIVAR BUSTAMANTE ERNESTO EDUARDO</t>
+          <t>ALAY BELTRAN JOFRE IVAN</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -7734,7 +7794,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ALMEIDA CUATIN JHONATANN CARLOS</t>
+          <t>ALCIVAR BUSTAMANTE ERNESTO EDUARDO</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -7761,11 +7821,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ANALUISA BELTRAN FABIAN OSWALDO</t>
+          <t>ALMEIDA CUATIN JHONATANN CARLOS</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>841.65</v>
+        <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>0</v>
@@ -7788,11 +7848,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ANGUETA GAHON ISRRAEL PAUL</t>
+          <t>ANALUISA BELTRAN FABIAN OSWALDO</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0</v>
+        <v>841.65</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>0</v>
@@ -7815,7 +7875,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ANGULO PARRALES CARMEN</t>
+          <t>ANGUETA GAHON ISRRAEL PAUL</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -7842,7 +7902,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>APARTEC SA</t>
+          <t>ANGULO PARRALES CARMEN</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -7869,7 +7929,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ARCE CANDO DENISSE YAJAIRA</t>
+          <t>APARTEC SA</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -7896,7 +7956,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ARMIJO AGUILAR ROBERT LENIN</t>
+          <t>ARCE CANDO DENISSE YAJAIRA</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -7923,7 +7983,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ARQUITECKSA S.A.</t>
+          <t>ARMIJO AGUILAR ROBERT LENIN</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -7950,7 +8010,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ARTCATORCE S.A. ART14</t>
+          <t>ARQUITECKSA S.A.</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -7977,7 +8037,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ASTUDILLO SARMIENTO PAUL BISMARK</t>
+          <t>ARTCATORCE S.A. ART14</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -8004,7 +8064,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AVILA TORRES RAFAEL ALEJANDRO</t>
+          <t>ASTUDILLO SARMIENTO PAUL BISMARK</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -8031,7 +8091,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>AYORA GUEVARA MARIA DANIELA</t>
+          <t>AVILA TORRES RAFAEL ALEJANDRO</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -8058,7 +8118,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BRAVO MANZABA MARIA CECILIA</t>
+          <t>AYORA GUEVARA MARIA DANIELA</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -8085,7 +8145,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BRIONES GOMEZ ASLEY YAMILEXY</t>
+          <t>BRAVO MANZABA MARIA CECILIA</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -8112,14 +8172,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BRITO MORALES MARIA SOLEDAD</t>
+          <t>BRIONES GOMEZ ASLEY YAMILEXY</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>200.78</v>
+        <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>0</v>
@@ -8139,14 +8199,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BURGOS OLVERA VICENTE JAVIER</t>
+          <t>BRITO MORALES MARIA SOLEDAD</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>150.73</v>
+        <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0</v>
+        <v>200.78</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>0</v>
@@ -8166,11 +8226,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CABRERA ANDA PABLO HERNAN</t>
+          <t>BURGOS OLVERA VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0</v>
+        <v>150.73</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>0</v>
@@ -8193,7 +8253,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
+          <t>CABRERA ANDA PABLO HERNAN</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -8220,7 +8280,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
+          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -8230,10 +8290,10 @@
         <v>0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>861.02</v>
+        <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>-861.02</v>
+        <v>0</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -8247,20 +8307,20 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
+          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>86.95999999999999</v>
+        <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0</v>
+        <v>861.02</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0</v>
+        <v>-861.02</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>0</v>
@@ -8274,11 +8334,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
+          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0</v>
+        <v>86.95999999999999</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>0</v>
@@ -8301,7 +8361,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CARRANZA AVILEZ WILSON</t>
+          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -8328,7 +8388,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CARRANZA JARA LEONARDO GABRIEL</t>
+          <t>CARRANZA AVILEZ WILSON</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -8355,7 +8415,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CARRANZA JARA LEONARDO GABRIEL</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -8382,7 +8442,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CASCO PENA HUGO VLADIMIR</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -8409,11 +8469,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CASCO PENA HUGO VLADIMIR</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>84.75</v>
+        <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>0</v>
@@ -8436,17 +8496,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0</v>
+        <v>84.75</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>110.88</v>
+        <v>0</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>-0.29</v>
+        <v>0</v>
       </c>
       <c r="F35" s="2" t="n">
         <v>0</v>
@@ -8463,17 +8523,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CASTRO CEDILLO BLANCA KARINA</t>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0</v>
+        <v>110.88</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0</v>
+        <v>-0.29</v>
       </c>
       <c r="F36" s="2" t="n">
         <v>0</v>
@@ -8490,7 +8550,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CATAECSA S.A.</t>
+          <t>CASTRO CEDILLO BLANCA KARINA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -8500,7 +8560,7 @@
         <v>0</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>642.42</v>
+        <v>0</v>
       </c>
       <c r="F37" s="2" t="n">
         <v>0</v>
@@ -8517,20 +8577,20 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CERAMICASAECUADOR S.A.</t>
+          <t>CATAECSA S.A.</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>6219.57</v>
+        <v>0</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>4739.16</v>
+        <v>0</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>-1554.57</v>
+        <v>642.42</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>1561.97</v>
+        <v>0</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>0</v>
@@ -8544,20 +8604,20 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
+          <t>CERAMICASAECUADOR S.A.</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0</v>
+        <v>6219.57</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0</v>
+        <v>4739.16</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>1686.69</v>
+        <v>-1554.57</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>314.51</v>
+        <v>1561.97</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>0</v>
@@ -8571,7 +8631,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CHICA ALBAN GILMERTH HOMERO</t>
+          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -8581,10 +8641,10 @@
         <v>0</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0</v>
+        <v>1686.69</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0</v>
+        <v>314.51</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>0</v>
@@ -8598,7 +8658,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CHONG GONZALEZ WASHINGTON ALAN</t>
+          <t>CHICA ALBAN GILMERTH HOMERO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -8625,7 +8685,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>CHONG GONZALEZ WASHINGTON ALAN</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -8652,7 +8712,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -8679,11 +8739,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
+          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>54.87</v>
+        <v>0</v>
       </c>
       <c r="D44" s="2" t="n">
         <v>0</v>
@@ -8706,11 +8766,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTE DE CARGA PESADA ALAY EXPRESS S.A.</t>
+          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>0</v>
+        <v>54.87</v>
       </c>
       <c r="D45" s="2" t="n">
         <v>0</v>
@@ -8733,7 +8793,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
+          <t>COMPAÑIA DE TRANSPORTE DE CARGA PESADA ALAY EXPRESS S.A.</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -8760,17 +8820,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>1125.31</v>
+        <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>24.18</v>
+        <v>0</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>0</v>
@@ -8787,17 +8847,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CONTRERAS JIMMY</t>
+          <t>CONSTRUMERCADO S.A.</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0</v>
+        <v>1125.31</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0</v>
+        <v>24.18</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>0</v>
@@ -8814,14 +8874,14 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Carlos Meza Peña</t>
+          <t>CONTRERAS JIMMY</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>11.45</v>
+        <v>0</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>0</v>
@@ -8841,14 +8901,14 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0</v>
+        <v>11.45</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>0</v>
@@ -8868,11 +8928,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>220.35</v>
+        <v>0</v>
       </c>
       <c r="D51" s="2" t="n">
         <v>0</v>
@@ -8895,17 +8955,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>682.11</v>
+        <v>220.35</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>2674.35</v>
+        <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>333</v>
+        <v>0</v>
       </c>
       <c r="F52" s="2" t="n">
         <v>0</v>
@@ -8922,17 +8982,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ECUARECYCLING S.A.</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>0</v>
+        <v>682.11</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>0</v>
+        <v>2674.35</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0</v>
+        <v>333</v>
       </c>
       <c r="F53" s="2" t="n">
         <v>0</v>
@@ -8949,14 +9009,14 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>ECUARECYCLING S.A.</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>1110.99</v>
+        <v>0</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>0</v>
@@ -8976,14 +9036,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>0</v>
+        <v>1110.99</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>0</v>
@@ -9003,7 +9063,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -9030,7 +9090,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ESPINOZA JIMENEZ JOSE EUGENIO</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -9057,7 +9117,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>ESPINOZA JIMENEZ JOSE EUGENIO</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -9084,7 +9144,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -9111,7 +9171,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>FERNANDEZ VILLARREAL MARIELA JACQUELINE</t>
+          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -9138,7 +9198,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>FERNANDEZ VILLARREAL MARIELA JACQUELINE</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -9151,7 +9211,7 @@
         <v>0</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>293.94</v>
+        <v>0</v>
       </c>
       <c r="G61" s="2" t="n">
         <v>0</v>
@@ -9165,7 +9225,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -9178,7 +9238,7 @@
         <v>0</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0</v>
+        <v>293.94</v>
       </c>
       <c r="G62" s="2" t="n">
         <v>0</v>
@@ -9192,7 +9252,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -9219,7 +9279,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -9229,7 +9289,7 @@
         <v>0</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>833.03</v>
+        <v>0</v>
       </c>
       <c r="F64" s="2" t="n">
         <v>0</v>
@@ -9246,7 +9306,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -9256,7 +9316,7 @@
         <v>0</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0</v>
+        <v>833.03</v>
       </c>
       <c r="F65" s="2" t="n">
         <v>0</v>
@@ -9273,7 +9333,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -9300,7 +9360,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -9327,7 +9387,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>HEREDIA BAYAS FRANK MANUEL</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -9354,7 +9414,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>HERRERA RUIZ MARIA ISABEL</t>
+          <t>HEREDIA BAYAS FRANK MANUEL</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -9381,7 +9441,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
+          <t>HERRERA RUIZ MARIA ISABEL</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -9408,7 +9468,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>HILL PEÑA JONATHAN STUART</t>
+          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -9435,7 +9495,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>IMPORTADORA COMERCIAL BARROS IMPORBARSA S.A.</t>
+          <t>HILL PEÑA JONATHAN STUART</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -9462,7 +9522,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>IMPORTADORA COMERCIAL BARROS IMPORBARSA S.A.</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -9472,10 +9532,10 @@
         <v>0</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>88.3</v>
+        <v>0</v>
       </c>
       <c r="F73" s="2" t="n">
-        <v>116.77</v>
+        <v>0</v>
       </c>
       <c r="G73" s="2" t="n">
         <v>0</v>
@@ -9489,7 +9549,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -9499,10 +9559,10 @@
         <v>0</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>0</v>
+        <v>88.3</v>
       </c>
       <c r="F74" s="2" t="n">
-        <v>0</v>
+        <v>116.77</v>
       </c>
       <c r="G74" s="2" t="n">
         <v>0</v>
@@ -9516,7 +9576,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -9543,7 +9603,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -9553,7 +9613,7 @@
         <v>0</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>453.32</v>
+        <v>0</v>
       </c>
       <c r="F76" s="2" t="n">
         <v>0</v>
@@ -9570,7 +9630,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -9580,7 +9640,7 @@
         <v>0</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0</v>
+        <v>453.32</v>
       </c>
       <c r="F77" s="2" t="n">
         <v>0</v>
@@ -9597,7 +9657,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>JIMENEZ MORALES JACQUELINE ALEXANDRA</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -9624,7 +9684,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ MORALES JACQUELINE ALEXANDRA</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -9651,7 +9711,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>LAM WONG NELLY ANGELA</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -9678,7 +9738,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>LANDREX S.A.</t>
+          <t>LAM WONG NELLY ANGELA</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -9705,7 +9765,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>LECANSA S.A.</t>
+          <t>LANDREX S.A.</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -9732,7 +9792,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>LEM S.A.</t>
+          <t>LECANSA S.A.</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -9759,7 +9819,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LEM S.A.</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -9786,7 +9846,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -9813,7 +9873,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -9840,7 +9900,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -9867,7 +9927,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>La Casa Del Coleccionista S.A.S</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -9894,7 +9954,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>La Casa Del Coleccionista S.A.S</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -9921,7 +9981,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -9948,7 +10008,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MATERIALES DE CONSTRUCCION MACON S.A.</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -9975,7 +10035,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MATERIALES DE CONSTRUCCION MACON S.A.</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -10002,14 +10062,14 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D93" s="2" t="n">
-        <v>99.14</v>
+        <v>0</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>0</v>
@@ -10029,14 +10089,14 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D94" s="2" t="n">
-        <v>0</v>
+        <v>99.14</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>0</v>
@@ -10056,7 +10116,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>MIELES SAN MARTIN JOHNNY JOEL</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -10083,7 +10143,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MIELES SAN MARTIN JOHNNY JOEL</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -10110,7 +10170,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -10137,7 +10197,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -10164,7 +10224,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>MORALES ESPINOZA DIEGO FERNANDO</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -10191,7 +10251,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES ESPINOZA DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -10218,14 +10278,14 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
-        <v>5212.87</v>
+        <v>0</v>
       </c>
       <c r="D101" s="2" t="n">
-        <v>3144.11</v>
+        <v>0</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>0</v>
@@ -10245,14 +10305,14 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
-        <v>0</v>
+        <v>5212.87</v>
       </c>
       <c r="D102" s="2" t="n">
-        <v>0</v>
+        <v>3144.11</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>0</v>
@@ -10272,7 +10332,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>MOSCOSO BLANCO JULIO ENRIQUE</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -10299,7 +10359,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>MOSCOSO MORALES ANNIE LISBETH</t>
+          <t>MOSCOSO BLANCO JULIO ENRIQUE</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -10326,7 +10386,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOSCOSO MORALES ANNIE LISBETH</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -10336,10 +10396,10 @@
         <v>0</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>347.34</v>
+        <v>0</v>
       </c>
       <c r="G105" s="2" t="n">
         <v>0</v>
@@ -10353,7 +10413,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -10363,10 +10423,10 @@
         <v>0</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>0</v>
+        <v>347.34</v>
       </c>
       <c r="G106" s="2" t="n">
         <v>0</v>
@@ -10380,7 +10440,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>MUÑOZ ALCIVAR ANGELA JUSTINA</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -10407,7 +10467,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ ALCIVAR ANGELA JUSTINA</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -10434,7 +10494,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>MUÑOZ MORAN ROBINSON JAVIER</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -10461,7 +10521,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ MORAN ROBINSON JAVIER</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -10488,7 +10548,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
@@ -10515,7 +10575,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>OLUNANEK S.A.</t>
+          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
@@ -10542,7 +10602,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>OLVERA SALCEDO LIDIA GEOMAR</t>
+          <t>OLUNANEK S.A.</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
@@ -10569,7 +10629,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>OLVERA SALCEDO LIDIA GEOMAR</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
@@ -10579,7 +10639,7 @@
         <v>0</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>346.79</v>
+        <v>0</v>
       </c>
       <c r="F114" s="2" t="n">
         <v>0</v>
@@ -10596,17 +10656,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D115" s="2" t="n">
-        <v>198.03</v>
+        <v>0</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>102.69</v>
+        <v>346.79</v>
       </c>
       <c r="F115" s="2" t="n">
         <v>0</v>
@@ -10623,17 +10683,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D116" s="2" t="n">
-        <v>0</v>
+        <v>198.03</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>0</v>
+        <v>102.69</v>
       </c>
       <c r="F116" s="2" t="n">
         <v>0</v>
@@ -10650,7 +10710,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
@@ -10677,17 +10737,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
-        <v>107.16</v>
+        <v>0</v>
       </c>
       <c r="D118" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>58.9</v>
+        <v>0</v>
       </c>
       <c r="F118" s="2" t="n">
         <v>0</v>
@@ -10704,17 +10764,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
-        <v>0</v>
+        <v>107.16</v>
       </c>
       <c r="D119" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>0</v>
+        <v>58.9</v>
       </c>
       <c r="F119" s="2" t="n">
         <v>0</v>
@@ -10731,7 +10791,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
@@ -10758,7 +10818,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>QUIROLA GOMEZ DIEGO FABRICIO</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
@@ -10785,7 +10845,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIROLA GOMEZ DIEGO FABRICIO</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
@@ -10812,7 +10872,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>RAMOS UGUÑA ERICK FABRICIO</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
@@ -10839,7 +10899,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>REALMIND S.A.</t>
+          <t>RAMOS UGUÑA ERICK FABRICIO</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
@@ -10866,7 +10926,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>REALMIND S.A.</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
@@ -10893,17 +10953,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D126" s="2" t="n">
-        <v>1390.66</v>
+        <v>0</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>1049.35</v>
+        <v>0</v>
       </c>
       <c r="F126" s="2" t="n">
         <v>0</v>
@@ -10920,17 +10980,17 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D127" s="2" t="n">
-        <v>0</v>
+        <v>1390.66</v>
       </c>
       <c r="E127" s="2" t="n">
-        <v>0</v>
+        <v>1049.35</v>
       </c>
       <c r="F127" s="2" t="n">
         <v>0</v>
@@ -10947,7 +11007,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>SAENZ ESPIN JOSE FERNANDO</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
@@ -10974,7 +11034,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>SAENZ ESPIN JOSE FERNANDO</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
@@ -11001,7 +11061,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
@@ -11028,17 +11088,17 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D131" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="E131" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="F131" s="2" t="n">
         <v>0</v>
@@ -11055,17 +11115,17 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>SERVICIO TECNICO DE DISTRIBUCION SERTECDI S.A.</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D132" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="E132" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="F132" s="2" t="n">
         <v>0</v>
@@ -11082,7 +11142,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>SILVA BLUM CARLOS ALFREDO</t>
+          <t>SERVICIO TECNICO DE DISTRIBUCION SERTECDI S.A.</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
@@ -11109,7 +11169,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SILVA BLUM CARLOS ALFREDO</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
@@ -11136,7 +11196,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
@@ -11163,7 +11223,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
@@ -11173,7 +11233,7 @@
         <v>0</v>
       </c>
       <c r="E136" s="2" t="n">
-        <v>107.46</v>
+        <v>0</v>
       </c>
       <c r="F136" s="2" t="n">
         <v>0</v>
@@ -11190,7 +11250,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
@@ -11200,7 +11260,7 @@
         <v>0</v>
       </c>
       <c r="E137" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="F137" s="2" t="n">
         <v>0</v>
@@ -11217,11 +11277,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
-        <v>34.56</v>
+        <v>0</v>
       </c>
       <c r="D138" s="2" t="n">
         <v>0</v>
@@ -11244,11 +11304,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
-        <v>21.58</v>
+        <v>34.56</v>
       </c>
       <c r="D139" s="2" t="n">
         <v>0</v>
@@ -11271,11 +11331,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
-        <v>719.26</v>
+        <v>21.58</v>
       </c>
       <c r="D140" s="2" t="n">
         <v>0</v>
@@ -11298,11 +11358,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
-        <v>0</v>
+        <v>719.26</v>
       </c>
       <c r="D141" s="2" t="n">
         <v>0</v>
@@ -11325,17 +11385,17 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C142" s="2" t="n">
-        <v>85.28</v>
+        <v>0</v>
       </c>
       <c r="D142" s="2" t="n">
-        <v>870.5</v>
+        <v>0</v>
       </c>
       <c r="E142" s="2" t="n">
-        <v>15.35</v>
+        <v>0</v>
       </c>
       <c r="F142" s="2" t="n">
         <v>0</v>
@@ -11352,17 +11412,17 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C143" s="2" t="n">
-        <v>0</v>
+        <v>85.28</v>
       </c>
       <c r="D143" s="2" t="n">
-        <v>0</v>
+        <v>870.5</v>
       </c>
       <c r="E143" s="2" t="n">
-        <v>0</v>
+        <v>15.35</v>
       </c>
       <c r="F143" s="2" t="n">
         <v>0</v>
@@ -11379,7 +11439,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C144" s="2" t="n">
@@ -11389,7 +11449,7 @@
         <v>0</v>
       </c>
       <c r="E144" s="2" t="n">
-        <v>50.16</v>
+        <v>0</v>
       </c>
       <c r="F144" s="2" t="n">
         <v>0</v>
@@ -11406,7 +11466,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C145" s="2" t="n">
@@ -11416,7 +11476,7 @@
         <v>0</v>
       </c>
       <c r="E145" s="2" t="n">
-        <v>0</v>
+        <v>50.16</v>
       </c>
       <c r="F145" s="2" t="n">
         <v>0</v>
@@ -11433,7 +11493,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C146" s="2" t="n">
@@ -11443,10 +11503,10 @@
         <v>0</v>
       </c>
       <c r="E146" s="2" t="n">
-        <v>176.6</v>
+        <v>0</v>
       </c>
       <c r="F146" s="2" t="n">
-        <v>217.99</v>
+        <v>0</v>
       </c>
       <c r="G146" s="2" t="n">
         <v>0</v>
@@ -11460,7 +11520,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C147" s="2" t="n">
@@ -11470,10 +11530,10 @@
         <v>0</v>
       </c>
       <c r="E147" s="2" t="n">
-        <v>0</v>
+        <v>176.6</v>
       </c>
       <c r="F147" s="2" t="n">
-        <v>0</v>
+        <v>217.99</v>
       </c>
       <c r="G147" s="2" t="n">
         <v>0</v>
@@ -11487,7 +11547,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C148" s="2" t="n">
@@ -11514,7 +11574,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C149" s="2" t="n">
@@ -11541,7 +11601,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>VILLARREAL ASANZA RODRIGO ALEXANDER</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C150" s="2" t="n">
@@ -11568,7 +11628,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLARREAL ASANZA RODRIGO ALEXANDER</t>
         </is>
       </c>
       <c r="C151" s="2" t="n">
@@ -11595,7 +11655,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C152" s="2" t="n">
@@ -11622,7 +11682,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C153" s="2" t="n">
@@ -11632,7 +11692,7 @@
         <v>0</v>
       </c>
       <c r="E153" s="2" t="n">
-        <v>3.94</v>
+        <v>0</v>
       </c>
       <c r="F153" s="2" t="n">
         <v>0</v>
@@ -11649,7 +11709,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C154" s="2" t="n">
@@ -11659,7 +11719,7 @@
         <v>0</v>
       </c>
       <c r="E154" s="2" t="n">
-        <v>0</v>
+        <v>3.94</v>
       </c>
       <c r="F154" s="2" t="n">
         <v>0</v>
@@ -11676,7 +11736,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C155" s="2" t="n">
@@ -11703,7 +11763,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C156" s="2" t="n">
@@ -11730,39 +11790,66 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D157" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E157" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F157" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
           <t>ZUÑIGA BUSTAMANTE ENRIQUE HAMLET</t>
         </is>
       </c>
-      <c r="C157" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D157" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E157" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F157" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G157" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="C158" s="4" t="n">
+      <c r="C158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G158" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="C159" s="4" t="n">
         <v>14521.7</v>
       </c>
-      <c r="D158" s="4" t="n">
+      <c r="D159" s="4" t="n">
         <v>15806.28</v>
       </c>
-      <c r="E158" s="4" t="n">
+      <c r="E159" s="4" t="n">
         <v>5516.26</v>
       </c>
-      <c r="F158" s="4" t="n">
-        <v>1991.5</v>
-      </c>
-      <c r="G158" s="4" t="n">
+      <c r="F159" s="4" t="n">
+        <v>2187.69</v>
+      </c>
+      <c r="G159" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-05-19 10:30:26
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -4617,7 +4617,7 @@
         <v>0</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>0</v>
+        <v>32.4</v>
       </c>
       <c r="N69" s="2" t="n">
         <v>0</v>
@@ -7388,7 +7388,7 @@
       </c>
       <c r="M115" s="3" t="inlineStr">
         <is>
-          <t>6 de 113</t>
+          <t>7 de 113</t>
         </is>
       </c>
       <c r="N115" s="3" t="inlineStr">
@@ -10063,7 +10063,7 @@
         <v>0</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>0</v>
+        <v>32.4</v>
       </c>
       <c r="G97" s="2" t="n">
         <v>0</v>
@@ -11727,7 +11727,7 @@
         <v>5457.36</v>
       </c>
       <c r="F159" s="4" t="n">
-        <v>3153.06</v>
+        <v>3185.46</v>
       </c>
       <c r="G159" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-22 08:30:21
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -5274,7 +5274,7 @@
         <v>0</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>0</v>
+        <v>192.19</v>
       </c>
       <c r="M80" s="2" t="n">
         <v>0</v>
@@ -7383,7 +7383,7 @@
       </c>
       <c r="L115" s="3" t="inlineStr">
         <is>
-          <t>3 de 113</t>
+          <t>4 de 113</t>
         </is>
       </c>
       <c r="M115" s="3" t="inlineStr">
@@ -10549,7 +10549,7 @@
         <v>346.79</v>
       </c>
       <c r="F115" s="2" t="n">
-        <v>0</v>
+        <v>192.19</v>
       </c>
       <c r="G115" s="2" t="n">
         <v>0</v>
@@ -11727,7 +11727,7 @@
         <v>5457.36</v>
       </c>
       <c r="F159" s="4" t="n">
-        <v>5520.88</v>
+        <v>5713.070000000001</v>
       </c>
       <c r="G159" s="4" t="n">
         <v>0</v>
@@ -11826,10 +11826,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1963.69</v>
+        <v>2155.88</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-1963.69</v>
+        <v>-2155.88</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -11869,13 +11869,13 @@
         <v>15133.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>6814.440000000001</v>
+        <v>7006.63</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>8319.059999999999</v>
+        <v>8126.87</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.4502884329467737</v>
+        <v>0.4629880728185813</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-05-26 10:30:23
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -2817,7 +2817,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>2272.8</v>
+        <v>3030.4</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -8875,7 +8875,7 @@
         <v>333</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>2272.8</v>
+        <v>3030.4</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>0</v>
@@ -11727,7 +11727,7 @@
         <v>5457.36</v>
       </c>
       <c r="F159" s="4" t="n">
-        <v>5713.070000000001</v>
+        <v>6470.67</v>
       </c>
       <c r="G159" s="4" t="n">
         <v>0</v>
@@ -11752,7 +11752,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11850,13 +11850,13 @@
         <v>15000</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>4850.75</v>
+        <v>5608.35</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>10149.25</v>
+        <v>9391.65</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.3233833333333334</v>
+        <v>0.37389</v>
       </c>
     </row>
     <row r="5">
@@ -11869,13 +11869,13 @@
         <v>15133.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>7006.63</v>
+        <v>7764.23</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>8126.87</v>
+        <v>7369.27</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.4629880728185813</v>
+        <v>0.5130491954934417</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-05-27 16:30:23
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -6657,7 +6657,7 @@
         <v>0</v>
       </c>
       <c r="M103" s="2" t="n">
-        <v>0</v>
+        <v>25.08</v>
       </c>
       <c r="N103" s="2" t="n">
         <v>0</v>
@@ -7388,7 +7388,7 @@
       </c>
       <c r="M115" s="3" t="inlineStr">
         <is>
-          <t>9 de 113</t>
+          <t>10 de 113</t>
         </is>
       </c>
       <c r="N115" s="3" t="inlineStr">
@@ -11359,7 +11359,7 @@
         <v>50.16</v>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0</v>
+        <v>25.08</v>
       </c>
       <c r="G145" s="2" t="n">
         <v>0</v>
@@ -11727,7 +11727,7 @@
         <v>5457.36</v>
       </c>
       <c r="F159" s="4" t="n">
-        <v>6470.67</v>
+        <v>6495.75</v>
       </c>
       <c r="G159" s="4" t="n">
         <v>0</v>
@@ -11850,13 +11850,13 @@
         <v>15000</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>5608.35</v>
+        <v>5633.43</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>9391.65</v>
+        <v>9366.57</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.37389</v>
+        <v>0.375562</v>
       </c>
     </row>
     <row r="5">
@@ -11869,13 +11869,13 @@
         <v>15133.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>21527.25</v>
+        <v>21552.33</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-6393.75</v>
+        <v>-6418.83</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1.42248984042026</v>
+        <v>1.42414709089107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-05-29 08:30:23
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R115"/>
+  <dimension ref="A1:R114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2817,7 +2817,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>2983.05</v>
+        <v>3030.4</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LEM S.A.</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4557,7 +4557,7 @@
         <v>0</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>0</v>
+        <v>32.4</v>
       </c>
       <c r="N68" s="2" t="n">
         <v>0</v>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4617,7 +4617,7 @@
         <v>0</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>32.4</v>
+        <v>0</v>
       </c>
       <c r="N69" s="2" t="n">
         <v>0</v>
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4917,7 +4917,7 @@
         <v>0</v>
       </c>
       <c r="M74" s="2" t="n">
-        <v>0</v>
+        <v>347.34</v>
       </c>
       <c r="N74" s="2" t="n">
         <v>0</v>
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -4977,7 +4977,7 @@
         <v>0</v>
       </c>
       <c r="M75" s="2" t="n">
-        <v>347.34</v>
+        <v>0</v>
       </c>
       <c r="N75" s="2" t="n">
         <v>0</v>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5214,7 +5214,7 @@
         <v>0</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>0</v>
+        <v>192.19</v>
       </c>
       <c r="M79" s="2" t="n">
         <v>0</v>
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5274,7 +5274,7 @@
         <v>0</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>192.19</v>
+        <v>0</v>
       </c>
       <c r="M80" s="2" t="n">
         <v>0</v>
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6417,7 +6417,7 @@
         <v>0</v>
       </c>
       <c r="M99" s="2" t="n">
-        <v>0</v>
+        <v>186.47</v>
       </c>
       <c r="N99" s="2" t="n">
         <v>0</v>
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6477,7 +6477,7 @@
         <v>0</v>
       </c>
       <c r="M100" s="2" t="n">
-        <v>186.47</v>
+        <v>0</v>
       </c>
       <c r="N100" s="2" t="n">
         <v>0</v>
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6597,7 +6597,7 @@
         <v>0</v>
       </c>
       <c r="M102" s="2" t="n">
-        <v>0</v>
+        <v>25.08</v>
       </c>
       <c r="N102" s="2" t="n">
         <v>0</v>
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6657,7 +6657,7 @@
         <v>0</v>
       </c>
       <c r="M103" s="2" t="n">
-        <v>25.08</v>
+        <v>0</v>
       </c>
       <c r="N103" s="2" t="n">
         <v>0</v>
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6717,7 +6717,7 @@
         <v>0</v>
       </c>
       <c r="M104" s="2" t="n">
-        <v>0</v>
+        <v>217.99</v>
       </c>
       <c r="N104" s="2" t="n">
         <v>0</v>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6777,7 +6777,7 @@
         <v>0</v>
       </c>
       <c r="M105" s="2" t="n">
-        <v>217.99</v>
+        <v>0</v>
       </c>
       <c r="N105" s="2" t="n">
         <v>0</v>
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -6923,7 +6923,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -7043,7 +7043,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -7103,7 +7103,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
@@ -7163,7 +7163,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
@@ -7223,7 +7223,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
@@ -7276,144 +7276,84 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R114" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="C115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
-        </is>
-      </c>
-      <c r="D115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
-        </is>
-      </c>
-      <c r="E115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
-        </is>
-      </c>
-      <c r="F115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
-        </is>
-      </c>
-      <c r="G115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
-        </is>
-      </c>
-      <c r="H115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
-        </is>
-      </c>
-      <c r="I115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
-        </is>
-      </c>
-      <c r="J115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
-        </is>
-      </c>
-      <c r="K115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
-        </is>
-      </c>
-      <c r="L115" s="3" t="inlineStr">
-        <is>
-          <t>4 de 113</t>
-        </is>
-      </c>
-      <c r="M115" s="3" t="inlineStr">
-        <is>
-          <t>10 de 113</t>
-        </is>
-      </c>
-      <c r="N115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
-        </is>
-      </c>
-      <c r="O115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
-        </is>
-      </c>
-      <c r="P115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
-        </is>
-      </c>
-      <c r="Q115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
-        </is>
-      </c>
-      <c r="R115" s="3" t="inlineStr">
-        <is>
-          <t>0 de 113</t>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="I114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="J114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="K114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="L114" s="3" t="inlineStr">
+        <is>
+          <t>4 de 112</t>
+        </is>
+      </c>
+      <c r="M114" s="3" t="inlineStr">
+        <is>
+          <t>10 de 112</t>
+        </is>
+      </c>
+      <c r="N114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="O114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="P114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="Q114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="R114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
         </is>
       </c>
     </row>
@@ -8875,7 +8815,7 @@
         <v>333</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>2983.05</v>
+        <v>3030.4</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>0</v>
@@ -11727,7 +11667,7 @@
         <v>5457.36</v>
       </c>
       <c r="F159" s="4" t="n">
-        <v>6448.400000000001</v>
+        <v>6495.75</v>
       </c>
       <c r="G159" s="4" t="n">
         <v>0</v>
@@ -11752,7 +11692,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11850,13 +11790,13 @@
         <v>15000</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>5586.08</v>
+        <v>5633.43</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>9413.92</v>
+        <v>9366.57</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.3724053333333333</v>
+        <v>0.375562</v>
       </c>
     </row>
     <row r="5">
@@ -11869,13 +11809,13 @@
         <v>15133.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>25964.02</v>
+        <v>26011.37</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-10830.52</v>
+        <v>-10877.87</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1.715665245977467</v>
+        <v>1.718794066144646</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-04 09:30:19
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -1833,7 +1833,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="F23" s="2" t="n">
         <v>0</v>
@@ -7228,7 +7228,7 @@
       </c>
       <c r="E113" s="3" t="inlineStr">
         <is>
-          <t>0 de 111</t>
+          <t>1 de 111</t>
         </is>
       </c>
       <c r="F113" s="3" t="inlineStr">
@@ -8161,7 +8161,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>0</v>
@@ -11580,7 +11580,7 @@
         <v>6624.3</v>
       </c>
       <c r="F158" s="4" t="n">
-        <v>747.15</v>
+        <v>854.61</v>
       </c>
       <c r="G158" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-05 08:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -5610,7 +5610,7 @@
         <v>0</v>
       </c>
       <c r="D86" s="2" t="n">
-        <v>0</v>
+        <v>685.85</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>0</v>
@@ -7223,7 +7223,7 @@
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>0 de 111</t>
+          <t>1 de 111</t>
         </is>
       </c>
       <c r="E113" s="3" t="inlineStr">
@@ -10699,7 +10699,7 @@
         <v>0</v>
       </c>
       <c r="F125" s="2" t="n">
-        <v>0</v>
+        <v>685.85</v>
       </c>
       <c r="G125" s="2" t="n">
         <v>0</v>
@@ -11580,7 +11580,7 @@
         <v>6624.3</v>
       </c>
       <c r="F158" s="4" t="n">
-        <v>708.6800000000001</v>
+        <v>1394.53</v>
       </c>
       <c r="G158" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-05 17:30:19
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -6408,7 +6408,7 @@
         <v>0</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0</v>
+        <v>28.32</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -7253,7 +7253,7 @@
       </c>
       <c r="J113" s="3" t="inlineStr">
         <is>
-          <t>1 de 111</t>
+          <t>2 de 111</t>
         </is>
       </c>
       <c r="K113" s="3" t="inlineStr">
@@ -11158,7 +11158,7 @@
         <v>0</v>
       </c>
       <c r="F142" s="2" t="n">
-        <v>0</v>
+        <v>28.32</v>
       </c>
       <c r="G142" s="2" t="n">
         <v>0</v>
@@ -11580,7 +11580,7 @@
         <v>6624.3</v>
       </c>
       <c r="F158" s="4" t="n">
-        <v>1394.53</v>
+        <v>1422.85</v>
       </c>
       <c r="G158" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-12 17:30:19
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -452,7 +452,7 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
@@ -2808,7 +2808,7 @@
         <v>0</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0</v>
+        <v>1070.94</v>
       </c>
       <c r="K39" s="2" t="n">
         <v>0</v>
@@ -6093,13 +6093,13 @@
         <v>0</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>0</v>
+        <v>83.3</v>
       </c>
       <c r="F94" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>0</v>
+        <v>59.25</v>
       </c>
       <c r="H94" s="2" t="n">
         <v>0</v>
@@ -7228,24 +7228,24 @@
       </c>
       <c r="E113" s="3" t="inlineStr">
         <is>
+          <t>2 de 111</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
           <t>1 de 111</t>
         </is>
       </c>
-      <c r="F113" s="3" t="inlineStr">
+      <c r="H113" s="3" t="inlineStr">
         <is>
           <t>0 de 111</t>
         </is>
       </c>
-      <c r="G113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
-      <c r="H113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
       <c r="I113" s="3" t="inlineStr">
         <is>
           <t>1 de 111</t>
@@ -7253,7 +7253,7 @@
       </c>
       <c r="J113" s="3" t="inlineStr">
         <is>
-          <t>2 de 111</t>
+          <t>3 de 111</t>
         </is>
       </c>
       <c r="K113" s="3" t="inlineStr">
@@ -8755,7 +8755,7 @@
         <v>0</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0</v>
+        <v>1070.94</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>0</v>
@@ -11023,7 +11023,7 @@
         <v>128.55</v>
       </c>
       <c r="F137" s="2" t="n">
-        <v>0</v>
+        <v>142.55</v>
       </c>
       <c r="G137" s="2" t="n">
         <v>0</v>
@@ -11580,7 +11580,7 @@
         <v>6624.3</v>
       </c>
       <c r="F158" s="4" t="n">
-        <v>3465.98</v>
+        <v>4679.47</v>
       </c>
       <c r="G158" s="4" t="n">
         <v>0</v>
@@ -11655,13 +11655,13 @@
         <v>133.5</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>59.25</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>133.5</v>
+        <v>74.25</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0</v>
+        <v>0.4438202247191011</v>
       </c>
     </row>
     <row r="3">
@@ -11679,10 +11679,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>14686.49</v>
+        <v>15840.73</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-14686.49</v>
+        <v>-15840.73</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -11722,13 +11722,13 @@
         <v>18333.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>17846.73</v>
+        <v>19060.22</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>486.7700000000004</v>
+        <v>-726.7199999999993</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.9734491504622685</v>
+        <v>1.039638912373524</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-16 10:30:20
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R112"/>
+  <dimension ref="A1:R113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1980,7 +1980,7 @@
         <v>47.92</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="O25" s="2" t="n">
         <v>0</v>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>FIENCO VILLACIS NARCISA ROCIO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3114,7 +3114,7 @@
         <v>0</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>0</v>
+        <v>92.81999999999999</v>
       </c>
       <c r="M44" s="2" t="n">
         <v>0</v>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3774,7 +3774,7 @@
         <v>0</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>138.47</v>
+        <v>0</v>
       </c>
       <c r="M55" s="2" t="n">
         <v>0</v>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3834,7 +3834,7 @@
         <v>0</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>0</v>
+        <v>138.47</v>
       </c>
       <c r="M56" s="2" t="n">
         <v>0</v>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4248,7 +4248,7 @@
         <v>0</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>12.72</v>
+        <v>0</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0</v>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4308,7 +4308,7 @@
         <v>0</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0</v>
+        <v>12.72</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5397,7 +5397,7 @@
         <v>0</v>
       </c>
       <c r="M82" s="2" t="n">
-        <v>2043.13</v>
+        <v>0</v>
       </c>
       <c r="N82" s="2" t="n">
         <v>0</v>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5457,7 +5457,7 @@
         <v>0</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>0</v>
+        <v>2043.13</v>
       </c>
       <c r="N83" s="2" t="n">
         <v>0</v>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,14 +5543,14 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D85" s="2" t="n">
-        <v>685.85</v>
+        <v>0</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>0</v>
@@ -5603,14 +5603,14 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D86" s="2" t="n">
-        <v>0</v>
+        <v>685.85</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>0</v>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6033,13 +6033,13 @@
         <v>0</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>83.3</v>
+        <v>0</v>
       </c>
       <c r="F93" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>59.25</v>
+        <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
         <v>0</v>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6093,13 +6093,13 @@
         <v>0</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>0</v>
+        <v>83.3</v>
       </c>
       <c r="F94" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>0</v>
+        <v>59.25</v>
       </c>
       <c r="H94" s="2" t="n">
         <v>0</v>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6348,7 +6348,7 @@
         <v>0</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>28.32</v>
+        <v>0</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6408,7 +6408,7 @@
         <v>0</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0</v>
+        <v>28.32</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -6923,7 +6923,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -7043,7 +7043,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -7103,137 +7103,197 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
+          <t>ZAZACORP S.A.</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R111" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
           <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
-      <c r="C111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R111" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="C112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="D112" s="3" t="inlineStr">
-        <is>
-          <t>1 de 110</t>
-        </is>
-      </c>
-      <c r="E112" s="3" t="inlineStr">
-        <is>
-          <t>2 de 110</t>
-        </is>
-      </c>
-      <c r="F112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="G112" s="3" t="inlineStr">
-        <is>
-          <t>1 de 110</t>
-        </is>
-      </c>
-      <c r="H112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="I112" s="3" t="inlineStr">
-        <is>
-          <t>1 de 110</t>
-        </is>
-      </c>
-      <c r="J112" s="3" t="inlineStr">
-        <is>
-          <t>3 de 110</t>
-        </is>
-      </c>
-      <c r="K112" s="3" t="inlineStr">
-        <is>
-          <t>1 de 110</t>
-        </is>
-      </c>
-      <c r="L112" s="3" t="inlineStr">
-        <is>
-          <t>1 de 110</t>
-        </is>
-      </c>
-      <c r="M112" s="3" t="inlineStr">
-        <is>
-          <t>2 de 110</t>
-        </is>
-      </c>
-      <c r="N112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="O112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="P112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="Q112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="R112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
+      <c r="C112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R112" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>1 de 111</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>2 de 111</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>1 de 111</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
+        </is>
+      </c>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
+          <t>1 de 111</t>
+        </is>
+      </c>
+      <c r="J113" s="3" t="inlineStr">
+        <is>
+          <t>3 de 111</t>
+        </is>
+      </c>
+      <c r="K113" s="3" t="inlineStr">
+        <is>
+          <t>1 de 111</t>
+        </is>
+      </c>
+      <c r="L113" s="3" t="inlineStr">
+        <is>
+          <t>2 de 111</t>
+        </is>
+      </c>
+      <c r="M113" s="3" t="inlineStr">
+        <is>
+          <t>2 de 111</t>
+        </is>
+      </c>
+      <c r="N113" s="3" t="inlineStr">
+        <is>
+          <t>1 de 111</t>
+        </is>
+      </c>
+      <c r="O113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
+        </is>
+      </c>
+      <c r="P113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
+        </is>
+      </c>
+      <c r="Q113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
+        </is>
+      </c>
+      <c r="R113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
         </is>
       </c>
     </row>
@@ -7248,7 +7308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G158"/>
+  <dimension ref="A1:G159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8236,7 +8296,7 @@
         <v>43.2</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>47.92</v>
+        <v>125.91</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>0</v>
@@ -8898,7 +8958,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>FIENCO VILLACIS NARCISA ROCIO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -8908,10 +8968,10 @@
         <v>0</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>293.94</v>
+        <v>0</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>0</v>
+        <v>92.81999999999999</v>
       </c>
       <c r="G61" s="2" t="n">
         <v>0</v>
@@ -8925,7 +8985,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -8935,7 +8995,7 @@
         <v>0</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0</v>
+        <v>293.94</v>
       </c>
       <c r="F62" s="2" t="n">
         <v>0</v>
@@ -8952,7 +9012,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -8979,14 +9039,14 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>833.03</v>
+        <v>0</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>0</v>
@@ -9006,14 +9066,14 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0</v>
+        <v>833.03</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>0</v>
@@ -9033,7 +9093,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -9060,7 +9120,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -9087,7 +9147,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>HEREDIA BAYAS FRANK MANUEL</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -9114,7 +9174,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>HERRERA RUIZ MARIA ISABEL</t>
+          <t>HEREDIA BAYAS FRANK MANUEL</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -9141,7 +9201,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
+          <t>HERRERA RUIZ MARIA ISABEL</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -9168,7 +9228,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>HILL PEÑA JONATHAN STUART</t>
+          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -9195,7 +9255,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>IMPORTADORA COMERCIAL BARROS IMPORBARSA S.A.</t>
+          <t>HILL PEÑA JONATHAN STUART</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -9222,17 +9282,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>IMPORTADORA COMERCIAL BARROS IMPORBARSA S.A.</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D73" s="2" t="n">
-        <v>88.3</v>
+        <v>0</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>116.77</v>
+        <v>0</v>
       </c>
       <c r="F73" s="2" t="n">
         <v>0</v>
@@ -9249,17 +9309,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D74" s="2" t="n">
-        <v>0</v>
+        <v>88.3</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>0</v>
+        <v>116.77</v>
       </c>
       <c r="F74" s="2" t="n">
         <v>0</v>
@@ -9276,7 +9336,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -9303,20 +9363,20 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D76" s="2" t="n">
-        <v>453.32</v>
+        <v>0</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>778.9</v>
+        <v>0</v>
       </c>
       <c r="F76" s="2" t="n">
-        <v>138.47</v>
+        <v>0</v>
       </c>
       <c r="G76" s="2" t="n">
         <v>0</v>
@@ -9330,20 +9390,20 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="2" t="n">
-        <v>0</v>
+        <v>453.32</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0</v>
+        <v>778.9</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>0</v>
+        <v>138.47</v>
       </c>
       <c r="G77" s="2" t="n">
         <v>0</v>
@@ -9357,7 +9417,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>JIMENEZ MORALES JACQUELINE ALEXANDRA</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -9384,7 +9444,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ MORALES JACQUELINE ALEXANDRA</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -9411,7 +9471,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>LAM WONG NELLY ANGELA</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -9438,7 +9498,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>LANDREX S.A.</t>
+          <t>LAM WONG NELLY ANGELA</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -9465,7 +9525,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>LECANSA S.A.</t>
+          <t>LANDREX S.A.</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -9492,7 +9552,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>LEM S.A.</t>
+          <t>LECANSA S.A.</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -9519,7 +9579,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LEM S.A.</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -9546,7 +9606,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -9573,7 +9633,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -9600,7 +9660,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -9627,7 +9687,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>La Casa Del Coleccionista S.A.S</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -9654,7 +9714,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>La Casa Del Coleccionista S.A.S</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -9681,7 +9741,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -9708,7 +9768,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MATERIALES DE CONSTRUCCION MACON S.A.</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -9735,7 +9795,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MATERIALES DE CONSTRUCCION MACON S.A.</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -9748,7 +9808,7 @@
         <v>0</v>
       </c>
       <c r="F92" s="2" t="n">
-        <v>12.72</v>
+        <v>0</v>
       </c>
       <c r="G92" s="2" t="n">
         <v>0</v>
@@ -9762,11 +9822,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
-        <v>99.14</v>
+        <v>0</v>
       </c>
       <c r="D93" s="2" t="n">
         <v>0</v>
@@ -9775,7 +9835,7 @@
         <v>0</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0</v>
+        <v>12.72</v>
       </c>
       <c r="G93" s="2" t="n">
         <v>0</v>
@@ -9789,11 +9849,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
-        <v>0</v>
+        <v>99.14</v>
       </c>
       <c r="D94" s="2" t="n">
         <v>0</v>
@@ -9816,7 +9876,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>MIELES SAN MARTIN JOHNNY JOEL</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -9843,7 +9903,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MIELES SAN MARTIN JOHNNY JOEL</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -9853,7 +9913,7 @@
         <v>0</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>32.4</v>
+        <v>0</v>
       </c>
       <c r="F96" s="2" t="n">
         <v>0</v>
@@ -9870,7 +9930,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -9880,7 +9940,7 @@
         <v>0</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>0</v>
+        <v>32.4</v>
       </c>
       <c r="F97" s="2" t="n">
         <v>0</v>
@@ -9897,7 +9957,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -9924,7 +9984,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>MORALES ESPINOZA DIEGO FERNANDO</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -9951,7 +10011,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES ESPINOZA DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -9978,11 +10038,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
-        <v>3144.11</v>
+        <v>0</v>
       </c>
       <c r="D101" s="2" t="n">
         <v>0</v>
@@ -10005,11 +10065,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
-        <v>0</v>
+        <v>3144.11</v>
       </c>
       <c r="D102" s="2" t="n">
         <v>0</v>
@@ -10032,7 +10092,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>MOSCOSO BLANCO JULIO ENRIQUE</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -10059,7 +10119,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>MOSCOSO MORALES ANNIE LISBETH</t>
+          <t>MOSCOSO BLANCO JULIO ENRIQUE</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -10086,17 +10146,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOSCOSO MORALES ANNIE LISBETH</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D105" s="2" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>347.34</v>
+        <v>0</v>
       </c>
       <c r="F105" s="2" t="n">
         <v>0</v>
@@ -10113,17 +10173,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D106" s="2" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>0</v>
+        <v>347.34</v>
       </c>
       <c r="F106" s="2" t="n">
         <v>0</v>
@@ -10140,7 +10200,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>MUÑOZ ALCIVAR ANGELA JUSTINA</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -10167,7 +10227,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ ALCIVAR ANGELA JUSTINA</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -10194,7 +10254,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>MUÑOZ MORAN ROBINSON JAVIER</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -10221,7 +10281,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ MORAN ROBINSON JAVIER</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -10248,7 +10308,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
@@ -10275,7 +10335,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>OLUNANEK S.A.</t>
+          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
@@ -10302,7 +10362,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>OLVERA SALCEDO LIDIA GEOMAR</t>
+          <t>OLUNANEK S.A.</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
@@ -10329,17 +10389,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>OLVERA SALCEDO LIDIA GEOMAR</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D114" s="2" t="n">
-        <v>346.79</v>
+        <v>0</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>192.19</v>
+        <v>0</v>
       </c>
       <c r="F114" s="2" t="n">
         <v>0</v>
@@ -10356,17 +10416,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
-        <v>198.03</v>
+        <v>0</v>
       </c>
       <c r="D115" s="2" t="n">
-        <v>102.69</v>
+        <v>346.79</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>0</v>
+        <v>192.19</v>
       </c>
       <c r="F115" s="2" t="n">
         <v>0</v>
@@ -10383,14 +10443,14 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
-        <v>0</v>
+        <v>198.03</v>
       </c>
       <c r="D116" s="2" t="n">
-        <v>0</v>
+        <v>102.69</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>0</v>
@@ -10410,7 +10470,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
@@ -10437,7 +10497,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
@@ -10464,7 +10524,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
@@ -10477,7 +10537,7 @@
         <v>0</v>
       </c>
       <c r="F119" s="2" t="n">
-        <v>2043.13</v>
+        <v>0</v>
       </c>
       <c r="G119" s="2" t="n">
         <v>0</v>
@@ -10491,7 +10551,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>QUIROLA GOMEZ DIEGO FABRICIO</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
@@ -10504,7 +10564,7 @@
         <v>0</v>
       </c>
       <c r="F120" s="2" t="n">
-        <v>0</v>
+        <v>2043.13</v>
       </c>
       <c r="G120" s="2" t="n">
         <v>0</v>
@@ -10518,7 +10578,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIROLA GOMEZ DIEGO FABRICIO</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
@@ -10545,7 +10605,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>RAMOS UGUÑA ERICK FABRICIO</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
@@ -10572,7 +10632,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>REALMIND S.A.</t>
+          <t>RAMOS UGUÑA ERICK FABRICIO</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
@@ -10599,7 +10659,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>REALMIND S.A.</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
@@ -10626,20 +10686,20 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
-        <v>1390.66</v>
+        <v>0</v>
       </c>
       <c r="D125" s="2" t="n">
-        <v>1049.35</v>
+        <v>0</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F125" s="2" t="n">
-        <v>685.85</v>
+        <v>0</v>
       </c>
       <c r="G125" s="2" t="n">
         <v>0</v>
@@ -10653,20 +10713,20 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
-        <v>0</v>
+        <v>1390.66</v>
       </c>
       <c r="D126" s="2" t="n">
-        <v>0</v>
+        <v>1049.35</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F126" s="2" t="n">
-        <v>0</v>
+        <v>685.85</v>
       </c>
       <c r="G126" s="2" t="n">
         <v>0</v>
@@ -10680,7 +10740,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>SAENZ ESPIN JOSE FERNANDO</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
@@ -10707,7 +10767,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>SAENZ ESPIN JOSE FERNANDO</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
@@ -10734,7 +10794,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
@@ -10761,14 +10821,14 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="D130" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="E130" s="2" t="n">
         <v>0</v>
@@ -10788,14 +10848,14 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>SERVICIO TECNICO DE DISTRIBUCION SERTECDI S.A.</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="D131" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="E131" s="2" t="n">
         <v>0</v>
@@ -10815,7 +10875,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>SILVA BLUM CARLOS ALFREDO</t>
+          <t>SERVICIO TECNICO DE DISTRIBUCION SERTECDI S.A.</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
@@ -10842,7 +10902,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SILVA BLUM CARLOS ALFREDO</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
@@ -10869,7 +10929,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
@@ -10896,14 +10956,14 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D135" s="2" t="n">
-        <v>107.46</v>
+        <v>0</v>
       </c>
       <c r="E135" s="2" t="n">
         <v>0</v>
@@ -10923,14 +10983,14 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D136" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="E136" s="2" t="n">
         <v>0</v>
@@ -10950,7 +11010,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
@@ -10960,10 +11020,10 @@
         <v>0</v>
       </c>
       <c r="E137" s="2" t="n">
-        <v>128.55</v>
+        <v>0</v>
       </c>
       <c r="F137" s="2" t="n">
-        <v>142.55</v>
+        <v>0</v>
       </c>
       <c r="G137" s="2" t="n">
         <v>0</v>
@@ -10977,7 +11037,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
@@ -10987,10 +11047,10 @@
         <v>0</v>
       </c>
       <c r="E138" s="2" t="n">
-        <v>19.42</v>
+        <v>128.55</v>
       </c>
       <c r="F138" s="2" t="n">
-        <v>0</v>
+        <v>142.55</v>
       </c>
       <c r="G138" s="2" t="n">
         <v>0</v>
@@ -11004,7 +11064,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
@@ -11014,7 +11074,7 @@
         <v>0</v>
       </c>
       <c r="E139" s="2" t="n">
-        <v>0</v>
+        <v>19.42</v>
       </c>
       <c r="F139" s="2" t="n">
         <v>0</v>
@@ -11031,7 +11091,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
@@ -11058,7 +11118,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
@@ -11068,7 +11128,7 @@
         <v>0</v>
       </c>
       <c r="E141" s="2" t="n">
-        <v>186.47</v>
+        <v>0</v>
       </c>
       <c r="F141" s="2" t="n">
         <v>0</v>
@@ -11085,20 +11145,20 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C142" s="2" t="n">
-        <v>870.5</v>
+        <v>0</v>
       </c>
       <c r="D142" s="2" t="n">
-        <v>15.35</v>
+        <v>0</v>
       </c>
       <c r="E142" s="2" t="n">
-        <v>0</v>
+        <v>186.47</v>
       </c>
       <c r="F142" s="2" t="n">
-        <v>28.32</v>
+        <v>0</v>
       </c>
       <c r="G142" s="2" t="n">
         <v>0</v>
@@ -11112,20 +11172,20 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C143" s="2" t="n">
-        <v>0</v>
+        <v>870.5</v>
       </c>
       <c r="D143" s="2" t="n">
-        <v>0</v>
+        <v>15.35</v>
       </c>
       <c r="E143" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F143" s="2" t="n">
-        <v>0</v>
+        <v>28.32</v>
       </c>
       <c r="G143" s="2" t="n">
         <v>0</v>
@@ -11139,17 +11199,17 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C144" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D144" s="2" t="n">
-        <v>50.16</v>
+        <v>0</v>
       </c>
       <c r="E144" s="2" t="n">
-        <v>25.08</v>
+        <v>0</v>
       </c>
       <c r="F144" s="2" t="n">
         <v>0</v>
@@ -11166,17 +11226,17 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C145" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D145" s="2" t="n">
-        <v>0</v>
+        <v>50.16</v>
       </c>
       <c r="E145" s="2" t="n">
-        <v>0</v>
+        <v>25.08</v>
       </c>
       <c r="F145" s="2" t="n">
         <v>0</v>
@@ -11193,17 +11253,17 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C146" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D146" s="2" t="n">
-        <v>176.6</v>
+        <v>0</v>
       </c>
       <c r="E146" s="2" t="n">
-        <v>217.99</v>
+        <v>0</v>
       </c>
       <c r="F146" s="2" t="n">
         <v>0</v>
@@ -11220,17 +11280,17 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C147" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D147" s="2" t="n">
-        <v>0</v>
+        <v>176.6</v>
       </c>
       <c r="E147" s="2" t="n">
-        <v>0</v>
+        <v>217.99</v>
       </c>
       <c r="F147" s="2" t="n">
         <v>0</v>
@@ -11247,7 +11307,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C148" s="2" t="n">
@@ -11274,7 +11334,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C149" s="2" t="n">
@@ -11301,7 +11361,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>VILLARREAL ASANZA RODRIGO ALEXANDER</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C150" s="2" t="n">
@@ -11328,7 +11388,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLARREAL ASANZA RODRIGO ALEXANDER</t>
         </is>
       </c>
       <c r="C151" s="2" t="n">
@@ -11355,7 +11415,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C152" s="2" t="n">
@@ -11382,14 +11442,14 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C153" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D153" s="2" t="n">
-        <v>3.94</v>
+        <v>0</v>
       </c>
       <c r="E153" s="2" t="n">
         <v>0</v>
@@ -11409,14 +11469,14 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C154" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D154" s="2" t="n">
-        <v>0</v>
+        <v>3.94</v>
       </c>
       <c r="E154" s="2" t="n">
         <v>0</v>
@@ -11436,7 +11496,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C155" s="2" t="n">
@@ -11463,7 +11523,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C156" s="2" t="n">
@@ -11490,39 +11550,66 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D157" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E157" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F157" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
           <t>ZUÑIGA BUSTAMANTE ENRIQUE HAMLET</t>
         </is>
       </c>
-      <c r="C157" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D157" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E157" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F157" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G157" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="C158" s="4" t="n">
+      <c r="C158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G158" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="C159" s="4" t="n">
         <v>14680.97</v>
       </c>
-      <c r="D158" s="4" t="n">
+      <c r="D159" s="4" t="n">
         <v>5433.18</v>
       </c>
-      <c r="E158" s="4" t="n">
+      <c r="E159" s="4" t="n">
         <v>6624.3</v>
       </c>
-      <c r="F158" s="4" t="n">
-        <v>4727.39</v>
-      </c>
-      <c r="G158" s="4" t="n">
+      <c r="F159" s="4" t="n">
+        <v>4898.2</v>
+      </c>
+      <c r="G159" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11619,10 +11706,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>15840.73</v>
+        <v>16011.54</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-15840.73</v>
+        <v>-16011.54</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -11662,13 +11749,13 @@
         <v>18333.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>19108.14</v>
+        <v>19278.95</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-774.6399999999994</v>
+        <v>-945.4500000000007</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1.042252706793575</v>
+        <v>1.05156953118608</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-16 13:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -4308,7 +4308,7 @@
         <v>0</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>12.72</v>
+        <v>39.4</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -9835,7 +9835,7 @@
         <v>0</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>12.72</v>
+        <v>39.4</v>
       </c>
       <c r="G93" s="2" t="n">
         <v>0</v>
@@ -11607,7 +11607,7 @@
         <v>6624.3</v>
       </c>
       <c r="F159" s="4" t="n">
-        <v>4898.2</v>
+        <v>4924.88</v>
       </c>
       <c r="G159" s="4" t="n">
         <v>0</v>
@@ -11706,10 +11706,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>16011.54</v>
+        <v>16038.22</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-16011.54</v>
+        <v>-16038.22</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -11749,13 +11749,13 @@
         <v>18333.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>19278.95</v>
+        <v>19305.63</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-945.4500000000007</v>
+        <v>-972.1299999999992</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1.05156953118608</v>
+        <v>1.053024790683721</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-17 16:30:19
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R113"/>
+  <dimension ref="A1:R114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3834,7 +3834,7 @@
         <v>0</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>138.47</v>
+        <v>0</v>
       </c>
       <c r="M56" s="2" t="n">
         <v>0</v>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3894,7 +3894,7 @@
         <v>0</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>0</v>
+        <v>138.47</v>
       </c>
       <c r="M57" s="2" t="n">
         <v>0</v>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4308,7 +4308,7 @@
         <v>0</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>39.4</v>
+        <v>0</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4368,7 +4368,7 @@
         <v>0</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0</v>
+        <v>39.4</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5457,7 +5457,7 @@
         <v>0</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>2054.5</v>
+        <v>0</v>
       </c>
       <c r="N83" s="2" t="n">
         <v>0</v>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5517,7 +5517,7 @@
         <v>0</v>
       </c>
       <c r="M84" s="2" t="n">
-        <v>0</v>
+        <v>2054.5</v>
       </c>
       <c r="N84" s="2" t="n">
         <v>0</v>
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,14 +5603,14 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D86" s="2" t="n">
-        <v>685.85</v>
+        <v>0</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>0</v>
@@ -5663,14 +5663,14 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D87" s="2" t="n">
-        <v>0</v>
+        <v>685.85</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>0</v>
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6093,13 +6093,13 @@
         <v>0</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>83.3</v>
+        <v>0</v>
       </c>
       <c r="F94" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>59.25</v>
+        <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
         <v>0</v>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6153,13 +6153,13 @@
         <v>0</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>0</v>
+        <v>83.3</v>
       </c>
       <c r="F95" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>0</v>
+        <v>59.25</v>
       </c>
       <c r="H95" s="2" t="n">
         <v>0</v>
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6408,7 +6408,7 @@
         <v>0</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>28.32</v>
+        <v>0</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6468,7 +6468,7 @@
         <v>0</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0</v>
+        <v>28.32</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -6923,7 +6923,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -7043,7 +7043,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -7103,7 +7103,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
@@ -7163,137 +7163,197 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
+          <t>ZAZACORP S.A.</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R112" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
           <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
-      <c r="C112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R112" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="C113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
-      <c r="D113" s="3" t="inlineStr">
-        <is>
-          <t>1 de 111</t>
-        </is>
-      </c>
-      <c r="E113" s="3" t="inlineStr">
-        <is>
-          <t>2 de 111</t>
-        </is>
-      </c>
-      <c r="F113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
-      <c r="G113" s="3" t="inlineStr">
-        <is>
-          <t>1 de 111</t>
-        </is>
-      </c>
-      <c r="H113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
-      <c r="I113" s="3" t="inlineStr">
-        <is>
-          <t>1 de 111</t>
-        </is>
-      </c>
-      <c r="J113" s="3" t="inlineStr">
-        <is>
-          <t>3 de 111</t>
-        </is>
-      </c>
-      <c r="K113" s="3" t="inlineStr">
-        <is>
-          <t>1 de 111</t>
-        </is>
-      </c>
-      <c r="L113" s="3" t="inlineStr">
-        <is>
-          <t>2 de 111</t>
-        </is>
-      </c>
-      <c r="M113" s="3" t="inlineStr">
-        <is>
-          <t>2 de 111</t>
-        </is>
-      </c>
-      <c r="N113" s="3" t="inlineStr">
-        <is>
-          <t>1 de 111</t>
-        </is>
-      </c>
-      <c r="O113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
-      <c r="P113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
-      <c r="Q113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
-      <c r="R113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
+      <c r="C113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R113" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>1 de 112</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>2 de 112</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>1 de 112</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="I114" s="3" t="inlineStr">
+        <is>
+          <t>1 de 112</t>
+        </is>
+      </c>
+      <c r="J114" s="3" t="inlineStr">
+        <is>
+          <t>3 de 112</t>
+        </is>
+      </c>
+      <c r="K114" s="3" t="inlineStr">
+        <is>
+          <t>1 de 112</t>
+        </is>
+      </c>
+      <c r="L114" s="3" t="inlineStr">
+        <is>
+          <t>2 de 112</t>
+        </is>
+      </c>
+      <c r="M114" s="3" t="inlineStr">
+        <is>
+          <t>2 de 112</t>
+        </is>
+      </c>
+      <c r="N114" s="3" t="inlineStr">
+        <is>
+          <t>1 de 112</t>
+        </is>
+      </c>
+      <c r="O114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="P114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="Q114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
+        </is>
+      </c>
+      <c r="R114" s="3" t="inlineStr">
+        <is>
+          <t>0 de 112</t>
         </is>
       </c>
     </row>
@@ -7308,7 +7368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G159"/>
+  <dimension ref="A1:G160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9390,20 +9450,20 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D77" s="2" t="n">
-        <v>453.32</v>
+        <v>0</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>778.9</v>
+        <v>0</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>138.47</v>
+        <v>28.77</v>
       </c>
       <c r="G77" s="2" t="n">
         <v>0</v>
@@ -9417,20 +9477,20 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D78" s="2" t="n">
-        <v>0</v>
+        <v>453.32</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>0</v>
+        <v>778.9</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>0</v>
+        <v>138.47</v>
       </c>
       <c r="G78" s="2" t="n">
         <v>0</v>
@@ -9444,7 +9504,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>JIMENEZ MORALES JACQUELINE ALEXANDRA</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -9471,7 +9531,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ MORALES JACQUELINE ALEXANDRA</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -9498,7 +9558,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>LAM WONG NELLY ANGELA</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -9525,7 +9585,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>LANDREX S.A.</t>
+          <t>LAM WONG NELLY ANGELA</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -9552,7 +9612,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>LECANSA S.A.</t>
+          <t>LANDREX S.A.</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -9579,7 +9639,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>LEM S.A.</t>
+          <t>LECANSA S.A.</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -9606,7 +9666,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LEM S.A.</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -9633,7 +9693,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -9660,7 +9720,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -9687,7 +9747,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -9714,7 +9774,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>La Casa Del Coleccionista S.A.S</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -9741,7 +9801,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>La Casa Del Coleccionista S.A.S</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -9768,7 +9828,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -9795,7 +9855,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>MATERIALES DE CONSTRUCCION MACON S.A.</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -9822,7 +9882,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MATERIALES DE CONSTRUCCION MACON S.A.</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -9835,7 +9895,7 @@
         <v>0</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>39.4</v>
+        <v>0</v>
       </c>
       <c r="G93" s="2" t="n">
         <v>0</v>
@@ -9849,11 +9909,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
-        <v>99.14</v>
+        <v>0</v>
       </c>
       <c r="D94" s="2" t="n">
         <v>0</v>
@@ -9862,7 +9922,7 @@
         <v>0</v>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0</v>
+        <v>39.4</v>
       </c>
       <c r="G94" s="2" t="n">
         <v>0</v>
@@ -9876,11 +9936,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
-        <v>0</v>
+        <v>99.14</v>
       </c>
       <c r="D95" s="2" t="n">
         <v>0</v>
@@ -9903,7 +9963,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>MIELES SAN MARTIN JOHNNY JOEL</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -9930,7 +9990,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MIELES SAN MARTIN JOHNNY JOEL</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -9940,7 +10000,7 @@
         <v>0</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>32.4</v>
+        <v>0</v>
       </c>
       <c r="F97" s="2" t="n">
         <v>0</v>
@@ -9957,7 +10017,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -9967,7 +10027,7 @@
         <v>0</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>0</v>
+        <v>32.4</v>
       </c>
       <c r="F98" s="2" t="n">
         <v>0</v>
@@ -9984,7 +10044,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -10011,7 +10071,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>MORALES ESPINOZA DIEGO FERNANDO</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -10038,7 +10098,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES ESPINOZA DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -10065,11 +10125,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
-        <v>3144.11</v>
+        <v>0</v>
       </c>
       <c r="D102" s="2" t="n">
         <v>0</v>
@@ -10092,11 +10152,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
-        <v>0</v>
+        <v>3144.11</v>
       </c>
       <c r="D103" s="2" t="n">
         <v>0</v>
@@ -10119,7 +10179,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>MOSCOSO BLANCO JULIO ENRIQUE</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -10146,7 +10206,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>MOSCOSO MORALES ANNIE LISBETH</t>
+          <t>MOSCOSO BLANCO JULIO ENRIQUE</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -10173,17 +10233,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOSCOSO MORALES ANNIE LISBETH</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D106" s="2" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>347.34</v>
+        <v>0</v>
       </c>
       <c r="F106" s="2" t="n">
         <v>0</v>
@@ -10200,17 +10260,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D107" s="2" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>0</v>
+        <v>347.34</v>
       </c>
       <c r="F107" s="2" t="n">
         <v>0</v>
@@ -10227,7 +10287,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>MUÑOZ ALCIVAR ANGELA JUSTINA</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -10254,7 +10314,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ ALCIVAR ANGELA JUSTINA</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -10281,7 +10341,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>MUÑOZ MORAN ROBINSON JAVIER</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -10308,7 +10368,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ MORAN ROBINSON JAVIER</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
@@ -10335,7 +10395,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
@@ -10362,7 +10422,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>OLUNANEK S.A.</t>
+          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
@@ -10389,7 +10449,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>OLVERA SALCEDO LIDIA GEOMAR</t>
+          <t>OLUNANEK S.A.</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
@@ -10416,17 +10476,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>OLVERA SALCEDO LIDIA GEOMAR</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D115" s="2" t="n">
-        <v>346.79</v>
+        <v>0</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>192.19</v>
+        <v>0</v>
       </c>
       <c r="F115" s="2" t="n">
         <v>0</v>
@@ -10443,17 +10503,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
-        <v>198.03</v>
+        <v>0</v>
       </c>
       <c r="D116" s="2" t="n">
-        <v>102.69</v>
+        <v>346.79</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>0</v>
+        <v>192.19</v>
       </c>
       <c r="F116" s="2" t="n">
         <v>0</v>
@@ -10470,14 +10530,14 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
-        <v>0</v>
+        <v>198.03</v>
       </c>
       <c r="D117" s="2" t="n">
-        <v>0</v>
+        <v>102.69</v>
       </c>
       <c r="E117" s="2" t="n">
         <v>0</v>
@@ -10497,7 +10557,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
@@ -10524,7 +10584,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
@@ -10551,7 +10611,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
@@ -10564,7 +10624,7 @@
         <v>0</v>
       </c>
       <c r="F120" s="2" t="n">
-        <v>2054.5</v>
+        <v>0</v>
       </c>
       <c r="G120" s="2" t="n">
         <v>0</v>
@@ -10578,7 +10638,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>QUIROLA GOMEZ DIEGO FABRICIO</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
@@ -10591,7 +10651,7 @@
         <v>0</v>
       </c>
       <c r="F121" s="2" t="n">
-        <v>0</v>
+        <v>2054.5</v>
       </c>
       <c r="G121" s="2" t="n">
         <v>0</v>
@@ -10605,7 +10665,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIROLA GOMEZ DIEGO FABRICIO</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
@@ -10632,7 +10692,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>RAMOS UGUÑA ERICK FABRICIO</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
@@ -10659,7 +10719,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>REALMIND S.A.</t>
+          <t>RAMOS UGUÑA ERICK FABRICIO</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
@@ -10686,7 +10746,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>REALMIND S.A.</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
@@ -10713,20 +10773,20 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
-        <v>1390.66</v>
+        <v>0</v>
       </c>
       <c r="D126" s="2" t="n">
-        <v>1049.35</v>
+        <v>0</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F126" s="2" t="n">
-        <v>685.85</v>
+        <v>0</v>
       </c>
       <c r="G126" s="2" t="n">
         <v>0</v>
@@ -10740,20 +10800,20 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
-        <v>0</v>
+        <v>1390.66</v>
       </c>
       <c r="D127" s="2" t="n">
-        <v>0</v>
+        <v>1049.35</v>
       </c>
       <c r="E127" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F127" s="2" t="n">
-        <v>0</v>
+        <v>685.85</v>
       </c>
       <c r="G127" s="2" t="n">
         <v>0</v>
@@ -10767,7 +10827,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>SAENZ ESPIN JOSE FERNANDO</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
@@ -10794,7 +10854,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>SAENZ ESPIN JOSE FERNANDO</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
@@ -10821,7 +10881,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
@@ -10848,14 +10908,14 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="D131" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="E131" s="2" t="n">
         <v>0</v>
@@ -10875,14 +10935,14 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>SERVICIO TECNICO DE DISTRIBUCION SERTECDI S.A.</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="D132" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="E132" s="2" t="n">
         <v>0</v>
@@ -10902,7 +10962,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>SILVA BLUM CARLOS ALFREDO</t>
+          <t>SERVICIO TECNICO DE DISTRIBUCION SERTECDI S.A.</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
@@ -10929,7 +10989,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SILVA BLUM CARLOS ALFREDO</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
@@ -10956,7 +11016,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
@@ -10983,14 +11043,14 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D136" s="2" t="n">
-        <v>107.46</v>
+        <v>0</v>
       </c>
       <c r="E136" s="2" t="n">
         <v>0</v>
@@ -11010,14 +11070,14 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D137" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="E137" s="2" t="n">
         <v>0</v>
@@ -11037,7 +11097,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
@@ -11047,10 +11107,10 @@
         <v>0</v>
       </c>
       <c r="E138" s="2" t="n">
-        <v>128.55</v>
+        <v>0</v>
       </c>
       <c r="F138" s="2" t="n">
-        <v>142.55</v>
+        <v>0</v>
       </c>
       <c r="G138" s="2" t="n">
         <v>0</v>
@@ -11064,7 +11124,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
@@ -11074,10 +11134,10 @@
         <v>0</v>
       </c>
       <c r="E139" s="2" t="n">
-        <v>19.42</v>
+        <v>128.55</v>
       </c>
       <c r="F139" s="2" t="n">
-        <v>0</v>
+        <v>142.55</v>
       </c>
       <c r="G139" s="2" t="n">
         <v>0</v>
@@ -11091,7 +11151,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
@@ -11101,7 +11161,7 @@
         <v>0</v>
       </c>
       <c r="E140" s="2" t="n">
-        <v>0</v>
+        <v>19.42</v>
       </c>
       <c r="F140" s="2" t="n">
         <v>0</v>
@@ -11118,7 +11178,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
@@ -11145,7 +11205,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C142" s="2" t="n">
@@ -11155,7 +11215,7 @@
         <v>0</v>
       </c>
       <c r="E142" s="2" t="n">
-        <v>186.47</v>
+        <v>0</v>
       </c>
       <c r="F142" s="2" t="n">
         <v>0</v>
@@ -11172,20 +11232,20 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C143" s="2" t="n">
-        <v>870.5</v>
+        <v>0</v>
       </c>
       <c r="D143" s="2" t="n">
-        <v>15.35</v>
+        <v>0</v>
       </c>
       <c r="E143" s="2" t="n">
-        <v>0</v>
+        <v>186.47</v>
       </c>
       <c r="F143" s="2" t="n">
-        <v>28.32</v>
+        <v>0</v>
       </c>
       <c r="G143" s="2" t="n">
         <v>0</v>
@@ -11199,20 +11259,20 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C144" s="2" t="n">
-        <v>0</v>
+        <v>870.5</v>
       </c>
       <c r="D144" s="2" t="n">
-        <v>0</v>
+        <v>15.35</v>
       </c>
       <c r="E144" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F144" s="2" t="n">
-        <v>0</v>
+        <v>28.32</v>
       </c>
       <c r="G144" s="2" t="n">
         <v>0</v>
@@ -11226,17 +11286,17 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C145" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D145" s="2" t="n">
-        <v>50.16</v>
+        <v>0</v>
       </c>
       <c r="E145" s="2" t="n">
-        <v>25.08</v>
+        <v>0</v>
       </c>
       <c r="F145" s="2" t="n">
         <v>0</v>
@@ -11253,17 +11313,17 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C146" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D146" s="2" t="n">
-        <v>0</v>
+        <v>50.16</v>
       </c>
       <c r="E146" s="2" t="n">
-        <v>0</v>
+        <v>25.08</v>
       </c>
       <c r="F146" s="2" t="n">
         <v>0</v>
@@ -11280,17 +11340,17 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C147" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D147" s="2" t="n">
-        <v>176.6</v>
+        <v>0</v>
       </c>
       <c r="E147" s="2" t="n">
-        <v>217.99</v>
+        <v>0</v>
       </c>
       <c r="F147" s="2" t="n">
         <v>0</v>
@@ -11307,17 +11367,17 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C148" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D148" s="2" t="n">
-        <v>0</v>
+        <v>176.6</v>
       </c>
       <c r="E148" s="2" t="n">
-        <v>0</v>
+        <v>217.99</v>
       </c>
       <c r="F148" s="2" t="n">
         <v>0</v>
@@ -11334,7 +11394,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C149" s="2" t="n">
@@ -11361,7 +11421,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C150" s="2" t="n">
@@ -11388,7 +11448,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>VILLARREAL ASANZA RODRIGO ALEXANDER</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C151" s="2" t="n">
@@ -11415,7 +11475,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLARREAL ASANZA RODRIGO ALEXANDER</t>
         </is>
       </c>
       <c r="C152" s="2" t="n">
@@ -11442,7 +11502,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C153" s="2" t="n">
@@ -11469,14 +11529,14 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C154" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D154" s="2" t="n">
-        <v>3.94</v>
+        <v>0</v>
       </c>
       <c r="E154" s="2" t="n">
         <v>0</v>
@@ -11496,14 +11556,14 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C155" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D155" s="2" t="n">
-        <v>0</v>
+        <v>3.94</v>
       </c>
       <c r="E155" s="2" t="n">
         <v>0</v>
@@ -11523,7 +11583,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C156" s="2" t="n">
@@ -11550,7 +11610,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C157" s="2" t="n">
@@ -11577,39 +11637,66 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G158" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
           <t>ZUÑIGA BUSTAMANTE ENRIQUE HAMLET</t>
         </is>
       </c>
-      <c r="C158" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D158" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E158" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F158" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G158" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="C159" s="4" t="n">
+      <c r="C159" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D159" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E159" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F159" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="C160" s="4" t="n">
         <v>14680.97</v>
       </c>
-      <c r="D159" s="4" t="n">
+      <c r="D160" s="4" t="n">
         <v>5433.18</v>
       </c>
-      <c r="E159" s="4" t="n">
+      <c r="E160" s="4" t="n">
         <v>6624.3</v>
       </c>
-      <c r="F159" s="4" t="n">
-        <v>4936.25</v>
-      </c>
-      <c r="G159" s="4" t="n">
+      <c r="F160" s="4" t="n">
+        <v>4965.02</v>
+      </c>
+      <c r="G160" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11706,10 +11793,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>16184.34</v>
+        <v>16213.11</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-16184.34</v>
+        <v>-16213.11</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -11749,13 +11836,13 @@
         <v>18333.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>19463.12</v>
+        <v>19491.89</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-1129.620000000001</v>
+        <v>-1158.390000000001</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1.06161507622658</v>
+        <v>1.063184334687866</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-22 08:30:19
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R114"/>
+  <dimension ref="A1:R113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -683,7 +683,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AGUAS MARIÑO RICARDO MICHAEL</t>
+          <t>AGUILERA ANDRADE FAUSTO ROGELIO</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -743,7 +743,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AGUILERA ANDRADE FAUSTO ROGELIO</t>
+          <t>ALAVA PACHAY TEDDY ALBERTO</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -803,7 +803,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ALAVA PACHAY TEDDY ALBERTO</t>
+          <t>ALCIVAR BUSTAMANTE ERNESTO EDUARDO</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -863,7 +863,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ALCIVAR BUSTAMANTE ERNESTO EDUARDO</t>
+          <t>ALMEIDA CUATIN JHONATANN CARLOS</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -923,7 +923,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ALMEIDA CUATIN JHONATANN CARLOS</t>
+          <t>ANALUISA BELTRAN FABIAN OSWALDO</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ANALUISA BELTRAN FABIAN OSWALDO</t>
+          <t>ANGULO PARRALES CARMEN</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ANGULO PARRALES CARMEN</t>
+          <t>ARCE CANDO DENISSE YAJAIRA</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ARCE CANDO DENISSE YAJAIRA</t>
+          <t>ARMIJO AGUILAR ROBERT LENIN</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ARMIJO AGUILAR ROBERT LENIN</t>
+          <t>ARQUITECKSA S.A.</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ARQUITECKSA S.A.</t>
+          <t>BRAVO MANZABA MARIA CECILIA</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BRAVO MANZABA MARIA CECILIA</t>
+          <t>BRIONES GOMEZ ASLEY YAMILEXY</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BRIONES GOMEZ ASLEY YAMILEXY</t>
+          <t>BRITO MORALES MARIA SOLEDAD</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BRITO MORALES MARIA SOLEDAD</t>
+          <t>BURGOS OLVERA VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BURGOS OLVERA VICENTE JAVIER</t>
+          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
+          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
+          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
+          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
+          <t>CARRANZA AVILEZ WILSON</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1713,7 +1713,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="F21" s="2" t="n">
         <v>0</v>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CARRANZA AVILEZ WILSON</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1773,7 +1773,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>107.46</v>
+        <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0</v>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1917,10 +1917,10 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>47.92</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0</v>
+        <v>77.98999999999999</v>
       </c>
       <c r="O24" s="2" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
+          <t>CATAECSA S.A.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -1977,10 +1977,10 @@
         <v>0</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>47.92</v>
+        <v>0</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>77.98999999999999</v>
+        <v>0</v>
       </c>
       <c r="O25" s="2" t="n">
         <v>0</v>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CATAECSA S.A.</t>
+          <t>CERAMICASAECUADOR S.A.</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CERAMICASAECUADOR S.A.</t>
+          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2091,7 +2091,7 @@
         <v>0</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>0</v>
+        <v>12.9</v>
       </c>
       <c r="L27" s="2" t="n">
         <v>0</v>
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
+          <t>CHICA ALBAN GILMERTH HOMERO</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2151,7 +2151,7 @@
         <v>0</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>12.9</v>
+        <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>0</v>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CHICA ALBAN GILMERTH HOMERO</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
+          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
+          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Carlos Meza Peña</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2625,7 +2625,7 @@
         <v>0</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0</v>
+        <v>445.73</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0</v>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>ECUARECYCLING S.A.</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2685,10 +2685,10 @@
         <v>0</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>445.73</v>
+        <v>0</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0</v>
+        <v>1070.94</v>
       </c>
       <c r="K37" s="2" t="n">
         <v>0</v>
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ECUARECYCLING S.A.</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2748,7 +2748,7 @@
         <v>0</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>1070.94</v>
+        <v>0</v>
       </c>
       <c r="K38" s="2" t="n">
         <v>0</v>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
+          <t>FIENCO VILLACIS NARCISA ROCIO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3054,7 +3054,7 @@
         <v>0</v>
       </c>
       <c r="L43" s="2" t="n">
-        <v>0</v>
+        <v>92.81999999999999</v>
       </c>
       <c r="M43" s="2" t="n">
         <v>0</v>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>FIENCO VILLACIS NARCISA ROCIO</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3114,7 +3114,7 @@
         <v>0</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>92.81999999999999</v>
+        <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
         <v>0</v>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3834,7 +3834,7 @@
         <v>0</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>0</v>
+        <v>138.47</v>
       </c>
       <c r="M56" s="2" t="n">
         <v>0</v>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3894,7 +3894,7 @@
         <v>0</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>138.47</v>
+        <v>0</v>
       </c>
       <c r="M57" s="2" t="n">
         <v>0</v>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4308,7 +4308,7 @@
         <v>0</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0</v>
+        <v>39.4</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4368,7 +4368,7 @@
         <v>0</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>39.4</v>
+        <v>0</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5457,7 +5457,7 @@
         <v>0</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>0</v>
+        <v>2043.13</v>
       </c>
       <c r="N83" s="2" t="n">
         <v>0</v>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5517,7 +5517,7 @@
         <v>0</v>
       </c>
       <c r="M84" s="2" t="n">
-        <v>2043.13</v>
+        <v>0</v>
       </c>
       <c r="N84" s="2" t="n">
         <v>0</v>
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,14 +5603,14 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D86" s="2" t="n">
-        <v>0</v>
+        <v>685.85</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>0</v>
@@ -5663,14 +5663,14 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D87" s="2" t="n">
-        <v>685.85</v>
+        <v>0</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>0</v>
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6093,13 +6093,13 @@
         <v>0</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>0</v>
+        <v>83.3</v>
       </c>
       <c r="F94" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>0</v>
+        <v>59.25</v>
       </c>
       <c r="H94" s="2" t="n">
         <v>0</v>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6153,13 +6153,13 @@
         <v>0</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>83.3</v>
+        <v>0</v>
       </c>
       <c r="F95" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>59.25</v>
+        <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
         <v>0</v>
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6408,7 +6408,7 @@
         <v>0</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0</v>
+        <v>28.32</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6468,7 +6468,7 @@
         <v>0</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>28.32</v>
+        <v>0</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -6923,7 +6923,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -7043,7 +7043,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -7103,7 +7103,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
@@ -7163,7 +7163,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
@@ -7216,144 +7216,84 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q113" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R113" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="C114" s="3" t="inlineStr">
-        <is>
-          <t>0 de 112</t>
-        </is>
-      </c>
-      <c r="D114" s="3" t="inlineStr">
-        <is>
-          <t>1 de 112</t>
-        </is>
-      </c>
-      <c r="E114" s="3" t="inlineStr">
-        <is>
-          <t>2 de 112</t>
-        </is>
-      </c>
-      <c r="F114" s="3" t="inlineStr">
-        <is>
-          <t>0 de 112</t>
-        </is>
-      </c>
-      <c r="G114" s="3" t="inlineStr">
-        <is>
-          <t>1 de 112</t>
-        </is>
-      </c>
-      <c r="H114" s="3" t="inlineStr">
-        <is>
-          <t>0 de 112</t>
-        </is>
-      </c>
-      <c r="I114" s="3" t="inlineStr">
-        <is>
-          <t>1 de 112</t>
-        </is>
-      </c>
-      <c r="J114" s="3" t="inlineStr">
-        <is>
-          <t>3 de 112</t>
-        </is>
-      </c>
-      <c r="K114" s="3" t="inlineStr">
-        <is>
-          <t>1 de 112</t>
-        </is>
-      </c>
-      <c r="L114" s="3" t="inlineStr">
-        <is>
-          <t>2 de 112</t>
-        </is>
-      </c>
-      <c r="M114" s="3" t="inlineStr">
-        <is>
-          <t>2 de 112</t>
-        </is>
-      </c>
-      <c r="N114" s="3" t="inlineStr">
-        <is>
-          <t>1 de 112</t>
-        </is>
-      </c>
-      <c r="O114" s="3" t="inlineStr">
-        <is>
-          <t>0 de 112</t>
-        </is>
-      </c>
-      <c r="P114" s="3" t="inlineStr">
-        <is>
-          <t>0 de 112</t>
-        </is>
-      </c>
-      <c r="Q114" s="3" t="inlineStr">
-        <is>
-          <t>0 de 112</t>
-        </is>
-      </c>
-      <c r="R114" s="3" t="inlineStr">
-        <is>
-          <t>0 de 112</t>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>1 de 111</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>2 de 111</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>1 de 111</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
+        </is>
+      </c>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
+          <t>1 de 111</t>
+        </is>
+      </c>
+      <c r="J113" s="3" t="inlineStr">
+        <is>
+          <t>3 de 111</t>
+        </is>
+      </c>
+      <c r="K113" s="3" t="inlineStr">
+        <is>
+          <t>1 de 111</t>
+        </is>
+      </c>
+      <c r="L113" s="3" t="inlineStr">
+        <is>
+          <t>2 de 111</t>
+        </is>
+      </c>
+      <c r="M113" s="3" t="inlineStr">
+        <is>
+          <t>2 de 111</t>
+        </is>
+      </c>
+      <c r="N113" s="3" t="inlineStr">
+        <is>
+          <t>1 de 111</t>
+        </is>
+      </c>
+      <c r="O113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
+        </is>
+      </c>
+      <c r="P113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
+        </is>
+      </c>
+      <c r="Q113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
+        </is>
+      </c>
+      <c r="R113" s="3" t="inlineStr">
+        <is>
+          <t>0 de 111</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-06-22 09:30:22
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -777,7 +777,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0</v>
+        <v>24.11</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -7268,7 +7268,7 @@
       </c>
       <c r="M113" s="3" t="inlineStr">
         <is>
-          <t>2 de 111</t>
+          <t>3 de 111</t>
         </is>
       </c>
       <c r="N113" s="3" t="inlineStr">
@@ -7513,7 +7513,7 @@
         <v>196.19</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0</v>
+        <v>24.11</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>0</v>
@@ -11634,7 +11634,7 @@
         <v>6624.3</v>
       </c>
       <c r="F160" s="4" t="n">
-        <v>4962.25</v>
+        <v>4986.360000000001</v>
       </c>
       <c r="G160" s="4" t="n">
         <v>0</v>
@@ -11757,13 +11757,13 @@
         <v>18200</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>3241.87</v>
+        <v>3265.98</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>14958.13</v>
+        <v>14934.02</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.1781247252747253</v>
+        <v>0.1794494505494506</v>
       </c>
     </row>
     <row r="5">
@@ -11776,13 +11776,13 @@
         <v>18333.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>19522.83</v>
+        <v>19546.94</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-1189.33</v>
+        <v>-1213.439999999999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1.064871955709493</v>
+        <v>1.066187034663321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-24 08:30:20
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R113"/>
+  <dimension ref="A1:R112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3774,7 +3774,7 @@
         <v>0</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>0</v>
+        <v>138.47</v>
       </c>
       <c r="M55" s="2" t="n">
         <v>0</v>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3834,7 +3834,7 @@
         <v>0</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>138.47</v>
+        <v>0</v>
       </c>
       <c r="M56" s="2" t="n">
         <v>0</v>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4248,7 +4248,7 @@
         <v>0</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0</v>
+        <v>39.4</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0</v>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4308,7 +4308,7 @@
         <v>0</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>39.4</v>
+        <v>0</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5094,7 +5094,7 @@
         <v>0</v>
       </c>
       <c r="L77" s="2" t="n">
-        <v>0</v>
+        <v>99.25</v>
       </c>
       <c r="M77" s="2" t="n">
         <v>0</v>
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5154,7 +5154,7 @@
         <v>0</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>99.25</v>
+        <v>0</v>
       </c>
       <c r="M78" s="2" t="n">
         <v>0</v>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5397,7 +5397,7 @@
         <v>0</v>
       </c>
       <c r="M82" s="2" t="n">
-        <v>0</v>
+        <v>2043.13</v>
       </c>
       <c r="N82" s="2" t="n">
         <v>0</v>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5457,7 +5457,7 @@
         <v>0</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>2043.13</v>
+        <v>0</v>
       </c>
       <c r="N83" s="2" t="n">
         <v>0</v>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>RIOS CARRION ANGEL BENIGNO</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,14 +5543,14 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D85" s="2" t="n">
-        <v>0</v>
+        <v>685.85</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>0</v>
@@ -5603,14 +5603,14 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D86" s="2" t="n">
-        <v>685.85</v>
+        <v>0</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>0</v>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6033,13 +6033,13 @@
         <v>0</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>0</v>
+        <v>83.3</v>
       </c>
       <c r="F93" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>0</v>
+        <v>59.25</v>
       </c>
       <c r="H93" s="2" t="n">
         <v>0</v>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6093,13 +6093,13 @@
         <v>0</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>83.3</v>
+        <v>0</v>
       </c>
       <c r="F94" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>59.25</v>
+        <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
         <v>0</v>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6348,7 +6348,7 @@
         <v>0</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0</v>
+        <v>28.32</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6408,7 +6408,7 @@
         <v>0</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>28.32</v>
+        <v>0</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -6923,7 +6923,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -7043,7 +7043,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -7103,7 +7103,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
@@ -7156,144 +7156,84 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q112" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R112" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="C113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
-      <c r="D113" s="3" t="inlineStr">
-        <is>
-          <t>1 de 111</t>
-        </is>
-      </c>
-      <c r="E113" s="3" t="inlineStr">
-        <is>
-          <t>2 de 111</t>
-        </is>
-      </c>
-      <c r="F113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
-      <c r="G113" s="3" t="inlineStr">
-        <is>
-          <t>1 de 111</t>
-        </is>
-      </c>
-      <c r="H113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
-      <c r="I113" s="3" t="inlineStr">
-        <is>
-          <t>1 de 111</t>
-        </is>
-      </c>
-      <c r="J113" s="3" t="inlineStr">
-        <is>
-          <t>3 de 111</t>
-        </is>
-      </c>
-      <c r="K113" s="3" t="inlineStr">
-        <is>
-          <t>2 de 111</t>
-        </is>
-      </c>
-      <c r="L113" s="3" t="inlineStr">
-        <is>
-          <t>3 de 111</t>
-        </is>
-      </c>
-      <c r="M113" s="3" t="inlineStr">
-        <is>
-          <t>3 de 111</t>
-        </is>
-      </c>
-      <c r="N113" s="3" t="inlineStr">
-        <is>
-          <t>1 de 111</t>
-        </is>
-      </c>
-      <c r="O113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
-      <c r="P113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
-      <c r="Q113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
-        </is>
-      </c>
-      <c r="R113" s="3" t="inlineStr">
-        <is>
-          <t>0 de 111</t>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>1 de 110</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>2 de 110</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>1 de 110</t>
+        </is>
+      </c>
+      <c r="H112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="I112" s="3" t="inlineStr">
+        <is>
+          <t>1 de 110</t>
+        </is>
+      </c>
+      <c r="J112" s="3" t="inlineStr">
+        <is>
+          <t>3 de 110</t>
+        </is>
+      </c>
+      <c r="K112" s="3" t="inlineStr">
+        <is>
+          <t>2 de 110</t>
+        </is>
+      </c>
+      <c r="L112" s="3" t="inlineStr">
+        <is>
+          <t>3 de 110</t>
+        </is>
+      </c>
+      <c r="M112" s="3" t="inlineStr">
+        <is>
+          <t>3 de 110</t>
+        </is>
+      </c>
+      <c r="N112" s="3" t="inlineStr">
+        <is>
+          <t>1 de 110</t>
+        </is>
+      </c>
+      <c r="O112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="P112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="Q112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="R112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-06-25 08:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R112"/>
+  <dimension ref="A1:R110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3714,7 +3714,7 @@
         <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>0</v>
+        <v>138.47</v>
       </c>
       <c r="M54" s="2" t="n">
         <v>0</v>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3774,7 +3774,7 @@
         <v>0</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>138.47</v>
+        <v>0</v>
       </c>
       <c r="M55" s="2" t="n">
         <v>0</v>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4188,7 +4188,7 @@
         <v>0</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0</v>
+        <v>39.4</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>0</v>
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4248,7 +4248,7 @@
         <v>0</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>39.4</v>
+        <v>0</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0</v>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5034,7 +5034,7 @@
         <v>0</v>
       </c>
       <c r="L76" s="2" t="n">
-        <v>0</v>
+        <v>99.25</v>
       </c>
       <c r="M76" s="2" t="n">
         <v>0</v>
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5094,7 +5094,7 @@
         <v>0</v>
       </c>
       <c r="L77" s="2" t="n">
-        <v>99.25</v>
+        <v>0</v>
       </c>
       <c r="M77" s="2" t="n">
         <v>0</v>
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5337,7 +5337,7 @@
         <v>0</v>
       </c>
       <c r="M81" s="2" t="n">
-        <v>0</v>
+        <v>2043.13</v>
       </c>
       <c r="N81" s="2" t="n">
         <v>0</v>
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5397,7 +5397,7 @@
         <v>0</v>
       </c>
       <c r="M82" s="2" t="n">
-        <v>2043.13</v>
+        <v>0</v>
       </c>
       <c r="N82" s="2" t="n">
         <v>0</v>
@@ -5423,14 +5423,14 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D83" s="2" t="n">
-        <v>0</v>
+        <v>685.85</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>0</v>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,14 +5543,14 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D85" s="2" t="n">
-        <v>685.85</v>
+        <v>0</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>0</v>
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5913,13 +5913,13 @@
         <v>0</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>0</v>
+        <v>83.3</v>
       </c>
       <c r="F91" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>0</v>
+        <v>59.25</v>
       </c>
       <c r="H91" s="2" t="n">
         <v>0</v>
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6033,13 +6033,13 @@
         <v>0</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>83.3</v>
+        <v>0</v>
       </c>
       <c r="F93" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>59.25</v>
+        <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
         <v>0</v>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6228,7 +6228,7 @@
         <v>0</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0</v>
+        <v>28.32</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6348,7 +6348,7 @@
         <v>0</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>28.32</v>
+        <v>0</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -6923,7 +6923,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -7036,204 +7036,84 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>ZAZACORP S.A.</t>
-        </is>
-      </c>
-      <c r="C110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R110" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R111" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="C112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="D112" s="3" t="inlineStr">
-        <is>
-          <t>1 de 110</t>
-        </is>
-      </c>
-      <c r="E112" s="3" t="inlineStr">
-        <is>
-          <t>2 de 110</t>
-        </is>
-      </c>
-      <c r="F112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="G112" s="3" t="inlineStr">
-        <is>
-          <t>1 de 110</t>
-        </is>
-      </c>
-      <c r="H112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="I112" s="3" t="inlineStr">
-        <is>
-          <t>1 de 110</t>
-        </is>
-      </c>
-      <c r="J112" s="3" t="inlineStr">
-        <is>
-          <t>3 de 110</t>
-        </is>
-      </c>
-      <c r="K112" s="3" t="inlineStr">
-        <is>
-          <t>2 de 110</t>
-        </is>
-      </c>
-      <c r="L112" s="3" t="inlineStr">
-        <is>
-          <t>3 de 110</t>
-        </is>
-      </c>
-      <c r="M112" s="3" t="inlineStr">
-        <is>
-          <t>3 de 110</t>
-        </is>
-      </c>
-      <c r="N112" s="3" t="inlineStr">
-        <is>
-          <t>1 de 110</t>
-        </is>
-      </c>
-      <c r="O112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="P112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="Q112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="R112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>1 de 108</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>2 de 108</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>1 de 108</t>
+        </is>
+      </c>
+      <c r="H110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
+        </is>
+      </c>
+      <c r="I110" s="3" t="inlineStr">
+        <is>
+          <t>1 de 108</t>
+        </is>
+      </c>
+      <c r="J110" s="3" t="inlineStr">
+        <is>
+          <t>3 de 108</t>
+        </is>
+      </c>
+      <c r="K110" s="3" t="inlineStr">
+        <is>
+          <t>2 de 108</t>
+        </is>
+      </c>
+      <c r="L110" s="3" t="inlineStr">
+        <is>
+          <t>3 de 108</t>
+        </is>
+      </c>
+      <c r="M110" s="3" t="inlineStr">
+        <is>
+          <t>3 de 108</t>
+        </is>
+      </c>
+      <c r="N110" s="3" t="inlineStr">
+        <is>
+          <t>1 de 108</t>
+        </is>
+      </c>
+      <c r="O110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
+        </is>
+      </c>
+      <c r="P110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
+        </is>
+      </c>
+      <c r="Q110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
+        </is>
+      </c>
+      <c r="R110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-06-25 09:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -2079,7 +2079,7 @@
         <v>0</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0</v>
+        <v>57.93</v>
       </c>
       <c r="H27" s="2" t="n">
         <v>0</v>
@@ -7058,7 +7058,7 @@
       </c>
       <c r="G110" s="3" t="inlineStr">
         <is>
-          <t>1 de 108</t>
+          <t>2 de 108</t>
         </is>
       </c>
       <c r="H110" s="3" t="inlineStr">
@@ -8224,7 +8224,7 @@
         <v>314.51</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>12.9</v>
+        <v>70.83</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>0</v>
@@ -11454,7 +11454,7 @@
         <v>6624.3</v>
       </c>
       <c r="F160" s="4" t="n">
-        <v>5114.37</v>
+        <v>5172.3</v>
       </c>
       <c r="G160" s="4" t="n">
         <v>0</v>
@@ -11478,7 +11478,7 @@
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -11529,13 +11529,13 @@
         <v>133.5</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>59.25</v>
+        <v>117.18</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>74.25</v>
+        <v>16.31999999999999</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.4438202247191011</v>
+        <v>0.8777528089887641</v>
       </c>
     </row>
     <row r="3">
@@ -11596,13 +11596,13 @@
         <v>18333.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>26212.42</v>
+        <v>26270.35</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-7878.919999999998</v>
+        <v>-7936.849999999999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1.42975536586031</v>
+        <v>1.43291515531677</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-29 11:30:19
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R109"/>
+  <dimension ref="A1:R110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5697,7 +5697,7 @@
         <v>0</v>
       </c>
       <c r="M87" s="2" t="n">
-        <v>0</v>
+        <v>2033.79</v>
       </c>
       <c r="N87" s="2" t="n">
         <v>0</v>
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5853,13 +5853,13 @@
         <v>0</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>83.3</v>
+        <v>0</v>
       </c>
       <c r="F90" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>59.25</v>
+        <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
         <v>0</v>
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5913,13 +5913,13 @@
         <v>0</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>0</v>
+        <v>83.3</v>
       </c>
       <c r="F91" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>0</v>
+        <v>59.25</v>
       </c>
       <c r="H91" s="2" t="n">
         <v>0</v>
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6168,7 +6168,7 @@
         <v>0</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>28.32</v>
+        <v>0</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6228,7 +6228,7 @@
         <v>0</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0</v>
+        <v>28.32</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -6923,137 +6923,197 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
+          <t>ZAZACORP S.A.</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R108" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
           <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
-      <c r="C108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R108" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="C109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="D109" s="3" t="inlineStr">
-        <is>
-          <t>1 de 107</t>
-        </is>
-      </c>
-      <c r="E109" s="3" t="inlineStr">
-        <is>
-          <t>2 de 107</t>
-        </is>
-      </c>
-      <c r="F109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="G109" s="3" t="inlineStr">
-        <is>
-          <t>2 de 107</t>
-        </is>
-      </c>
-      <c r="H109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="I109" s="3" t="inlineStr">
-        <is>
-          <t>1 de 107</t>
-        </is>
-      </c>
-      <c r="J109" s="3" t="inlineStr">
-        <is>
-          <t>3 de 107</t>
-        </is>
-      </c>
-      <c r="K109" s="3" t="inlineStr">
-        <is>
-          <t>2 de 107</t>
-        </is>
-      </c>
-      <c r="L109" s="3" t="inlineStr">
-        <is>
-          <t>3 de 107</t>
-        </is>
-      </c>
-      <c r="M109" s="3" t="inlineStr">
-        <is>
-          <t>3 de 107</t>
-        </is>
-      </c>
-      <c r="N109" s="3" t="inlineStr">
-        <is>
-          <t>1 de 107</t>
-        </is>
-      </c>
-      <c r="O109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="P109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="Q109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="R109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
+      <c r="C109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R109" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>1 de 108</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>2 de 108</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>2 de 108</t>
+        </is>
+      </c>
+      <c r="H110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
+        </is>
+      </c>
+      <c r="I110" s="3" t="inlineStr">
+        <is>
+          <t>1 de 108</t>
+        </is>
+      </c>
+      <c r="J110" s="3" t="inlineStr">
+        <is>
+          <t>3 de 108</t>
+        </is>
+      </c>
+      <c r="K110" s="3" t="inlineStr">
+        <is>
+          <t>2 de 108</t>
+        </is>
+      </c>
+      <c r="L110" s="3" t="inlineStr">
+        <is>
+          <t>3 de 108</t>
+        </is>
+      </c>
+      <c r="M110" s="3" t="inlineStr">
+        <is>
+          <t>4 de 108</t>
+        </is>
+      </c>
+      <c r="N110" s="3" t="inlineStr">
+        <is>
+          <t>1 de 108</t>
+        </is>
+      </c>
+      <c r="O110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
+        </is>
+      </c>
+      <c r="P110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
+        </is>
+      </c>
+      <c r="Q110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
+        </is>
+      </c>
+      <c r="R110" s="3" t="inlineStr">
+        <is>
+          <t>0 de 108</t>
         </is>
       </c>
     </row>
@@ -7068,7 +7128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G130"/>
+  <dimension ref="A1:G131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10014,7 +10074,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -10027,7 +10087,7 @@
         <v>0</v>
       </c>
       <c r="F109" s="2" t="n">
-        <v>0</v>
+        <v>2033.79</v>
       </c>
       <c r="G109" s="2" t="n">
         <v>0</v>
@@ -10041,7 +10101,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -10068,14 +10128,14 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D111" s="2" t="n">
-        <v>107.46</v>
+        <v>0</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>0</v>
@@ -10095,14 +10155,14 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D112" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>0</v>
@@ -10122,7 +10182,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
@@ -10149,7 +10209,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
@@ -10176,7 +10236,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
@@ -10186,7 +10246,7 @@
         <v>0</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>186.47</v>
+        <v>0</v>
       </c>
       <c r="F115" s="2" t="n">
         <v>0</v>
@@ -10203,7 +10263,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
@@ -10213,7 +10273,7 @@
         <v>0</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>0</v>
+        <v>186.47</v>
       </c>
       <c r="F116" s="2" t="n">
         <v>0</v>
@@ -10230,17 +10290,17 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D117" s="2" t="n">
-        <v>50.16</v>
+        <v>0</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>25.08</v>
+        <v>0</v>
       </c>
       <c r="F117" s="2" t="n">
         <v>0</v>
@@ -10257,17 +10317,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D118" s="2" t="n">
-        <v>0</v>
+        <v>50.16</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>0</v>
+        <v>25.08</v>
       </c>
       <c r="F118" s="2" t="n">
         <v>0</v>
@@ -10284,17 +10344,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D119" s="2" t="n">
-        <v>176.6</v>
+        <v>0</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>217.99</v>
+        <v>0</v>
       </c>
       <c r="F119" s="2" t="n">
         <v>0</v>
@@ -10311,17 +10371,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D120" s="2" t="n">
-        <v>0</v>
+        <v>176.6</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>0</v>
+        <v>217.99</v>
       </c>
       <c r="F120" s="2" t="n">
         <v>0</v>
@@ -10338,7 +10398,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
@@ -10365,7 +10425,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
@@ -10392,7 +10452,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
@@ -10419,7 +10479,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
@@ -10446,14 +10506,14 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D125" s="2" t="n">
-        <v>3.94</v>
+        <v>0</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>0</v>
@@ -10473,14 +10533,14 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D126" s="2" t="n">
-        <v>0</v>
+        <v>3.94</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>0</v>
@@ -10500,7 +10560,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
@@ -10527,7 +10587,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
@@ -10554,39 +10614,66 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G129" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
           <t>ZUÑIGA BUSTAMANTE ENRIQUE HAMLET</t>
         </is>
       </c>
-      <c r="C129" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D129" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E129" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F129" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G129" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="C130" s="4" t="n">
+      <c r="C130" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D130" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E130" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F130" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G130" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="C131" s="4" t="n">
         <v>13664.47</v>
       </c>
-      <c r="D130" s="4" t="n">
+      <c r="D131" s="4" t="n">
         <v>4775.7</v>
       </c>
-      <c r="E130" s="4" t="n">
+      <c r="E131" s="4" t="n">
         <v>6400.73</v>
       </c>
-      <c r="F130" s="4" t="n">
-        <v>3804.58</v>
-      </c>
-      <c r="G130" s="4" t="n">
+      <c r="F131" s="4" t="n">
+        <v>5838.37</v>
+      </c>
+      <c r="G131" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10707,13 +10794,13 @@
         <v>18200</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>3265.98</v>
+        <v>5299.77</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>14934.02</v>
+        <v>12900.23</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.1794494505494506</v>
+        <v>0.2911961538461539</v>
       </c>
     </row>
     <row r="5">
@@ -10726,13 +10813,13 @@
         <v>18333.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>26270.35</v>
+        <v>28304.14</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-7936.849999999999</v>
+        <v>-9970.639999999999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1.43291515531677</v>
+        <v>1.543848146835029</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-30 14:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>47.92</v>
+        <v>84.16</v>
       </c>
       <c r="N25" s="2" t="n">
         <v>77.98999999999999</v>
@@ -10881,13 +10881,13 @@
         <v>18200</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>5299.77</v>
+        <v>5336.01</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>12900.23</v>
+        <v>12863.99</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.2911961538461539</v>
+        <v>0.2931873626373627</v>
       </c>
     </row>
     <row r="5">
@@ -10900,13 +10900,13 @@
         <v>18333.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>28304.14</v>
+        <v>28340.38</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-9970.639999999999</v>
+        <v>-10006.88</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1.543848146835029</v>
+        <v>1.545824856137671</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-01 16:30:17
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R108"/>
+  <dimension ref="A1:R109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3213,13 +3213,13 @@
         <v>0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>0</v>
+        <v>88.34</v>
       </c>
       <c r="F46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0</v>
+        <v>65.12</v>
       </c>
       <c r="H46" s="2" t="n">
         <v>0</v>
@@ -3234,10 +3234,10 @@
         <v>0</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>0</v>
+        <v>968.42</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>0</v>
+        <v>1674.61</v>
       </c>
       <c r="N46" s="2" t="n">
         <v>0</v>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6863,137 +6863,197 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
+          <t>ZAZACORP S.A.</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R107" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
           <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
-      <c r="C107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R107" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="C108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="D108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="E108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="F108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="G108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="H108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="I108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="J108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="K108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="L108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="M108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="N108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="O108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="P108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="Q108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="R108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
+      <c r="C108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R108" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>1 de 107</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>1 de 107</t>
+        </is>
+      </c>
+      <c r="H109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="J109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="K109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="L109" s="3" t="inlineStr">
+        <is>
+          <t>1 de 107</t>
+        </is>
+      </c>
+      <c r="M109" s="3" t="inlineStr">
+        <is>
+          <t>1 de 107</t>
+        </is>
+      </c>
+      <c r="N109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="O109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="P109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="Q109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="R109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
         </is>
       </c>
     </row>
@@ -7008,7 +7068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G132"/>
+  <dimension ref="A1:G133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7016,7 +7076,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -8496,7 +8556,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -8509,7 +8569,7 @@
         <v>0</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>0</v>
+        <v>2796.49</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>0</v>
@@ -8523,7 +8583,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -8550,11 +8610,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>833.03</v>
+        <v>0</v>
       </c>
       <c r="D57" s="2" t="n">
         <v>0</v>
@@ -8577,11 +8637,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>0</v>
+        <v>833.03</v>
       </c>
       <c r="D58" s="2" t="n">
         <v>0</v>
@@ -8604,7 +8664,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>HILL PEÑA JONATHAN STUART</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -8631,14 +8691,14 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>HILL PEÑA JONATHAN STUART</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>88.3</v>
+        <v>0</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>116.77</v>
+        <v>0</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>0</v>
@@ -8658,14 +8718,14 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
-        <v>0</v>
+        <v>88.3</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>0</v>
+        <v>116.77</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>0</v>
@@ -8685,7 +8745,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -8712,7 +8772,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -8722,7 +8782,7 @@
         <v>0</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>28.77</v>
+        <v>0</v>
       </c>
       <c r="F63" s="2" t="n">
         <v>0</v>
@@ -8739,17 +8799,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>453.32</v>
+        <v>0</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>778.9</v>
+        <v>0</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>138.47</v>
+        <v>28.77</v>
       </c>
       <c r="F64" s="2" t="n">
         <v>0</v>
@@ -8766,17 +8826,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>0</v>
+        <v>453.32</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0</v>
+        <v>778.9</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0</v>
+        <v>138.47</v>
       </c>
       <c r="F65" s="2" t="n">
         <v>0</v>
@@ -8793,7 +8853,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>JIMENEZ MORALES JACQUELINE ALEXANDRA</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -8820,7 +8880,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ MORALES JACQUELINE ALEXANDRA</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -8847,7 +8907,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>LAM WONG NELLY ANGELA</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -8874,7 +8934,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>LECANSA S.A.</t>
+          <t>LAM WONG NELLY ANGELA</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -8901,7 +8961,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>LEM S.A.</t>
+          <t>LECANSA S.A.</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -8928,7 +8988,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LEM S.A.</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -8955,7 +9015,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -8982,7 +9042,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -9009,7 +9069,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -9036,7 +9096,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>La Casa Del Coleccionista S.A.S</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -9063,7 +9123,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>La Casa Del Coleccionista S.A.S</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -9090,7 +9150,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -9117,7 +9177,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -9127,7 +9187,7 @@
         <v>0</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>39.4</v>
+        <v>0</v>
       </c>
       <c r="F78" s="2" t="n">
         <v>0</v>
@@ -9144,7 +9204,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -9154,7 +9214,7 @@
         <v>0</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>0</v>
+        <v>39.4</v>
       </c>
       <c r="F79" s="2" t="n">
         <v>0</v>
@@ -9171,7 +9231,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -9198,7 +9258,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>MIELES SAN MARTIN JOHNNY JOEL</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -9225,7 +9285,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MIELES SAN MARTIN JOHNNY JOEL</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -9252,7 +9312,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -9279,7 +9339,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -9306,7 +9366,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -9333,7 +9393,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -9360,7 +9420,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>MOSCOSO BLANCO JULIO ENRIQUE</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -9387,7 +9447,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>MOSCOSO MORALES ANNIE LISBETH</t>
+          <t>MOSCOSO BLANCO JULIO ENRIQUE</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -9414,14 +9474,14 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOSCOSO MORALES ANNIE LISBETH</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="D89" s="2" t="n">
-        <v>347.34</v>
+        <v>0</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>0</v>
@@ -9441,14 +9501,14 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="D90" s="2" t="n">
-        <v>0</v>
+        <v>347.34</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>0</v>
@@ -9468,7 +9528,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -9495,7 +9555,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -9522,7 +9582,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>OLUNANEK S.A.</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -9549,17 +9609,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>OLUNANEK S.A.</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
-        <v>346.79</v>
+        <v>0</v>
       </c>
       <c r="D94" s="2" t="n">
-        <v>192.19</v>
+        <v>0</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>99.25</v>
+        <v>0</v>
       </c>
       <c r="F94" s="2" t="n">
         <v>0</v>
@@ -9576,17 +9636,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
-        <v>102.69</v>
+        <v>346.79</v>
       </c>
       <c r="D95" s="2" t="n">
-        <v>0</v>
+        <v>192.19</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>0</v>
+        <v>99.25</v>
       </c>
       <c r="F95" s="2" t="n">
         <v>0</v>
@@ -9603,11 +9663,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
-        <v>0</v>
+        <v>102.69</v>
       </c>
       <c r="D96" s="2" t="n">
         <v>0</v>
@@ -9630,7 +9690,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -9657,7 +9717,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -9684,7 +9744,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -9694,7 +9754,7 @@
         <v>0</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>2043.13</v>
+        <v>0</v>
       </c>
       <c r="F99" s="2" t="n">
         <v>0</v>
@@ -9711,7 +9771,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>QUIROLA GOMEZ DIEGO FABRICIO</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -9721,7 +9781,7 @@
         <v>0</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>0</v>
+        <v>2043.13</v>
       </c>
       <c r="F100" s="2" t="n">
         <v>0</v>
@@ -9738,7 +9798,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIROLA GOMEZ DIEGO FABRICIO</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -9765,7 +9825,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>RAMOS UGUÑA ERICK FABRICIO</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -9792,7 +9852,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>REALMIND S.A.</t>
+          <t>RAMOS UGUÑA ERICK FABRICIO</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -9819,17 +9879,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>REALMIND S.A.</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
-        <v>1049.35</v>
+        <v>0</v>
       </c>
       <c r="D104" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>2248.94</v>
+        <v>0</v>
       </c>
       <c r="F104" s="2" t="n">
         <v>0</v>
@@ -9846,17 +9906,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
-        <v>0</v>
+        <v>1049.35</v>
       </c>
       <c r="D105" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>0</v>
+        <v>2248.94</v>
       </c>
       <c r="F105" s="2" t="n">
         <v>0</v>
@@ -9873,7 +9933,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -9900,7 +9960,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -9927,11 +9987,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="D108" s="2" t="n">
         <v>0</v>
@@ -9954,11 +10014,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>SILVA BLUM CARLOS ALFREDO</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="D109" s="2" t="n">
         <v>0</v>
@@ -9981,7 +10041,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SILVA BLUM CARLOS ALFREDO</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -9991,7 +10051,7 @@
         <v>0</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>2033.79</v>
+        <v>0</v>
       </c>
       <c r="F110" s="2" t="n">
         <v>0</v>
@@ -10008,7 +10068,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
@@ -10018,7 +10078,7 @@
         <v>0</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>0</v>
+        <v>2033.79</v>
       </c>
       <c r="F111" s="2" t="n">
         <v>0</v>
@@ -10035,7 +10095,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
@@ -10062,11 +10122,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
-        <v>107.46</v>
+        <v>0</v>
       </c>
       <c r="D113" s="2" t="n">
         <v>0</v>
@@ -10089,11 +10149,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="D114" s="2" t="n">
         <v>0</v>
@@ -10116,7 +10176,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
@@ -10143,7 +10203,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
@@ -10170,14 +10230,14 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D117" s="2" t="n">
-        <v>186.47</v>
+        <v>0</v>
       </c>
       <c r="E117" s="2" t="n">
         <v>0</v>
@@ -10197,14 +10257,14 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D118" s="2" t="n">
-        <v>0</v>
+        <v>186.47</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>0</v>
@@ -10224,14 +10284,14 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
-        <v>50.16</v>
+        <v>0</v>
       </c>
       <c r="D119" s="2" t="n">
-        <v>25.08</v>
+        <v>0</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>0</v>
@@ -10251,14 +10311,14 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
-        <v>0</v>
+        <v>50.16</v>
       </c>
       <c r="D120" s="2" t="n">
-        <v>0</v>
+        <v>25.08</v>
       </c>
       <c r="E120" s="2" t="n">
         <v>0</v>
@@ -10278,14 +10338,14 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
-        <v>176.6</v>
+        <v>0</v>
       </c>
       <c r="D121" s="2" t="n">
-        <v>217.99</v>
+        <v>0</v>
       </c>
       <c r="E121" s="2" t="n">
         <v>0</v>
@@ -10305,14 +10365,14 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
-        <v>0</v>
+        <v>176.6</v>
       </c>
       <c r="D122" s="2" t="n">
-        <v>0</v>
+        <v>217.99</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>0</v>
@@ -10332,7 +10392,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
@@ -10359,7 +10419,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
@@ -10386,7 +10446,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
@@ -10413,7 +10473,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
@@ -10440,11 +10500,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
-        <v>3.94</v>
+        <v>0</v>
       </c>
       <c r="D127" s="2" t="n">
         <v>0</v>
@@ -10467,11 +10527,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
-        <v>0</v>
+        <v>3.94</v>
       </c>
       <c r="D128" s="2" t="n">
         <v>0</v>
@@ -10494,7 +10554,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
@@ -10521,7 +10581,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
@@ -10548,39 +10608,66 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D131" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E131" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F131" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G131" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
           <t>ZUÑIGA BUSTAMANTE ENRIQUE HAMLET</t>
         </is>
       </c>
-      <c r="C131" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D131" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E131" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F131" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G131" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="C132" s="4" t="n">
+      <c r="C132" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D132" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E132" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F132" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G132" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="C133" s="4" t="n">
         <v>4799.88</v>
       </c>
-      <c r="D132" s="4" t="n">
+      <c r="D133" s="4" t="n">
         <v>6400.73</v>
       </c>
-      <c r="E132" s="4" t="n">
+      <c r="E133" s="4" t="n">
         <v>7722.25</v>
       </c>
-      <c r="F132" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G132" s="4" t="n">
+      <c r="F133" s="4" t="n">
+        <v>2796.49</v>
+      </c>
+      <c r="G133" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-07-02 08:30:16
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R109"/>
+  <dimension ref="A1:R108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -983,7 +983,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ANGULO PARRALES CARMEN</t>
+          <t>ARCE CANDO DENISSE YAJAIRA</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ARCE CANDO DENISSE YAJAIRA</t>
+          <t>ARMIJO AGUILAR ROBERT LENIN</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ARMIJO AGUILAR ROBERT LENIN</t>
+          <t>ARQUITECKSA S.A.</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ARQUITECKSA S.A.</t>
+          <t>BRAVO MANZABA MARIA CECILIA</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BRAVO MANZABA MARIA CECILIA</t>
+          <t>BRIONES GOMEZ ASLEY YAMILEXY</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BRIONES GOMEZ ASLEY YAMILEXY</t>
+          <t>BRITO MORALES MARIA SOLEDAD</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BRITO MORALES MARIA SOLEDAD</t>
+          <t>BURGOS OLVERA VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BURGOS OLVERA VICENTE JAVIER</t>
+          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
+          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
+          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
+          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
+          <t>CARRANZA AVILEZ WILSON</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CARRANZA AVILEZ WILSON</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CASTRO ALCIVAR EDA MARIA</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CASTRO ALCIVAR EDA MARIA</t>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
+          <t>CATAECSA S.A.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CATAECSA S.A.</t>
+          <t>CERAMICASAECUADOR S.A.</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CERAMICASAECUADOR S.A.</t>
+          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
+          <t>CHICA ALBAN GILMERTH HOMERO</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CHICA ALBAN GILMERTH HOMERO</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
+          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
+          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
+          <t>CONSTRUMERCADO S.A.</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Carlos Meza Peña</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>ECUARECYCLING S.A.</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ECUARECYCLING S.A.</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>FIENCO VILLACIS NARCISA ROCIO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>FIENCO VILLACIS NARCISA ROCIO</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3153,13 +3153,13 @@
         <v>0</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0</v>
+        <v>88.34</v>
       </c>
       <c r="F45" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0</v>
+        <v>65.12</v>
       </c>
       <c r="H45" s="2" t="n">
         <v>0</v>
@@ -3174,10 +3174,10 @@
         <v>0</v>
       </c>
       <c r="L45" s="2" t="n">
-        <v>0</v>
+        <v>968.42</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>0</v>
+        <v>1674.61</v>
       </c>
       <c r="N45" s="2" t="n">
         <v>0</v>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3213,13 +3213,13 @@
         <v>0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>88.34</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>65.12</v>
+        <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
         <v>0</v>
@@ -3234,10 +3234,10 @@
         <v>0</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>968.42</v>
+        <v>0</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>1674.61</v>
+        <v>0</v>
       </c>
       <c r="N46" s="2" t="n">
         <v>0</v>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -6916,144 +6916,84 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q108" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R108" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="C109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="D109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="E109" s="3" t="inlineStr">
-        <is>
-          <t>1 de 107</t>
-        </is>
-      </c>
-      <c r="F109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="G109" s="3" t="inlineStr">
-        <is>
-          <t>1 de 107</t>
-        </is>
-      </c>
-      <c r="H109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="I109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="J109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="K109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="L109" s="3" t="inlineStr">
-        <is>
-          <t>1 de 107</t>
-        </is>
-      </c>
-      <c r="M109" s="3" t="inlineStr">
-        <is>
-          <t>1 de 107</t>
-        </is>
-      </c>
-      <c r="N109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="O109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="P109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="Q109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
-        </is>
-      </c>
-      <c r="R109" s="3" t="inlineStr">
-        <is>
-          <t>0 de 107</t>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>1 de 106</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="G108" s="3" t="inlineStr">
+        <is>
+          <t>1 de 106</t>
+        </is>
+      </c>
+      <c r="H108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="I108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="J108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="K108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="L108" s="3" t="inlineStr">
+        <is>
+          <t>1 de 106</t>
+        </is>
+      </c>
+      <c r="M108" s="3" t="inlineStr">
+        <is>
+          <t>1 de 106</t>
+        </is>
+      </c>
+      <c r="N108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="O108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="P108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="Q108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="R108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-07-02 09:30:22
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0</v>
+        <v>23.6</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1917,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>-36.24</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -6968,7 +6968,7 @@
       </c>
       <c r="M108" s="3" t="inlineStr">
         <is>
-          <t>1 de 106</t>
+          <t>2 de 106</t>
         </is>
       </c>
       <c r="N108" s="3" t="inlineStr">
@@ -7888,7 +7888,7 @@
         <v>0</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0</v>
+        <v>23.6</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>0</v>
@@ -10605,7 +10605,7 @@
         <v>7722.25</v>
       </c>
       <c r="F133" s="4" t="n">
-        <v>2796.49</v>
+        <v>2820.09</v>
       </c>
       <c r="G133" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-03 12:30:15
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -2490,7 +2490,7 @@
         <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0</v>
+        <v>568.71</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
@@ -7103,7 +7103,7 @@
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>0 de 109</t>
+          <t>1 de 109</t>
         </is>
       </c>
       <c r="E111" s="3" t="inlineStr">
@@ -8392,7 +8392,7 @@
         <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0</v>
+        <v>568.71</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>0</v>
@@ -10893,7 +10893,7 @@
         <v>8618.370000000001</v>
       </c>
       <c r="F137" s="4" t="n">
-        <v>2832.73</v>
+        <v>3401.44</v>
       </c>
       <c r="G137" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-03 17:30:16
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R111"/>
+  <dimension ref="A1:R112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -983,7 +983,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ARCE CANDO DENISSE YAJAIRA</t>
+          <t>APOLO GALLARDO RICARDO ISRAEL</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -1017,7 +1017,7 @@
         <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>248.52</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ARMIJO AGUILAR ROBERT LENIN</t>
+          <t>ARCE CANDO DENISSE YAJAIRA</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ARQUITECKSA S.A.</t>
+          <t>ARMIJO AGUILAR ROBERT LENIN</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BRAVO MANZABA MARIA CECILIA</t>
+          <t>ARQUITECKSA S.A.</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BRIONES GOMEZ ASLEY YAMILEXY</t>
+          <t>BRAVO MANZABA MARIA CECILIA</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BRITO MORALES MARIA SOLEDAD</t>
+          <t>BRIONES GOMEZ ASLEY YAMILEXY</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BURGOS OLVERA VICENTE JAVIER</t>
+          <t>BRITO MORALES MARIA SOLEDAD</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
+          <t>BURGOS OLVERA VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
+          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
+          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
+          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CARRANZA AVILEZ WILSON</t>
+          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CARRANZA AVILEZ WILSON</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CASTRO ALCIVAR EDA MARIA</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>36.24</v>
+        <v>0</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
+          <t>CASTRO ALCIVAR EDA MARIA</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1917,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>-36.24</v>
+        <v>36.24</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CATAECSA S.A.</t>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>0</v>
+        <v>-36.24</v>
       </c>
       <c r="N25" s="2" t="n">
         <v>0</v>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CERAMICASAECUADOR S.A.</t>
+          <t>CATAECSA S.A.</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
+          <t>CERAMICASAECUADOR S.A.</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CHICA ALBAN GILMERTH HOMERO</t>
+          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>CHICA ALBAN GILMERTH HOMERO</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
+          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
+          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,14 +2483,14 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>COQUE TONATO RICHARD PAUL</t>
+          <t>CONSTRUMERCADO S.A.</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>568.71</v>
+        <v>0</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
@@ -2543,14 +2543,14 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Carlos Meza Peña</t>
+          <t>COQUE TONATO RICHARD PAUL</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0</v>
+        <v>568.71</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>0</v>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ECUARECYCLING S.A.</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EDESA SA</t>
+          <t>ECUARECYCLING S.A.</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>EDESA SA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>FIENCO VILLACIS NARCISA ROCIO</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>FIENCO VILLACIS NARCISA ROCIO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3273,13 +3273,13 @@
         <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>88.34</v>
+        <v>0</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>65.12</v>
+        <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
         <v>0</v>
@@ -3294,10 +3294,10 @@
         <v>0</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>968.42</v>
+        <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>1674.61</v>
+        <v>0</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3333,13 +3333,13 @@
         <v>0</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0</v>
+        <v>88.34</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0</v>
+        <v>65.12</v>
       </c>
       <c r="H48" s="2" t="n">
         <v>0</v>
@@ -3354,10 +3354,10 @@
         <v>0</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>0</v>
+        <v>968.42</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0</v>
+        <v>1674.61</v>
       </c>
       <c r="N48" s="2" t="n">
         <v>0</v>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -6923,7 +6923,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -7043,137 +7043,197 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
+          <t>ZAZACORP S.A.</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R110" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
           <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
-      <c r="C110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R110" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="C111" s="3" t="inlineStr">
-        <is>
-          <t>0 de 109</t>
-        </is>
-      </c>
-      <c r="D111" s="3" t="inlineStr">
-        <is>
-          <t>1 de 109</t>
-        </is>
-      </c>
-      <c r="E111" s="3" t="inlineStr">
-        <is>
-          <t>1 de 109</t>
-        </is>
-      </c>
-      <c r="F111" s="3" t="inlineStr">
-        <is>
-          <t>0 de 109</t>
-        </is>
-      </c>
-      <c r="G111" s="3" t="inlineStr">
-        <is>
-          <t>1 de 109</t>
-        </is>
-      </c>
-      <c r="H111" s="3" t="inlineStr">
-        <is>
-          <t>0 de 109</t>
-        </is>
-      </c>
-      <c r="I111" s="3" t="inlineStr">
-        <is>
-          <t>0 de 109</t>
-        </is>
-      </c>
-      <c r="J111" s="3" t="inlineStr">
-        <is>
-          <t>0 de 109</t>
-        </is>
-      </c>
-      <c r="K111" s="3" t="inlineStr">
-        <is>
-          <t>0 de 109</t>
-        </is>
-      </c>
-      <c r="L111" s="3" t="inlineStr">
-        <is>
-          <t>1 de 109</t>
-        </is>
-      </c>
-      <c r="M111" s="3" t="inlineStr">
-        <is>
-          <t>2 de 109</t>
-        </is>
-      </c>
-      <c r="N111" s="3" t="inlineStr">
-        <is>
-          <t>0 de 109</t>
-        </is>
-      </c>
-      <c r="O111" s="3" t="inlineStr">
-        <is>
-          <t>0 de 109</t>
-        </is>
-      </c>
-      <c r="P111" s="3" t="inlineStr">
-        <is>
-          <t>0 de 109</t>
-        </is>
-      </c>
-      <c r="Q111" s="3" t="inlineStr">
-        <is>
-          <t>0 de 109</t>
-        </is>
-      </c>
-      <c r="R111" s="3" t="inlineStr">
-        <is>
-          <t>0 de 109</t>
+      <c r="C111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R111" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>1 de 110</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>1 de 110</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>1 de 110</t>
+        </is>
+      </c>
+      <c r="H112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="I112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="J112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="K112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="L112" s="3" t="inlineStr">
+        <is>
+          <t>1 de 110</t>
+        </is>
+      </c>
+      <c r="M112" s="3" t="inlineStr">
+        <is>
+          <t>3 de 110</t>
+        </is>
+      </c>
+      <c r="N112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="O112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="P112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="Q112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
+        </is>
+      </c>
+      <c r="R112" s="3" t="inlineStr">
+        <is>
+          <t>0 de 110</t>
         </is>
       </c>
     </row>
@@ -7188,7 +7248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G137"/>
+  <dimension ref="A1:G138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7569,7 +7629,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ARCE CANDO DENISSE YAJAIRA</t>
+          <t>APOLO GALLARDO RICARDO ISRAEL</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -7582,7 +7642,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>248.52</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>0</v>
@@ -7596,7 +7656,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ARMIJO AGUILAR ROBERT LENIN</t>
+          <t>ARCE CANDO DENISSE YAJAIRA</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -7623,7 +7683,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ARQUITECKSA S.A.</t>
+          <t>ARMIJO AGUILAR ROBERT LENIN</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -7650,7 +7710,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ASTUDILLO SARMIENTO PAUL BISMARK</t>
+          <t>ARQUITECKSA S.A.</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -7677,7 +7737,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AVILA TORRES RAFAEL ALEJANDRO</t>
+          <t>ASTUDILLO SARMIENTO PAUL BISMARK</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -7704,7 +7764,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AYORA GUEVARA MARIA DANIELA</t>
+          <t>AVILA TORRES RAFAEL ALEJANDRO</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -7731,7 +7791,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BRAVO MANZABA MARIA CECILIA</t>
+          <t>AYORA GUEVARA MARIA DANIELA</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -7758,7 +7818,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BRIONES GOMEZ ASLEY YAMILEXY</t>
+          <t>BRAVO MANZABA MARIA CECILIA</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -7785,7 +7845,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BRITO MORALES MARIA SOLEDAD</t>
+          <t>BRIONES GOMEZ ASLEY YAMILEXY</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -7812,7 +7872,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BURGOS OLVERA VICENTE JAVIER</t>
+          <t>BRITO MORALES MARIA SOLEDAD</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -7839,7 +7899,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
+          <t>BURGOS OLVERA VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -7866,17 +7926,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
+          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>861.02</v>
+        <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>-861.02</v>
+        <v>0</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>28.76</v>
+        <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>0</v>
@@ -7893,17 +7953,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
+          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0</v>
+        <v>861.02</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0</v>
+        <v>-861.02</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0</v>
+        <v>28.76</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>0</v>
@@ -7920,7 +7980,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CARRANZA AVILEZ WILSON</t>
+          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -7930,7 +7990,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>107.46</v>
+        <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>0</v>
@@ -7947,7 +8007,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CARRANZA JARA LEONARDO GABRIEL</t>
+          <t>CARRANZA AVILEZ WILSON</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -7957,7 +8017,7 @@
         <v>0</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>0</v>
@@ -7974,7 +8034,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CARRANZA JARA LEONARDO GABRIEL</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -8001,7 +8061,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CASCO PENA HUGO VLADIMIR</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -8028,7 +8088,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CASCO PENA HUGO VLADIMIR</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -8055,7 +8115,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CASTRO ALCIVAR EDA MARIA</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -8068,7 +8128,7 @@
         <v>0</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>36.24</v>
+        <v>0</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>0</v>
@@ -8082,7 +8142,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CASTRO CEDILLO BLANCA KARINA</t>
+          <t>CASTRO ALCIVAR EDA MARIA</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -8095,7 +8155,7 @@
         <v>0</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0</v>
+        <v>36.24</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>0</v>
@@ -8109,14 +8169,14 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CERAMICASAECUADOR S.A.</t>
+          <t>CASTRO CEDILLO BLANCA KARINA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>-1554.57</v>
+        <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>1561.97</v>
+        <v>0</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
@@ -8136,17 +8196,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
+          <t>CERAMICASAECUADOR S.A.</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>1686.69</v>
+        <v>-1554.57</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>314.51</v>
+        <v>1561.97</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>70.83</v>
+        <v>0</v>
       </c>
       <c r="F35" s="2" t="n">
         <v>0</v>
@@ -8163,17 +8223,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CHICA ALBAN GILMERTH HOMERO</t>
+          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0</v>
+        <v>1686.69</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0</v>
+        <v>314.51</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0</v>
+        <v>70.83</v>
       </c>
       <c r="F36" s="2" t="n">
         <v>0</v>
@@ -8190,7 +8250,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>CHICA ALBAN GILMERTH HOMERO</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -8217,7 +8277,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -8244,7 +8304,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
+          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -8271,7 +8331,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTE DE CARGA PESADA ALAY EXPRESS S.A.</t>
+          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -8298,7 +8358,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
+          <t>COMPAÑIA DE TRANSPORTE DE CARGA PESADA ALAY EXPRESS S.A.</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -8325,17 +8385,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>24.18</v>
+        <v>0</v>
       </c>
       <c r="D42" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>320.79</v>
+        <v>0</v>
       </c>
       <c r="F42" s="2" t="n">
         <v>0</v>
@@ -8352,17 +8412,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CONTRERAS JIMMY</t>
+          <t>CONSTRUMERCADO S.A.</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>0</v>
+        <v>24.18</v>
       </c>
       <c r="D43" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0</v>
+        <v>320.79</v>
       </c>
       <c r="F43" s="2" t="n">
         <v>0</v>
@@ -8379,7 +8439,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>COQUE TONATO RICHARD PAUL</t>
+          <t>CONTRERAS JIMMY</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -8392,7 +8452,7 @@
         <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>568.71</v>
+        <v>0</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>0</v>
@@ -8406,7 +8466,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>COQUE TONATO RICHARD PAUL</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -8419,7 +8479,7 @@
         <v>0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>568.71</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>0</v>
@@ -8433,7 +8493,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -8460,17 +8520,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>333</v>
+        <v>0</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>3030.4</v>
+        <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>445.73</v>
+        <v>0</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>0</v>
@@ -8487,17 +8547,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EDESA SA</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>0</v>
+        <v>333</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0</v>
+        <v>3030.4</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>503.56</v>
+        <v>445.73</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>0</v>
@@ -8514,7 +8574,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>EDESA SA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -8524,7 +8584,7 @@
         <v>0</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0</v>
+        <v>503.56</v>
       </c>
       <c r="F49" s="2" t="n">
         <v>0</v>
@@ -8541,7 +8601,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -8568,7 +8628,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -8595,7 +8655,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -8622,7 +8682,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -8649,7 +8709,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>FERNANDEZ VILLARREAL MARIELA JACQUELINE</t>
+          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -8676,7 +8736,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>FIENCO VILLACIS NARCISA ROCIO</t>
+          <t>FERNANDEZ VILLARREAL MARIELA JACQUELINE</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -8686,7 +8746,7 @@
         <v>0</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>92.81999999999999</v>
+        <v>0</v>
       </c>
       <c r="F55" s="2" t="n">
         <v>0</v>
@@ -8703,17 +8763,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>FIENCO VILLACIS NARCISA ROCIO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>293.94</v>
+        <v>0</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0</v>
+        <v>92.81999999999999</v>
       </c>
       <c r="F56" s="2" t="n">
         <v>0</v>
@@ -8730,20 +8790,20 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>0</v>
+        <v>293.94</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>2796.49</v>
+        <v>0</v>
       </c>
       <c r="G57" s="2" t="n">
         <v>0</v>
@@ -8757,7 +8817,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -8770,7 +8830,7 @@
         <v>0</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>0</v>
+        <v>2796.49</v>
       </c>
       <c r="G58" s="2" t="n">
         <v>0</v>
@@ -8784,7 +8844,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -8811,11 +8871,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>833.03</v>
+        <v>0</v>
       </c>
       <c r="D60" s="2" t="n">
         <v>0</v>
@@ -8838,11 +8898,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
-        <v>0</v>
+        <v>833.03</v>
       </c>
       <c r="D61" s="2" t="n">
         <v>0</v>
@@ -8865,7 +8925,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>HILL PEÑA JONATHAN STUART</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -8892,14 +8952,14 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>HILL PEÑA JONATHAN STUART</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>88.3</v>
+        <v>0</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>116.77</v>
+        <v>0</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>0</v>
@@ -8919,14 +8979,14 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>0</v>
+        <v>88.3</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>0</v>
+        <v>116.77</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>0</v>
@@ -8946,7 +9006,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -8973,7 +9033,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -8983,7 +9043,7 @@
         <v>0</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>28.77</v>
+        <v>0</v>
       </c>
       <c r="F66" s="2" t="n">
         <v>0</v>
@@ -9000,17 +9060,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
-        <v>453.32</v>
+        <v>0</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>778.9</v>
+        <v>0</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>138.47</v>
+        <v>28.77</v>
       </c>
       <c r="F67" s="2" t="n">
         <v>0</v>
@@ -9027,17 +9087,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
-        <v>0</v>
+        <v>453.32</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>0</v>
+        <v>778.9</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0</v>
+        <v>138.47</v>
       </c>
       <c r="F68" s="2" t="n">
         <v>0</v>
@@ -9054,7 +9114,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>JIMENEZ MORALES JACQUELINE ALEXANDRA</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -9081,7 +9141,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ MORALES JACQUELINE ALEXANDRA</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -9108,7 +9168,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>LAM WONG NELLY ANGELA</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -9135,7 +9195,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>LECANSA S.A.</t>
+          <t>LAM WONG NELLY ANGELA</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -9162,7 +9222,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>LEM S.A.</t>
+          <t>LECANSA S.A.</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -9189,7 +9249,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LEM S.A.</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -9216,7 +9276,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -9243,7 +9303,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -9270,7 +9330,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -9297,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>La Casa Del Coleccionista S.A.S</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -9324,7 +9384,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>La Casa Del Coleccionista S.A.S</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -9351,7 +9411,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -9378,7 +9438,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -9388,7 +9448,7 @@
         <v>0</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>39.4</v>
+        <v>0</v>
       </c>
       <c r="F81" s="2" t="n">
         <v>0</v>
@@ -9405,7 +9465,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -9415,7 +9475,7 @@
         <v>0</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>0</v>
+        <v>39.4</v>
       </c>
       <c r="F82" s="2" t="n">
         <v>0</v>
@@ -9432,7 +9492,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -9459,7 +9519,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>MIELES SAN MARTIN JOHNNY JOEL</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -9486,7 +9546,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MIELES SAN MARTIN JOHNNY JOEL</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -9513,7 +9573,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -9540,7 +9600,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -9567,7 +9627,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -9594,7 +9654,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -9621,7 +9681,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MOSCOSO BLANCO JULIO ENRIQUE</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -9648,7 +9708,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MOSCOSO MORALES ANNIE LISBETH</t>
+          <t>MOSCOSO BLANCO JULIO ENRIQUE</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -9675,14 +9735,14 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOSCOSO MORALES ANNIE LISBETH</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="D92" s="2" t="n">
-        <v>347.34</v>
+        <v>0</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>0</v>
@@ -9702,14 +9762,14 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="D93" s="2" t="n">
-        <v>0</v>
+        <v>347.34</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>0</v>
@@ -9729,7 +9789,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -9756,7 +9816,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -9783,7 +9843,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>OLUNANEK S.A.</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -9810,17 +9870,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>OLUNANEK S.A.</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
-        <v>346.79</v>
+        <v>0</v>
       </c>
       <c r="D97" s="2" t="n">
-        <v>192.19</v>
+        <v>0</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>99.25</v>
+        <v>0</v>
       </c>
       <c r="F97" s="2" t="n">
         <v>0</v>
@@ -9837,17 +9897,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
-        <v>102.69</v>
+        <v>346.79</v>
       </c>
       <c r="D98" s="2" t="n">
-        <v>0</v>
+        <v>192.19</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>0</v>
+        <v>99.25</v>
       </c>
       <c r="F98" s="2" t="n">
         <v>0</v>
@@ -9864,11 +9924,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
-        <v>0</v>
+        <v>102.69</v>
       </c>
       <c r="D99" s="2" t="n">
         <v>0</v>
@@ -9891,7 +9951,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -9918,11 +9978,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
-        <v>58.9</v>
+        <v>0</v>
       </c>
       <c r="D101" s="2" t="n">
         <v>0</v>
@@ -9945,11 +10005,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
-        <v>0</v>
+        <v>58.9</v>
       </c>
       <c r="D102" s="2" t="n">
         <v>0</v>
@@ -9972,7 +10032,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -9982,7 +10042,7 @@
         <v>0</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>2043.13</v>
+        <v>0</v>
       </c>
       <c r="F103" s="2" t="n">
         <v>0</v>
@@ -9999,7 +10059,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>QUIROLA GOMEZ DIEGO FABRICIO</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -10009,7 +10069,7 @@
         <v>0</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>0</v>
+        <v>2043.13</v>
       </c>
       <c r="F104" s="2" t="n">
         <v>0</v>
@@ -10026,7 +10086,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIROLA GOMEZ DIEGO FABRICIO</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -10053,7 +10113,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>RAMOS UGUÑA ERICK FABRICIO</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -10080,7 +10140,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>REALMIND S.A.</t>
+          <t>RAMOS UGUÑA ERICK FABRICIO</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -10107,17 +10167,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>REALMIND S.A.</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
-        <v>1049.35</v>
+        <v>0</v>
       </c>
       <c r="D108" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>2248.94</v>
+        <v>0</v>
       </c>
       <c r="F108" s="2" t="n">
         <v>0</v>
@@ -10134,17 +10194,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
-        <v>0</v>
+        <v>1049.35</v>
       </c>
       <c r="D109" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>0</v>
+        <v>2248.94</v>
       </c>
       <c r="F109" s="2" t="n">
         <v>0</v>
@@ -10161,7 +10221,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -10188,7 +10248,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
@@ -10215,11 +10275,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
-        <v>130.92</v>
+        <v>0</v>
       </c>
       <c r="D112" s="2" t="n">
         <v>0</v>
@@ -10242,11 +10302,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>SILVA BLUM CARLOS ALFREDO</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
-        <v>0</v>
+        <v>130.92</v>
       </c>
       <c r="D113" s="2" t="n">
         <v>0</v>
@@ -10269,7 +10329,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SILVA BLUM CARLOS ALFREDO</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
@@ -10279,7 +10339,7 @@
         <v>0</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>2033.79</v>
+        <v>0</v>
       </c>
       <c r="F114" s="2" t="n">
         <v>0</v>
@@ -10296,7 +10356,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
@@ -10306,7 +10366,7 @@
         <v>0</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>0</v>
+        <v>2033.79</v>
       </c>
       <c r="F115" s="2" t="n">
         <v>0</v>
@@ -10323,7 +10383,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
@@ -10350,11 +10410,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
-        <v>107.46</v>
+        <v>0</v>
       </c>
       <c r="D117" s="2" t="n">
         <v>0</v>
@@ -10377,11 +10437,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="D118" s="2" t="n">
         <v>0</v>
@@ -10404,17 +10464,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D119" s="2" t="n">
-        <v>720.05</v>
+        <v>0</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>392.56</v>
+        <v>0</v>
       </c>
       <c r="F119" s="2" t="n">
         <v>0</v>
@@ -10431,17 +10491,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D120" s="2" t="n">
-        <v>0</v>
+        <v>720.05</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>0</v>
+        <v>392.56</v>
       </c>
       <c r="F120" s="2" t="n">
         <v>0</v>
@@ -10458,7 +10518,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
@@ -10485,14 +10545,14 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D122" s="2" t="n">
-        <v>186.47</v>
+        <v>0</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>0</v>
@@ -10512,14 +10572,14 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D123" s="2" t="n">
-        <v>0</v>
+        <v>186.47</v>
       </c>
       <c r="E123" s="2" t="n">
         <v>0</v>
@@ -10539,14 +10599,14 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
-        <v>50.16</v>
+        <v>0</v>
       </c>
       <c r="D124" s="2" t="n">
-        <v>25.08</v>
+        <v>0</v>
       </c>
       <c r="E124" s="2" t="n">
         <v>0</v>
@@ -10566,14 +10626,14 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
-        <v>0</v>
+        <v>50.16</v>
       </c>
       <c r="D125" s="2" t="n">
-        <v>0</v>
+        <v>25.08</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>0</v>
@@ -10593,14 +10653,14 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
-        <v>176.6</v>
+        <v>0</v>
       </c>
       <c r="D126" s="2" t="n">
-        <v>217.99</v>
+        <v>0</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>0</v>
@@ -10620,14 +10680,14 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
-        <v>0</v>
+        <v>176.6</v>
       </c>
       <c r="D127" s="2" t="n">
-        <v>0</v>
+        <v>217.99</v>
       </c>
       <c r="E127" s="2" t="n">
         <v>0</v>
@@ -10647,7 +10707,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
@@ -10674,7 +10734,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
@@ -10701,7 +10761,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
@@ -10728,7 +10788,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
@@ -10755,11 +10815,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
-        <v>3.94</v>
+        <v>0</v>
       </c>
       <c r="D132" s="2" t="n">
         <v>0</v>
@@ -10782,11 +10842,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
-        <v>0</v>
+        <v>3.94</v>
       </c>
       <c r="D133" s="2" t="n">
         <v>0</v>
@@ -10809,7 +10869,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
@@ -10836,7 +10896,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
@@ -10863,39 +10923,66 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D136" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E136" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F136" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G136" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
           <t>ZUÑIGA BUSTAMANTE ENRIQUE HAMLET</t>
         </is>
       </c>
-      <c r="C136" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D136" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E136" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F136" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G136" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="137">
-      <c r="C137" s="4" t="n">
+      <c r="C137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G137" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="C138" s="4" t="n">
         <v>4858.78</v>
       </c>
-      <c r="D137" s="4" t="n">
+      <c r="D138" s="4" t="n">
         <v>7120.78</v>
       </c>
-      <c r="E137" s="4" t="n">
+      <c r="E138" s="4" t="n">
         <v>8618.370000000001</v>
       </c>
-      <c r="F137" s="4" t="n">
-        <v>3401.44</v>
-      </c>
-      <c r="G137" s="4" t="n">
+      <c r="F138" s="4" t="n">
+        <v>3649.96</v>
+      </c>
+      <c r="G138" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-07-07 08:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -452,7 +452,7 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
@@ -2028,7 +2028,7 @@
         <v>0</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0</v>
+        <v>85.28</v>
       </c>
       <c r="K26" s="2" t="n">
         <v>0</v>
@@ -7193,7 +7193,7 @@
       </c>
       <c r="J112" s="3" t="inlineStr">
         <is>
-          <t>0 de 110</t>
+          <t>1 de 110</t>
         </is>
       </c>
       <c r="K112" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática 2026-07-09 08:30:17
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -2868,7 +2868,7 @@
         <v>0</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0</v>
+        <v>46.82</v>
       </c>
       <c r="K40" s="2" t="n">
         <v>0</v>
@@ -7253,7 +7253,7 @@
       </c>
       <c r="J113" s="3" t="inlineStr">
         <is>
-          <t>1 de 111</t>
+          <t>2 de 111</t>
         </is>
       </c>
       <c r="K113" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática 2026-07-16 08:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R112"/>
+  <dimension ref="A1:R109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BRIONES GOMEZ ASLEY YAMILEXY</t>
+          <t>BRITO MORALES MARIA SOLEDAD</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BRITO MORALES MARIA SOLEDAD</t>
+          <t>BURGOS OLVERA VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BURGOS OLVERA VICENTE JAVIER</t>
+          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
+          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
+          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
+          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
+          <t>CARRANZA AVILEZ WILSON</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CARRANZA AVILEZ WILSON</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CASTRO ALCIVAR EDA MARIA</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1797,7 +1797,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>0</v>
+        <v>36.24</v>
       </c>
       <c r="N22" s="2" t="n">
         <v>0</v>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CASTRO ALCIVAR EDA MARIA</t>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>36.24</v>
+        <v>-36.24</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1883,14 +1883,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
+          <t>CATAECSA S.A.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0</v>
+        <v>612.34</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>0</v>
@@ -1908,7 +1908,7 @@
         <v>0</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0</v>
+        <v>127.92</v>
       </c>
       <c r="K24" s="2" t="n">
         <v>0</v>
@@ -1917,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>-36.24</v>
+        <v>80.05</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -1943,14 +1943,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CATAECSA S.A.</t>
+          <t>CERAMICASAECUADOR S.A.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>612.34</v>
+        <v>0</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>0</v>
@@ -1968,7 +1968,7 @@
         <v>0</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>127.92</v>
+        <v>0</v>
       </c>
       <c r="K25" s="2" t="n">
         <v>0</v>
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>80.05</v>
+        <v>0</v>
       </c>
       <c r="N25" s="2" t="n">
         <v>0</v>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CERAMICASAECUADOR S.A.</t>
+          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
+          <t>CHICA ALBAN GILMERTH HOMERO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CHICA ALBAN GILMERTH HOMERO</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
+          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
+          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
+          <t>CONSTRUMERCADO S.A.</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,14 +2423,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>COQUE TONATO RICHARD PAUL</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0</v>
+        <v>568.71</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>0</v>
@@ -2483,14 +2483,14 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>COQUE TONATO RICHARD PAUL</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>568.71</v>
+        <v>0</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Carlos Meza Peña</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>ECUARECYCLING S.A.</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2748,7 +2748,7 @@
         <v>0</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0</v>
+        <v>46.82</v>
       </c>
       <c r="K38" s="2" t="n">
         <v>0</v>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ECUARECYCLING S.A.</t>
+          <t>EDESA SA</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2808,7 +2808,7 @@
         <v>0</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>46.82</v>
+        <v>0</v>
       </c>
       <c r="K39" s="2" t="n">
         <v>0</v>
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EDESA SA</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>FIENCO VILLACIS NARCISA ROCIO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>FIENCO VILLACIS NARCISA ROCIO</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3213,13 +3213,13 @@
         <v>0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>0</v>
+        <v>88.34</v>
       </c>
       <c r="F46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0</v>
+        <v>65.12</v>
       </c>
       <c r="H46" s="2" t="n">
         <v>0</v>
@@ -3234,10 +3234,10 @@
         <v>0</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>0</v>
+        <v>968.42</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>0</v>
+        <v>1674.61</v>
       </c>
       <c r="N46" s="2" t="n">
         <v>0</v>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3273,13 +3273,13 @@
         <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>88.34</v>
+        <v>0</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>65.12</v>
+        <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
         <v>0</v>
@@ -3294,10 +3294,10 @@
         <v>0</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>968.42</v>
+        <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>1674.61</v>
+        <v>0</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3357,7 +3357,7 @@
         <v>0</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0</v>
+        <v>303.63</v>
       </c>
       <c r="N48" s="2" t="n">
         <v>0</v>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3417,7 +3417,7 @@
         <v>0</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>303.63</v>
+        <v>0</v>
       </c>
       <c r="N49" s="2" t="n">
         <v>0</v>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3717,7 +3717,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0</v>
+        <v>120.53</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3777,7 +3777,7 @@
         <v>0</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>120.53</v>
+        <v>0</v>
       </c>
       <c r="N55" s="2" t="n">
         <v>0</v>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,14 +5363,14 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D82" s="2" t="n">
-        <v>0</v>
+        <v>-1264.02</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>0</v>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,14 +5483,14 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D84" s="2" t="n">
-        <v>-1264.02</v>
+        <v>0</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>0</v>
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -6923,7 +6923,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -6976,264 +6976,84 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
-        </is>
-      </c>
-      <c r="C109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R109" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>ZAZACORP S.A.</t>
-        </is>
-      </c>
-      <c r="C110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R110" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q111" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R111" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="C112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="D112" s="3" t="inlineStr">
-        <is>
-          <t>2 de 110</t>
-        </is>
-      </c>
-      <c r="E112" s="3" t="inlineStr">
-        <is>
-          <t>1 de 110</t>
-        </is>
-      </c>
-      <c r="F112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="G112" s="3" t="inlineStr">
-        <is>
-          <t>1 de 110</t>
-        </is>
-      </c>
-      <c r="H112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="I112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="J112" s="3" t="inlineStr">
-        <is>
-          <t>2 de 110</t>
-        </is>
-      </c>
-      <c r="K112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="L112" s="3" t="inlineStr">
-        <is>
-          <t>1 de 110</t>
-        </is>
-      </c>
-      <c r="M112" s="3" t="inlineStr">
-        <is>
-          <t>6 de 110</t>
-        </is>
-      </c>
-      <c r="N112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="O112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="P112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="Q112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
-        </is>
-      </c>
-      <c r="R112" s="3" t="inlineStr">
-        <is>
-          <t>0 de 110</t>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>2 de 107</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>1 de 107</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>1 de 107</t>
+        </is>
+      </c>
+      <c r="H109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="J109" s="3" t="inlineStr">
+        <is>
+          <t>2 de 107</t>
+        </is>
+      </c>
+      <c r="K109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="L109" s="3" t="inlineStr">
+        <is>
+          <t>1 de 107</t>
+        </is>
+      </c>
+      <c r="M109" s="3" t="inlineStr">
+        <is>
+          <t>6 de 107</t>
+        </is>
+      </c>
+      <c r="N109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="O109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="P109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="Q109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="R109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-07-17 09:30:19
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -2037,7 +2037,7 @@
         <v>0</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>0</v>
+        <v>290.82</v>
       </c>
       <c r="N26" s="2" t="n">
         <v>0</v>
@@ -7028,7 +7028,7 @@
       </c>
       <c r="M109" s="3" t="inlineStr">
         <is>
-          <t>6 de 107</t>
+          <t>7 de 107</t>
         </is>
       </c>
       <c r="N109" s="3" t="inlineStr">
@@ -8029,7 +8029,7 @@
         <v>70.83</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0</v>
+        <v>290.82</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>0</v>
@@ -10800,7 +10800,7 @@
         <v>8618.370000000001</v>
       </c>
       <c r="F138" s="4" t="n">
-        <v>2773.86</v>
+        <v>3064.68</v>
       </c>
       <c r="G138" s="4" t="n">
         <v>0</v>
@@ -10923,13 +10923,13 @@
         <v>20172</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>3051.94</v>
+        <v>3342.76</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>17120.06</v>
+        <v>16829.24</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.1512958556414832</v>
+        <v>0.1657128693238152</v>
       </c>
     </row>
     <row r="5">
@@ -10942,13 +10942,13 @@
         <v>20344.82</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>4837.13</v>
+        <v>5127.950000000001</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>15507.69</v>
+        <v>15216.87</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.2377573259434097</v>
+        <v>0.2520518736464614</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-29 17:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R108"/>
+  <dimension ref="A1:R109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -923,14 +923,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>APOLO GALLARDO RICARDO ISRAEL</t>
+          <t>ANGUETA GAHON ISRRAEL PAUL</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>628.8200000000001</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>0</v>
@@ -957,7 +957,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>248.52</v>
+        <v>0</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>0</v>
@@ -983,7 +983,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ARCE CANDO DENISSE YAJAIRA</t>
+          <t>APOLO GALLARDO RICARDO ISRAEL</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -1017,7 +1017,7 @@
         <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>248.52</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ARMIJO AGUILAR ROBERT LENIN</t>
+          <t>ARCE CANDO DENISSE YAJAIRA</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ARQUITECKSA S.A.</t>
+          <t>ARMIJO AGUILAR ROBERT LENIN</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BRAVO MANZABA MARIA CECILIA</t>
+          <t>ARQUITECKSA S.A.</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BRITO MORALES MARIA SOLEDAD</t>
+          <t>BRAVO MANZABA MARIA CECILIA</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BURGOS OLVERA VICENTE JAVIER</t>
+          <t>BRITO MORALES MARIA SOLEDAD</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
+          <t>BURGOS OLVERA VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
+          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
+          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
+          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CARRANZA AVILEZ WILSON</t>
+          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CARRANZA AVILEZ WILSON</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CASTRO ALCIVAR EDA MARIA</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1797,7 +1797,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>36.24</v>
+        <v>0</v>
       </c>
       <c r="N22" s="2" t="n">
         <v>0</v>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
+          <t>CASTRO ALCIVAR EDA MARIA</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>-36.24</v>
+        <v>36.24</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1883,14 +1883,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CATAECSA S.A.</t>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>612.34</v>
+        <v>0</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>0</v>
@@ -1908,7 +1908,7 @@
         <v>0</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>127.92</v>
+        <v>0</v>
       </c>
       <c r="K24" s="2" t="n">
         <v>0</v>
@@ -1917,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>80.05</v>
+        <v>-36.24</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -1943,14 +1943,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CERAMICASAECUADOR S.A.</t>
+          <t>CATAECSA S.A.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0</v>
+        <v>612.34</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>0</v>
@@ -1968,7 +1968,7 @@
         <v>0</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0</v>
+        <v>127.92</v>
       </c>
       <c r="K25" s="2" t="n">
         <v>0</v>
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>0</v>
+        <v>80.05</v>
       </c>
       <c r="N25" s="2" t="n">
         <v>0</v>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
+          <t>CERAMICASAECUADOR S.A.</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2037,7 +2037,7 @@
         <v>0</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>290.82</v>
+        <v>0</v>
       </c>
       <c r="N26" s="2" t="n">
         <v>0</v>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CHICA ALBAN GILMERTH HOMERO</t>
+          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2097,7 +2097,7 @@
         <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0</v>
+        <v>290.82</v>
       </c>
       <c r="N27" s="2" t="n">
         <v>0</v>
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>CHICA ALBAN GILMERTH HOMERO</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
+          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
+          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,14 +2423,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>COQUE TONATO RICHARD PAUL</t>
+          <t>CONSTRUMERCADO S.A.</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>568.71</v>
+        <v>0</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>0</v>
@@ -2483,14 +2483,14 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Carlos Meza Peña</t>
+          <t>COQUE TONATO RICHARD PAUL</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0</v>
+        <v>568.71</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2634,7 +2634,7 @@
         <v>0</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>189.58</v>
+        <v>0</v>
       </c>
       <c r="M36" s="2" t="n">
         <v>0</v>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2694,7 +2694,7 @@
         <v>0</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>0</v>
+        <v>189.58</v>
       </c>
       <c r="M37" s="2" t="n">
         <v>0</v>
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ECUARECYCLING S.A.</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2748,7 +2748,7 @@
         <v>0</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>46.82</v>
+        <v>0</v>
       </c>
       <c r="K38" s="2" t="n">
         <v>0</v>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EDESA SA</t>
+          <t>ECUARECYCLING S.A.</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2808,7 +2808,7 @@
         <v>0</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0</v>
+        <v>46.82</v>
       </c>
       <c r="K39" s="2" t="n">
         <v>0</v>
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>EDESA SA</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>FIENCO VILLACIS NARCISA ROCIO</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>FIENCO VILLACIS NARCISA ROCIO</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3213,13 +3213,13 @@
         <v>0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>88.34</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>65.12</v>
+        <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
         <v>0</v>
@@ -3234,10 +3234,10 @@
         <v>0</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>968.42</v>
+        <v>0</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>1962.59</v>
+        <v>0</v>
       </c>
       <c r="N46" s="2" t="n">
         <v>0</v>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3273,13 +3273,13 @@
         <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0</v>
+        <v>88.34</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0</v>
+        <v>65.12</v>
       </c>
       <c r="H47" s="2" t="n">
         <v>0</v>
@@ -3294,10 +3294,10 @@
         <v>0</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>0</v>
+        <v>968.42</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0</v>
+        <v>1962.59</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3357,7 +3357,7 @@
         <v>0</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>303.63</v>
+        <v>0</v>
       </c>
       <c r="N48" s="2" t="n">
         <v>0</v>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3417,7 +3417,7 @@
         <v>0</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>0</v>
+        <v>303.63</v>
       </c>
       <c r="N49" s="2" t="n">
         <v>0</v>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3573,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>88.3</v>
+        <v>0</v>
       </c>
       <c r="F52" s="2" t="n">
         <v>0</v>
@@ -3597,7 +3597,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>342.69</v>
+        <v>0</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3633,7 +3633,7 @@
         <v>0</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0</v>
+        <v>88.3</v>
       </c>
       <c r="F53" s="2" t="n">
         <v>0</v>
@@ -3657,7 +3657,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>0</v>
+        <v>342.69</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3717,7 +3717,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>120.53</v>
+        <v>0</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3777,7 +3777,7 @@
         <v>0</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>0</v>
+        <v>120.53</v>
       </c>
       <c r="N55" s="2" t="n">
         <v>0</v>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4854,7 +4854,7 @@
         <v>0</v>
       </c>
       <c r="L73" s="2" t="n">
-        <v>81.90000000000001</v>
+        <v>0</v>
       </c>
       <c r="M73" s="2" t="n">
         <v>0</v>
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4914,7 +4914,7 @@
         <v>0</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>0</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="M74" s="2" t="n">
         <v>0</v>
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,14 +5303,14 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D81" s="2" t="n">
-        <v>-1264.02</v>
+        <v>0</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>0</v>
@@ -5363,14 +5363,14 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D82" s="2" t="n">
-        <v>0</v>
+        <v>-1264.02</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>0</v>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5877,7 +5877,7 @@
         <v>0</v>
       </c>
       <c r="M90" s="2" t="n">
-        <v>23.49</v>
+        <v>0</v>
       </c>
       <c r="N90" s="2" t="n">
         <v>0</v>
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5937,7 +5937,7 @@
         <v>0</v>
       </c>
       <c r="M91" s="2" t="n">
-        <v>0</v>
+        <v>23.49</v>
       </c>
       <c r="N91" s="2" t="n">
         <v>0</v>
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6863,137 +6863,197 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
+          <t>ZAZACORP S.A.</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R107" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
           <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
-      <c r="C107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R107" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="C108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="D108" s="3" t="inlineStr">
-        <is>
-          <t>2 de 106</t>
-        </is>
-      </c>
-      <c r="E108" s="3" t="inlineStr">
-        <is>
-          <t>2 de 106</t>
-        </is>
-      </c>
-      <c r="F108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="G108" s="3" t="inlineStr">
-        <is>
-          <t>1 de 106</t>
-        </is>
-      </c>
-      <c r="H108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="I108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="J108" s="3" t="inlineStr">
-        <is>
-          <t>2 de 106</t>
-        </is>
-      </c>
-      <c r="K108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="L108" s="3" t="inlineStr">
-        <is>
-          <t>3 de 106</t>
-        </is>
-      </c>
-      <c r="M108" s="3" t="inlineStr">
-        <is>
-          <t>9 de 106</t>
-        </is>
-      </c>
-      <c r="N108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="O108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="P108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="Q108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="R108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
+      <c r="C108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R108" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>3 de 107</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>2 de 107</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>1 de 107</t>
+        </is>
+      </c>
+      <c r="H109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="J109" s="3" t="inlineStr">
+        <is>
+          <t>2 de 107</t>
+        </is>
+      </c>
+      <c r="K109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="L109" s="3" t="inlineStr">
+        <is>
+          <t>3 de 107</t>
+        </is>
+      </c>
+      <c r="M109" s="3" t="inlineStr">
+        <is>
+          <t>9 de 107</t>
+        </is>
+      </c>
+      <c r="N109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="O109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="P109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="Q109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
+        </is>
+      </c>
+      <c r="R109" s="3" t="inlineStr">
+        <is>
+          <t>0 de 107</t>
         </is>
       </c>
     </row>
@@ -7321,7 +7381,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0</v>
+        <v>628.8200000000001</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>0</v>
@@ -10740,7 +10800,7 @@
         <v>8618.370000000001</v>
       </c>
       <c r="F138" s="4" t="n">
-        <v>4078.62</v>
+        <v>4707.44</v>
       </c>
       <c r="G138" s="4" t="n">
         <v>0</v>
@@ -10839,10 +10899,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>11104.49</v>
+        <v>11733.31</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-11104.49</v>
+        <v>-11733.31</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -10882,13 +10942,13 @@
         <v>20344.82</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>15291.76</v>
+        <v>15920.58</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5053.060000000001</v>
+        <v>4424.240000000002</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.7516291616244332</v>
+        <v>0.7825372748444076</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-31 10:30:19
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R107"/>
+  <dimension ref="A1:R108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2094,7 +2094,7 @@
         <v>0</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0</v>
+        <v>190.36</v>
       </c>
       <c r="M27" s="2" t="n">
         <v>290.82</v>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6120,7 +6120,7 @@
         <v>0</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0</v>
+        <v>147.45</v>
       </c>
       <c r="O94" s="2" t="n">
         <v>0</v>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,137 +6803,197 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
+          <t>ZAZACORP S.A.</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R106" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
           <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
-      <c r="C106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R106" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="C107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="D107" s="3" t="inlineStr">
-        <is>
-          <t>3 de 105</t>
-        </is>
-      </c>
-      <c r="E107" s="3" t="inlineStr">
-        <is>
-          <t>2 de 105</t>
-        </is>
-      </c>
-      <c r="F107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="G107" s="3" t="inlineStr">
-        <is>
-          <t>1 de 105</t>
-        </is>
-      </c>
-      <c r="H107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="I107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="J107" s="3" t="inlineStr">
-        <is>
-          <t>2 de 105</t>
-        </is>
-      </c>
-      <c r="K107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="L107" s="3" t="inlineStr">
-        <is>
-          <t>3 de 105</t>
-        </is>
-      </c>
-      <c r="M107" s="3" t="inlineStr">
-        <is>
-          <t>9 de 105</t>
-        </is>
-      </c>
-      <c r="N107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="O107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="P107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="Q107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="R107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
+      <c r="C107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R107" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>3 de 106</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>2 de 106</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="G108" s="3" t="inlineStr">
+        <is>
+          <t>1 de 106</t>
+        </is>
+      </c>
+      <c r="H108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="I108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="J108" s="3" t="inlineStr">
+        <is>
+          <t>2 de 106</t>
+        </is>
+      </c>
+      <c r="K108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="L108" s="3" t="inlineStr">
+        <is>
+          <t>4 de 106</t>
+        </is>
+      </c>
+      <c r="M108" s="3" t="inlineStr">
+        <is>
+          <t>9 de 106</t>
+        </is>
+      </c>
+      <c r="N108" s="3" t="inlineStr">
+        <is>
+          <t>1 de 106</t>
+        </is>
+      </c>
+      <c r="O108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="P108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="Q108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
+        </is>
+      </c>
+      <c r="R108" s="3" t="inlineStr">
+        <is>
+          <t>0 de 106</t>
         </is>
       </c>
     </row>
@@ -6948,7 +7008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G138"/>
+  <dimension ref="A1:G139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7909,7 +7969,7 @@
         <v>70.83</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>290.82</v>
+        <v>481.18</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>0</v>
@@ -10299,7 +10359,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
@@ -10312,7 +10372,7 @@
         <v>0</v>
       </c>
       <c r="F124" s="2" t="n">
-        <v>0</v>
+        <v>147.45</v>
       </c>
       <c r="G124" s="2" t="n">
         <v>0</v>
@@ -10326,14 +10386,14 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
-        <v>50.16</v>
+        <v>0</v>
       </c>
       <c r="D125" s="2" t="n">
-        <v>25.08</v>
+        <v>0</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>0</v>
@@ -10353,14 +10413,14 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
-        <v>0</v>
+        <v>50.16</v>
       </c>
       <c r="D126" s="2" t="n">
-        <v>0</v>
+        <v>25.08</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>0</v>
@@ -10380,14 +10440,14 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
-        <v>176.6</v>
+        <v>0</v>
       </c>
       <c r="D127" s="2" t="n">
-        <v>217.99</v>
+        <v>0</v>
       </c>
       <c r="E127" s="2" t="n">
         <v>0</v>
@@ -10407,14 +10467,14 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
-        <v>0</v>
+        <v>176.6</v>
       </c>
       <c r="D128" s="2" t="n">
-        <v>0</v>
+        <v>217.99</v>
       </c>
       <c r="E128" s="2" t="n">
         <v>0</v>
@@ -10434,7 +10494,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
@@ -10461,7 +10521,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
@@ -10488,7 +10548,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
@@ -10515,7 +10575,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
@@ -10542,11 +10602,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
-        <v>3.94</v>
+        <v>0</v>
       </c>
       <c r="D133" s="2" t="n">
         <v>0</v>
@@ -10569,11 +10629,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
-        <v>0</v>
+        <v>3.94</v>
       </c>
       <c r="D134" s="2" t="n">
         <v>0</v>
@@ -10596,7 +10656,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
@@ -10623,7 +10683,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
@@ -10650,39 +10710,66 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G137" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
           <t>ZUÑIGA BUSTAMANTE ENRIQUE HAMLET</t>
         </is>
       </c>
-      <c r="C137" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D137" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E137" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F137" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G137" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="C138" s="4" t="n">
+      <c r="C138" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D138" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E138" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F138" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G138" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="C139" s="4" t="n">
         <v>4858.78</v>
       </c>
-      <c r="D138" s="4" t="n">
+      <c r="D139" s="4" t="n">
         <v>7120.78</v>
       </c>
-      <c r="E138" s="4" t="n">
+      <c r="E139" s="4" t="n">
         <v>8618.370000000001</v>
       </c>
-      <c r="F138" s="4" t="n">
-        <v>4707.44</v>
-      </c>
-      <c r="G138" s="4" t="n">
+      <c r="F139" s="4" t="n">
+        <v>5045.25</v>
+      </c>
+      <c r="G139" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10779,10 +10866,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>11733.31</v>
+        <v>12071.12</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-11733.31</v>
+        <v>-12071.12</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -10822,13 +10909,13 @@
         <v>20344.82</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>15920.58</v>
+        <v>16258.39</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>4424.240000000002</v>
+        <v>4086.43</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.7825372748444076</v>
+        <v>0.7991415013747972</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-04 11:30:16
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -2037,7 +2037,7 @@
         <v>0</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>0</v>
+        <v>1132.88</v>
       </c>
       <c r="N26" s="2" t="n">
         <v>0</v>
@@ -6968,7 +6968,7 @@
       </c>
       <c r="M108" s="3" t="inlineStr">
         <is>
-          <t>0 de 106</t>
+          <t>1 de 106</t>
         </is>
       </c>
       <c r="N108" s="3" t="inlineStr">
@@ -7016,7 +7016,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -7942,7 +7942,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0</v>
+        <v>1132.88</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>0</v>
@@ -10767,7 +10767,7 @@
         <v>5045.25</v>
       </c>
       <c r="F139" s="4" t="n">
-        <v>0</v>
+        <v>1132.88</v>
       </c>
       <c r="G139" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-08-05 13:30:17
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -5817,7 +5817,7 @@
         <v>0</v>
       </c>
       <c r="M89" s="2" t="n">
-        <v>0</v>
+        <v>150.37</v>
       </c>
       <c r="N89" s="2" t="n">
         <v>0</v>
@@ -6968,7 +6968,7 @@
       </c>
       <c r="M108" s="3" t="inlineStr">
         <is>
-          <t>1 de 106</t>
+          <t>2 de 106</t>
         </is>
       </c>
       <c r="N108" s="3" t="inlineStr">
@@ -10264,7 +10264,7 @@
         <v>23.49</v>
       </c>
       <c r="F120" s="2" t="n">
-        <v>0</v>
+        <v>150.37</v>
       </c>
       <c r="G120" s="2" t="n">
         <v>0</v>
@@ -10767,7 +10767,7 @@
         <v>5045.25</v>
       </c>
       <c r="F139" s="4" t="n">
-        <v>1132.88</v>
+        <v>1283.25</v>
       </c>
       <c r="G139" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-08-06 08:30:19
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R108"/>
+  <dimension ref="A1:R107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
+          <t>CARRANZA AVILEZ WILSON</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CARRANZA AVILEZ WILSON</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CASTRO ALCIVAR EDA MARIA</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CASTRO ALCIVAR EDA MARIA</t>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
+          <t>CATAECSA S.A.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1917,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>39.1</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CATAECSA S.A.</t>
+          <t>CERAMICASAECUADOR S.A.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>39.1</v>
+        <v>1132.88</v>
       </c>
       <c r="N25" s="2" t="n">
         <v>0</v>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CERAMICASAECUADOR S.A.</t>
+          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2037,7 +2037,7 @@
         <v>0</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>1132.88</v>
+        <v>0</v>
       </c>
       <c r="N26" s="2" t="n">
         <v>0</v>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
+          <t>CHICA ALBAN GILMERTH HOMERO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CHICA ALBAN GILMERTH HOMERO</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
+          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
+          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
+          <t>CONSTRUMERCADO S.A.</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>COQUE TONATO RICHARD PAUL</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>COQUE TONATO RICHARD PAUL</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Carlos Meza Peña</t>
+          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>ECUARECYCLING S.A.</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ECUARECYCLING S.A.</t>
+          <t>EDESA SA</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EDESA SA</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>FIENCO VILLACIS NARCISA ROCIO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>FIENCO VILLACIS NARCISA ROCIO</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GITI ECUADOR CIA. LTDA.</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GITI ECUADOR CIA. LTDA.</t>
+          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5757,7 +5757,7 @@
         <v>0</v>
       </c>
       <c r="M88" s="2" t="n">
-        <v>0</v>
+        <v>150.37</v>
       </c>
       <c r="N88" s="2" t="n">
         <v>0</v>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5817,7 +5817,7 @@
         <v>0</v>
       </c>
       <c r="M89" s="2" t="n">
-        <v>150.37</v>
+        <v>0</v>
       </c>
       <c r="N89" s="2" t="n">
         <v>0</v>
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -6856,144 +6856,84 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R107" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="C108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="D108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="E108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="F108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="G108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="H108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="I108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="J108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="K108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="L108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="M108" s="3" t="inlineStr">
-        <is>
-          <t>3 de 106</t>
-        </is>
-      </c>
-      <c r="N108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="O108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="P108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="Q108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
-        </is>
-      </c>
-      <c r="R108" s="3" t="inlineStr">
-        <is>
-          <t>0 de 106</t>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="G107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="H107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="J107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="K107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="L107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="M107" s="3" t="inlineStr">
+        <is>
+          <t>3 de 105</t>
+        </is>
+      </c>
+      <c r="N107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="O107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="P107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="Q107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
+        </is>
+      </c>
+      <c r="R107" s="3" t="inlineStr">
+        <is>
+          <t>0 de 105</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-08-07 08:30:15
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R107"/>
+  <dimension ref="A1:R106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ARCE CANDO DENISSE YAJAIRA</t>
+          <t>ARMIJO AGUILAR ROBERT LENIN</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ARMIJO AGUILAR ROBERT LENIN</t>
+          <t>ARQUITECKSA S.A.</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ARQUITECKSA S.A.</t>
+          <t>BRAVO MANZABA MARIA CECILIA</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BRAVO MANZABA MARIA CECILIA</t>
+          <t>BRITO MORALES MARIA SOLEDAD</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BRITO MORALES MARIA SOLEDAD</t>
+          <t>BURGOS OLVERA VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BURGOS OLVERA VICENTE JAVIER</t>
+          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
+          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
+          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
+          <t>CARRANZA AVILEZ WILSON</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CARRANZA AVILEZ WILSON</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CASTRO ALCIVAR EDA MARIA</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CASTRO ALCIVAR EDA MARIA</t>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
+          <t>CATAECSA S.A.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0</v>
+        <v>39.1</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CATAECSA S.A.</t>
+          <t>CERAMICASAECUADOR S.A.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1917,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>39.1</v>
+        <v>1132.88</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CERAMICASAECUADOR S.A.</t>
+          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>1132.88</v>
+        <v>0</v>
       </c>
       <c r="N25" s="2" t="n">
         <v>0</v>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
+          <t>CHICA ALBAN GILMERTH HOMERO</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CHICA ALBAN GILMERTH HOMERO</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
+          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
+          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
+          <t>CONSTRUMERCADO S.A.</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>COQUE TONATO RICHARD PAUL</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>COQUE TONATO RICHARD PAUL</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Carlos Meza Peña</t>
+          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>ECUARECYCLING S.A.</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ECUARECYCLING S.A.</t>
+          <t>EDESA SA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EDESA SA</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>FIENCO VILLACIS NARCISA ROCIO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>FIENCO VILLACIS NARCISA ROCIO</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GITI ECUADOR CIA. LTDA.</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GITI ECUADOR CIA. LTDA.</t>
+          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5697,7 +5697,7 @@
         <v>0</v>
       </c>
       <c r="M87" s="2" t="n">
-        <v>0</v>
+        <v>150.37</v>
       </c>
       <c r="N87" s="2" t="n">
         <v>0</v>
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5757,7 +5757,7 @@
         <v>0</v>
       </c>
       <c r="M88" s="2" t="n">
-        <v>150.37</v>
+        <v>0</v>
       </c>
       <c r="N88" s="2" t="n">
         <v>0</v>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -6796,144 +6796,84 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R106" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="C107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="D107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="E107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="F107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="G107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="H107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="I107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="J107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="K107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="L107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="M107" s="3" t="inlineStr">
-        <is>
-          <t>3 de 105</t>
-        </is>
-      </c>
-      <c r="N107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="O107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="P107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="Q107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
-        </is>
-      </c>
-      <c r="R107" s="3" t="inlineStr">
-        <is>
-          <t>0 de 105</t>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="F106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="G106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="H106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="I106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="J106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="K106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="L106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="M106" s="3" t="inlineStr">
+        <is>
+          <t>3 de 104</t>
+        </is>
+      </c>
+      <c r="N106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="O106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="P106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="Q106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
+        </is>
+      </c>
+      <c r="R106" s="3" t="inlineStr">
+        <is>
+          <t>0 de 104</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-08-13 08:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R106"/>
+  <dimension ref="A1:R105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5637,7 +5637,7 @@
         <v>0</v>
       </c>
       <c r="M86" s="2" t="n">
-        <v>0</v>
+        <v>150.37</v>
       </c>
       <c r="N86" s="2" t="n">
         <v>0</v>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5697,7 +5697,7 @@
         <v>0</v>
       </c>
       <c r="M87" s="2" t="n">
-        <v>150.37</v>
+        <v>0</v>
       </c>
       <c r="N87" s="2" t="n">
         <v>0</v>
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -6736,144 +6736,84 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R105" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="C106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="D106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="E106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="F106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="G106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="H106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="I106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="J106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="K106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="L106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="M106" s="3" t="inlineStr">
-        <is>
-          <t>3 de 104</t>
-        </is>
-      </c>
-      <c r="N106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="O106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="P106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="Q106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
-        </is>
-      </c>
-      <c r="R106" s="3" t="inlineStr">
-        <is>
-          <t>0 de 104</t>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="G105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="H105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="I105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="J105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="K105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="L105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="M105" s="3" t="inlineStr">
+        <is>
+          <t>3 de 103</t>
+        </is>
+      </c>
+      <c r="N105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="O105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="P105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="Q105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
+        </is>
+      </c>
+      <c r="R105" s="3" t="inlineStr">
+        <is>
+          <t>0 de 103</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-08-17 08:30:19
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R105"/>
+  <dimension ref="A1:R104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5577,7 +5577,7 @@
         <v>0</v>
       </c>
       <c r="M85" s="2" t="n">
-        <v>0</v>
+        <v>150.37</v>
       </c>
       <c r="N85" s="2" t="n">
         <v>0</v>
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5637,7 +5637,7 @@
         <v>0</v>
       </c>
       <c r="M86" s="2" t="n">
-        <v>150.37</v>
+        <v>0</v>
       </c>
       <c r="N86" s="2" t="n">
         <v>0</v>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6676,144 +6676,84 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R104" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="C105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="D105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="E105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="F105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="G105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="H105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="I105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="J105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="K105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="L105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="M105" s="3" t="inlineStr">
-        <is>
-          <t>4 de 103</t>
-        </is>
-      </c>
-      <c r="N105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="O105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="P105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="Q105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="R105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="G104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="H104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="I104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="J104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="K104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="L104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="M104" s="3" t="inlineStr">
+        <is>
+          <t>4 de 102</t>
+        </is>
+      </c>
+      <c r="N104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="O104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="P104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="Q104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="R104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-08-20 08:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R105"/>
+  <dimension ref="A1:R104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CABRERA SALAVARRIA PAUL BRUCE</t>
+          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1377,7 +1377,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>24.35</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CALDERON BELTRAN OSWALDO ENRIQUE</t>
+          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1437,7 +1437,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>24.35</v>
+        <v>0</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
+          <t>CARRANZA AVILEZ WILSON</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CARRANZA AVILEZ WILSON</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CASTRO ALCIVAR EDA MARIA</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CASTRO ALCIVAR EDA MARIA</t>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
+          <t>CATAECSA S.A.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1797,7 +1797,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>0</v>
+        <v>39.1</v>
       </c>
       <c r="N22" s="2" t="n">
         <v>0</v>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CATAECSA S.A.</t>
+          <t>CERAMICASAECUADOR S.A.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>39.1</v>
+        <v>1132.88</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CERAMICASAECUADOR S.A.</t>
+          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1917,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>1132.88</v>
+        <v>0</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
+          <t>CHICA ALBAN GILMERTH HOMERO</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CHICA ALBAN GILMERTH HOMERO</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
+          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
+          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
+          <t>CONSTRUMERCADO S.A.</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>COQUE TONATO RICHARD PAUL</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>COQUE TONATO RICHARD PAUL</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Carlos Meza Peña</t>
+          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>ECUARECYCLING S.A.</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ECUARECYCLING S.A.</t>
+          <t>EDESA SA</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>EDESA SA</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>FIENCO VILLACIS NARCISA ROCIO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>FIENCO VILLACIS NARCISA ROCIO</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GITI ECUADOR CIA. LTDA.</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GITI ECUADOR CIA. LTDA.</t>
+          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5517,7 +5517,7 @@
         <v>0</v>
       </c>
       <c r="M84" s="2" t="n">
-        <v>0</v>
+        <v>150.37</v>
       </c>
       <c r="N84" s="2" t="n">
         <v>0</v>
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>TOCAGON PILA ANA ROSA</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5577,7 +5577,7 @@
         <v>0</v>
       </c>
       <c r="M85" s="2" t="n">
-        <v>150.37</v>
+        <v>120.45</v>
       </c>
       <c r="N85" s="2" t="n">
         <v>0</v>
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>TOCAGON PILA ANA ROSA</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5637,7 +5637,7 @@
         <v>0</v>
       </c>
       <c r="M86" s="2" t="n">
-        <v>120.45</v>
+        <v>0</v>
       </c>
       <c r="N86" s="2" t="n">
         <v>0</v>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -6676,144 +6676,84 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q104" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R104" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="C105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="D105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="E105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="F105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="G105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="H105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="I105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="J105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="K105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="L105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="M105" s="3" t="inlineStr">
-        <is>
-          <t>5 de 103</t>
-        </is>
-      </c>
-      <c r="N105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="O105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="P105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="Q105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
-        </is>
-      </c>
-      <c r="R105" s="3" t="inlineStr">
-        <is>
-          <t>0 de 103</t>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="G104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="H104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="I104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="J104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="K104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="L104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="M104" s="3" t="inlineStr">
+        <is>
+          <t>5 de 102</t>
+        </is>
+      </c>
+      <c r="N104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="O104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="P104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="Q104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="R104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-08-25 08:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R103"/>
+  <dimension ref="A1:R104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
+          <t>CALDERON IDROVO WILLIAM GAVINO</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1437,7 +1437,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0</v>
+        <v>237.6</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CARRANZA AVILEZ WILSON</t>
+          <t>CAMPUZANO FAGGISON LILIBETH ISAMAR</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CARRANZA AVILEZ WILSON</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CASTRO ALCIVAR EDA MARIA</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
+          <t>CASTRO ALCIVAR EDA MARIA</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CATAECSA S.A.</t>
+          <t>CASTRO CALDERON VERONICA SOBEIDA</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1797,7 +1797,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>39.1</v>
+        <v>0</v>
       </c>
       <c r="N22" s="2" t="n">
         <v>0</v>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CERAMICASAECUADOR S.A.</t>
+          <t>CATAECSA S.A.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>1132.88</v>
+        <v>39.1</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
+          <t>CERAMICASAECUADOR S.A.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1917,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>1132.88</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CHICA ALBAN GILMERTH HOMERO</t>
+          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>CHICA ALBAN GILMERTH HOMERO</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
+          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
+          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>COQUE TONATO RICHARD PAUL</t>
+          <t>CONSTRUMERCADO S.A.</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Carlos Meza Peña</t>
+          <t>COQUE TONATO RICHARD PAUL</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
+          <t>Carlos Meza Peña</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2517,7 +2517,7 @@
         <v>0</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>5742.21</v>
+        <v>0</v>
       </c>
       <c r="N34" s="2" t="n">
         <v>0</v>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ECUARECYCLING S.A.</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2577,7 +2577,7 @@
         <v>0</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>0</v>
+        <v>5742.21</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EDESA SA</t>
+          <t>ECUARECYCLING S.A.</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>EDESA SA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>FIENCO VILLACIS NARCISA ROCIO</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>FIENCO VILLACIS NARCISA ROCIO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>GITI ECUADOR CIA. LTDA.</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
+          <t>GITI ECUADOR CIA. LTDA.</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GRUPO UNIVERSAL</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GRUPO UNIVERSAL</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MIRANDA COPPIANO JOSE JAVIER</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MIRANDA COPPIANO JOSE JAVIER</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5457,7 +5457,7 @@
         <v>0</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>150.37</v>
+        <v>0</v>
       </c>
       <c r="N83" s="2" t="n">
         <v>0</v>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>TOCAGON PILA ANA ROSA</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5517,7 +5517,7 @@
         <v>0</v>
       </c>
       <c r="M84" s="2" t="n">
-        <v>120.45</v>
+        <v>150.37</v>
       </c>
       <c r="N84" s="2" t="n">
         <v>0</v>
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TOCAGON PILA ANA ROSA</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5577,7 +5577,7 @@
         <v>0</v>
       </c>
       <c r="M85" s="2" t="n">
-        <v>0</v>
+        <v>120.45</v>
       </c>
       <c r="N85" s="2" t="n">
         <v>0</v>
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,137 +6563,197 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
+          <t>ZAZACORP S.A.</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R102" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
           <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
-      <c r="C102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R102" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="C103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="D103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="E103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="F103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="G103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="H103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="I103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="J103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="K103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="L103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="M103" s="3" t="inlineStr">
-        <is>
-          <t>6 de 101</t>
-        </is>
-      </c>
-      <c r="N103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="O103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="P103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="Q103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
-        </is>
-      </c>
-      <c r="R103" s="3" t="inlineStr">
-        <is>
-          <t>0 de 101</t>
+      <c r="C103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R103" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="G104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="H104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="I104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="J104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="K104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="L104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="M104" s="3" t="inlineStr">
+        <is>
+          <t>7 de 102</t>
+        </is>
+      </c>
+      <c r="N104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="O104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="P104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="Q104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
+        </is>
+      </c>
+      <c r="R104" s="3" t="inlineStr">
+        <is>
+          <t>0 de 102</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7440,7 +7500,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
+          <t>CALDERON IDROVO WILLIAM GAVINO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -7453,7 +7513,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>237.6</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -7467,14 +7527,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CARRANZA AVILEZ WILSON</t>
+          <t>CARAVEDO PAZMIÑO  JAHAIRA PAMELA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>107.46</v>
+        <v>0</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>0</v>
@@ -7494,14 +7554,14 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CARRANZA JARA LEONARDO GABRIEL</t>
+          <t>CARRANZA AVILEZ WILSON</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0</v>
+        <v>107.46</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>0</v>
@@ -7521,7 +7581,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CARRION ALVAREZ MARIO ANDRES</t>
+          <t>CARRANZA JARA LEONARDO GABRIEL</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -7548,7 +7608,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CASCO PENA HUGO VLADIMIR</t>
+          <t>CARRION ALVAREZ MARIO ANDRES</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -7575,7 +7635,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
+          <t>CASCO PENA HUGO VLADIMIR</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -7602,7 +7662,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CASTRO CEDILLO BLANCA KARINA</t>
+          <t>CASTILLO CHOEZ CRISTIAN MARIANO</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -7629,11 +7689,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CERAMICASAECUADOR S.A.</t>
+          <t>CASTRO CEDILLO BLANCA KARINA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>1561.97</v>
+        <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>0</v>
@@ -7642,7 +7702,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>1132.88</v>
+        <v>0</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>0</v>
@@ -7656,20 +7716,20 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
+          <t>CERAMICASAECUADOR S.A.</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>314.51</v>
+        <v>1561.97</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>70.83</v>
+        <v>0</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>481.18</v>
+        <v>0</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0</v>
+        <v>1132.88</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>0</v>
@@ -7683,17 +7743,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CHICA ALBAN GILMERTH HOMERO</t>
+          <t>CEVALLOS SOTOMAYOR NADHIA KATHERINE</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0</v>
+        <v>314.51</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0</v>
+        <v>70.83</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0</v>
+        <v>481.18</v>
       </c>
       <c r="F36" s="2" t="n">
         <v>0</v>
@@ -7710,7 +7770,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>COBO FOLLECO JORGE ERNESTO</t>
+          <t>CHICA ALBAN GILMERTH HOMERO</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -7737,7 +7797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
+          <t>COBO FOLLECO JORGE ERNESTO</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -7764,7 +7824,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
+          <t>COMERCIAL MAYA COMPAÑIA LIMITADA</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -7791,7 +7851,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTE DE CARGA PESADA ALAY EXPRESS S.A.</t>
+          <t>COMPAÑIA DE CARGA PESADA Y MANTENIMIENTO VIAL ANGUETRANS S.A</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -7818,7 +7878,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
+          <t>COMPAÑIA DE TRANSPORTE DE CARGA PESADA ALAY EXPRESS S.A.</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -7845,14 +7905,14 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CONSTRUMERCADO S.A.</t>
+          <t>COMPAÑIA DE TRANSPORTES MORA&amp;CASTRO TRANSMORACASTRO C.A.</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>320.79</v>
+        <v>0</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>0</v>
@@ -7872,14 +7932,14 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CONTRERAS JIMMY</t>
+          <t>CONSTRUMERCADO S.A.</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0</v>
+        <v>320.79</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>0</v>
@@ -7899,7 +7959,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>COQUE TONATO RICHARD PAUL</t>
+          <t>CONTRERAS JIMMY</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -7909,7 +7969,7 @@
         <v>0</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>568.71</v>
+        <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
         <v>0</v>
@@ -7926,7 +7986,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
+          <t>COQUE TONATO RICHARD PAUL</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -7936,7 +7996,7 @@
         <v>0</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0</v>
+        <v>568.71</v>
       </c>
       <c r="F45" s="2" t="n">
         <v>0</v>
@@ -7953,7 +8013,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
+          <t>DANIELA ELIZABETH BECERRA BECERRA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -7963,7 +8023,7 @@
         <v>0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>189.58</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
         <v>0</v>
@@ -7980,20 +8040,20 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ECUAFERRI S.A.</t>
+          <t>ECHEVERRIA MEJIA MADELEINE JAZMIN</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>3030.4</v>
+        <v>0</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>445.73</v>
+        <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0</v>
+        <v>189.58</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>5742.21</v>
+        <v>0</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>0</v>
@@ -8007,20 +8067,20 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EDESA SA</t>
+          <t>ECUAFERRI S.A.</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>0</v>
+        <v>3030.4</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>503.56</v>
+        <v>445.73</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0</v>
+        <v>5742.21</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>0</v>
@@ -8034,14 +8094,14 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ELITESERVI S.A.</t>
+          <t>EDESA SA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0</v>
+        <v>503.56</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>0</v>
@@ -8061,7 +8121,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EQUISAB S.A.</t>
+          <t>ELITESERVI S.A.</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -8088,7 +8148,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
+          <t>EQUISAB S.A.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -8115,7 +8175,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
+          <t>ESPINOSA PAZUNA FREDDY PATRICIO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -8142,7 +8202,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
+          <t>ESTUPINAN MERA ROMINA STEFANIA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -8169,7 +8229,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>FERNANDEZ VILLARREAL MARIELA JACQUELINE</t>
+          <t>FARIAS CAICEDO GABRIELA PATRICIA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -8196,14 +8256,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>FIENCO VILLACIS NARCISA ROCIO</t>
+          <t>FERNANDEZ VILLARREAL MARIELA JACQUELINE</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>92.81999999999999</v>
+        <v>0</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>0</v>
@@ -8223,14 +8283,14 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>GALERIAS SU CASA GALESA S.A.</t>
+          <t>FIENCO VILLACIS NARCISA ROCIO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>293.94</v>
+        <v>0</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>0</v>
+        <v>92.81999999999999</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>0</v>
@@ -8250,17 +8310,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
+          <t>GALERIAS SU CASA GALESA S.A.</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>0</v>
+        <v>293.94</v>
       </c>
       <c r="D57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>3084.47</v>
+        <v>0</v>
       </c>
       <c r="F57" s="2" t="n">
         <v>0</v>
@@ -8277,7 +8337,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>GARCES MORALES ANA CRISTINA</t>
+          <t>GAMA BUSSINES, GAMBUSSI S.A.</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -8287,7 +8347,7 @@
         <v>0</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0</v>
+        <v>3084.47</v>
       </c>
       <c r="F58" s="2" t="n">
         <v>0</v>
@@ -8304,7 +8364,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
+          <t>GARCES MORALES ANA CRISTINA</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -8331,7 +8391,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
+          <t>GONZALEZ CASTRO OMARY MICHELLE</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -8341,7 +8401,7 @@
         <v>0</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>303.63</v>
+        <v>0</v>
       </c>
       <c r="F60" s="2" t="n">
         <v>0</v>
@@ -8358,7 +8418,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>GONZALO CORDOVA ALVARADO</t>
+          <t>GONZALEZ VELASCO MARLON MAURICIO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -8368,7 +8428,7 @@
         <v>0</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>0</v>
+        <v>303.63</v>
       </c>
       <c r="F61" s="2" t="n">
         <v>0</v>
@@ -8385,7 +8445,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
+          <t>GONZALO CORDOVA ALVARADO</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -8412,7 +8472,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>HILL PEÑA JONATHAN STUART</t>
+          <t>GUERRERO GARCIA OLIMPIA ANNABELLE</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -8439,17 +8499,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>INMOBIRCOMSA S.A.</t>
+          <t>HILL PEÑA JONATHAN STUART</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>116.77</v>
+        <v>0</v>
       </c>
       <c r="D64" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>430.99</v>
+        <v>0</v>
       </c>
       <c r="F64" s="2" t="n">
         <v>0</v>
@@ -8466,17 +8526,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>IPAC S.A.</t>
+          <t>INMOBIRCOMSA S.A.</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>0</v>
+        <v>116.77</v>
       </c>
       <c r="D65" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0</v>
+        <v>430.99</v>
       </c>
       <c r="F65" s="2" t="n">
         <v>0</v>
@@ -8493,7 +8553,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ISTARTDIGITAL S.A.</t>
+          <t>IPAC S.A.</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -8503,7 +8563,7 @@
         <v>0</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>120.53</v>
+        <v>0</v>
       </c>
       <c r="F66" s="2" t="n">
         <v>0</v>
@@ -8520,17 +8580,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>JAIME COELLO ALBERTO FERNANDO</t>
+          <t>ISTARTDIGITAL S.A.</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>28.77</v>
+        <v>0</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>0</v>
+        <v>120.53</v>
       </c>
       <c r="F67" s="2" t="n">
         <v>0</v>
@@ -8547,14 +8607,14 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>JIMARE DESIGN S.A.S.</t>
+          <t>JAIME COELLO ALBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
-        <v>778.9</v>
+        <v>0</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>138.47</v>
+        <v>28.77</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>0</v>
@@ -8574,14 +8634,14 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
+          <t>JIMARE DESIGN S.A.S.</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
-        <v>0</v>
+        <v>778.9</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>0</v>
+        <v>138.47</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>0</v>
@@ -8601,7 +8661,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>JIMENEZ MORALES JACQUELINE ALEXANDRA</t>
+          <t>JIMENEZ CORDERO WILLIAM GUSTAVO</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -8628,7 +8688,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
+          <t>JIMENEZ MORALES JACQUELINE ALEXANDRA</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -8655,7 +8715,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>LAM WONG NELLY ANGELA</t>
+          <t>JUNCO SANCHEZ ARTURO ENRIQUE</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -8682,7 +8742,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>LECANSA S.A.</t>
+          <t>LAM WONG NELLY ANGELA</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -8709,7 +8769,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>LEM S.A.</t>
+          <t>LECANSA S.A.</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -8736,7 +8796,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
+          <t>LEM S.A.</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -8763,7 +8823,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>LOAIZA TINOCO JUAN PABLO</t>
+          <t>LINDAO RODRIGUEZ ANTONIO COLON</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -8790,7 +8850,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
+          <t>LOAIZA TINOCO JUAN PABLO</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -8817,7 +8877,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>LOZANO MOLINA TITO JERSON</t>
+          <t>LOPEZ GARCIA ANGELO EMMANUEL</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -8844,7 +8904,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>La Casa Del Coleccionista S.A.S</t>
+          <t>LOZANO MOLINA TITO JERSON</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -8871,7 +8931,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>MACHARE BARCO LISSETTE STEFANIA</t>
+          <t>La Casa Del Coleccionista S.A.S</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -8898,7 +8958,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
+          <t>MACHARE BARCO LISSETTE STEFANIA</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -8925,14 +8985,14 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
+          <t>MATAMOROS RUBIO DENISSE MICHELLE</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D82" s="2" t="n">
-        <v>39.4</v>
+        <v>0</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>0</v>
@@ -8952,14 +9012,14 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>MERO MERA HECTOR ALEJANDRO</t>
+          <t>MENDOZA COPPIANO LEONARDO ELICIO</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D83" s="2" t="n">
-        <v>0</v>
+        <v>39.4</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>0</v>
@@ -8979,7 +9039,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
+          <t>MERO MERA HECTOR ALEJANDRO</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -9006,7 +9066,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>MIELES SAN MARTIN JOHNNY JOEL</t>
+          <t>MEZA FERNANDEZ JONATHAN ALEXIS</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -9033,7 +9093,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
+          <t>MIELES SAN MARTIN JOHNNY JOEL</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -9060,7 +9120,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>MORALES CAIZA SERGIO IVAN</t>
+          <t>MORA RODRIGUEZ BYRON RIQUELME</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -9087,7 +9147,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MORALES CAIZA SERGIO IVAN</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -9114,7 +9174,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MORAN MARQUEZ DAYSE MARCELA</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -9141,7 +9201,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -9168,7 +9228,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MOSCOSO BLANCO JULIO ENRIQUE</t>
+          <t>MOROCHO PLAZA SHIRLEY AURELIA</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -9195,7 +9255,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>MOSCOSO MORALES ANNIE LISBETH</t>
+          <t>MOSCOSO BLANCO JULIO ENRIQUE</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -9222,11 +9282,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MOSCOSO MORALES ANNIE LISBETH</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
-        <v>347.34</v>
+        <v>0</v>
       </c>
       <c r="D93" s="2" t="n">
         <v>0</v>
@@ -9249,11 +9309,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
-        <v>0</v>
+        <v>347.34</v>
       </c>
       <c r="D94" s="2" t="n">
         <v>0</v>
@@ -9276,7 +9336,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -9303,7 +9363,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -9330,7 +9390,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>OLUNANEK S.A.</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -9357,17 +9417,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>OLUNANEK S.A.</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
-        <v>192.19</v>
+        <v>0</v>
       </c>
       <c r="D98" s="2" t="n">
-        <v>99.25</v>
+        <v>0</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>81.90000000000001</v>
+        <v>0</v>
       </c>
       <c r="F98" s="2" t="n">
         <v>0</v>
@@ -9384,17 +9444,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
-        <v>0</v>
+        <v>192.19</v>
       </c>
       <c r="D99" s="2" t="n">
-        <v>0</v>
+        <v>99.25</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>0</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="F99" s="2" t="n">
         <v>0</v>
@@ -9411,7 +9471,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -9438,7 +9498,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -9465,7 +9525,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -9492,7 +9552,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -9519,14 +9579,14 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>QUIJIJE MENDOZA GENESIS XIOMARA</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D104" s="2" t="n">
-        <v>2043.13</v>
+        <v>0</v>
       </c>
       <c r="E104" s="2" t="n">
         <v>0</v>
@@ -9546,14 +9606,14 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>QUIROLA GOMEZ DIEGO FABRICIO</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D105" s="2" t="n">
-        <v>0</v>
+        <v>2043.13</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>0</v>
@@ -9573,7 +9633,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>QUIROLA GOMEZ DIEGO FABRICIO</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -9600,7 +9660,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>RAMOS UGUÑA ERICK FABRICIO</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -9627,7 +9687,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>REALMIND S.A.</t>
+          <t>RAMOS UGUÑA ERICK FABRICIO</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -9654,17 +9714,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>REALMIND S.A.</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D109" s="2" t="n">
-        <v>2248.94</v>
+        <v>0</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>-1264.02</v>
+        <v>0</v>
       </c>
       <c r="F109" s="2" t="n">
         <v>0</v>
@@ -9681,17 +9741,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D110" s="2" t="n">
-        <v>0</v>
+        <v>2248.94</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>0</v>
+        <v>-1264.02</v>
       </c>
       <c r="F110" s="2" t="n">
         <v>0</v>
@@ -9708,7 +9768,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
@@ -9735,7 +9795,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SALVATIERRA SEGURA JOSELYN XIOMARA</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
@@ -9762,7 +9822,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
@@ -9789,7 +9849,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>SILVA BLUM CARLOS ALFREDO</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
@@ -9816,14 +9876,14 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SILVA BLUM CARLOS ALFREDO</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D115" s="2" t="n">
-        <v>2033.79</v>
+        <v>0</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>0</v>
@@ -9843,14 +9903,14 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>SOLIS OCAMPO DIMAS ABDON</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D116" s="2" t="n">
-        <v>0</v>
+        <v>2033.79</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>0</v>
@@ -9870,7 +9930,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLIS OCAMPO DIMAS ABDON</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
@@ -9897,7 +9957,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
@@ -9924,7 +9984,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
@@ -9951,20 +10011,20 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>SOLORZANO PROAÑO CARLOS ALBERTO</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
-        <v>720.05</v>
+        <v>0</v>
       </c>
       <c r="D120" s="2" t="n">
-        <v>392.56</v>
+        <v>0</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>23.49</v>
+        <v>0</v>
       </c>
       <c r="F120" s="2" t="n">
-        <v>150.37</v>
+        <v>0</v>
       </c>
       <c r="G120" s="2" t="n">
         <v>0</v>
@@ -9978,20 +10038,20 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>TOCAGON PILA ANA ROSA</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
-        <v>0</v>
+        <v>720.05</v>
       </c>
       <c r="D121" s="2" t="n">
-        <v>0</v>
+        <v>392.56</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>0</v>
+        <v>23.49</v>
       </c>
       <c r="F121" s="2" t="n">
-        <v>120.45</v>
+        <v>150.37</v>
       </c>
       <c r="G121" s="2" t="n">
         <v>0</v>
@@ -10005,7 +10065,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TOCAGON PILA ANA ROSA</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
@@ -10018,7 +10078,7 @@
         <v>0</v>
       </c>
       <c r="F122" s="2" t="n">
-        <v>0</v>
+        <v>120.45</v>
       </c>
       <c r="G122" s="2" t="n">
         <v>0</v>
@@ -10032,7 +10092,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
@@ -10059,11 +10119,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
-        <v>186.47</v>
+        <v>0</v>
       </c>
       <c r="D124" s="2" t="n">
         <v>0</v>
@@ -10086,17 +10146,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
-        <v>0</v>
+        <v>186.47</v>
       </c>
       <c r="D125" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>147.45</v>
+        <v>0</v>
       </c>
       <c r="F125" s="2" t="n">
         <v>0</v>
@@ -10113,7 +10173,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
@@ -10123,7 +10183,7 @@
         <v>0</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>0</v>
+        <v>147.45</v>
       </c>
       <c r="F126" s="2" t="n">
         <v>0</v>
@@ -10140,11 +10200,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
-        <v>25.08</v>
+        <v>0</v>
       </c>
       <c r="D127" s="2" t="n">
         <v>0</v>
@@ -10167,11 +10227,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
-        <v>0</v>
+        <v>25.08</v>
       </c>
       <c r="D128" s="2" t="n">
         <v>0</v>
@@ -10194,11 +10254,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
-        <v>217.99</v>
+        <v>0</v>
       </c>
       <c r="D129" s="2" t="n">
         <v>0</v>
@@ -10221,11 +10281,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
-        <v>0</v>
+        <v>217.99</v>
       </c>
       <c r="D130" s="2" t="n">
         <v>0</v>
@@ -10248,7 +10308,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
@@ -10275,7 +10335,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
@@ -10302,7 +10362,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
@@ -10329,7 +10389,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
@@ -10356,7 +10416,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
@@ -10383,7 +10443,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
@@ -10410,7 +10470,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
@@ -10437,7 +10497,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
@@ -10464,39 +10524,66 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G139" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>OFICINA-CATAECSA</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
           <t>ZUÑIGA BUSTAMANTE ENRIQUE HAMLET</t>
         </is>
       </c>
-      <c r="C139" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D139" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E139" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F139" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G139" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="C140" s="4" t="n">
+      <c r="C140" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D140" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E140" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F140" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G140" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="C141" s="4" t="n">
         <v>7120.78</v>
       </c>
-      <c r="D140" s="4" t="n">
+      <c r="D141" s="4" t="n">
         <v>8618.370000000001</v>
       </c>
-      <c r="E140" s="4" t="n">
+      <c r="E141" s="4" t="n">
         <v>5045.25</v>
       </c>
-      <c r="F140" s="4" t="n">
-        <v>7170.26</v>
-      </c>
-      <c r="G140" s="4" t="n">
+      <c r="F141" s="4" t="n">
+        <v>7407.860000000001</v>
+      </c>
+      <c r="G141" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10593,13 +10680,13 @@
         <v>25808</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>7170.26</v>
+        <v>7407.86</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>18637.74</v>
+        <v>18400.14</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.2778309051456913</v>
+        <v>0.2870373527588345</v>
       </c>
     </row>
     <row r="4">
@@ -10612,13 +10699,13 @@
         <v>25808</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>26754.03</v>
+        <v>26991.63</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-946.0299999999988</v>
+        <v>-1183.630000000001</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>1.036656463112213</v>
+        <v>1.045862910725357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-31 08:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R104"/>
+  <dimension ref="A1:R103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MORAN MARQUEZ DAYSE MARCELA</t>
+          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA CRISTHIAN FERNANDO</t>
+          <t>MULTISERVI-CLIMANSA S.A.S.</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MULTISERVI-CLIMANSA S.A.S.</t>
+          <t>MURELO S.A.S.</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MURELO S.A.S.</t>
+          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MUÑOZ CALDERON JUAN ADOLFO</t>
+          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MUÑOZ RODRIGUEZ ANDRY EDWAR</t>
+          <t>PALMA ALONZO OSCAR XAVIER</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PALMA ALONZO OSCAR XAVIER</t>
+          <t>PALMA PICO OSCAR FILIDEL</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PALMA PICO OSCAR FILIDEL</t>
+          <t>PARRALES LIRIANO CARLOS JULIO</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PARRALES LIRIANO CARLOS JULIO</t>
+          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PERDOMO BRIONES JOSÉ ALBERTO</t>
+          <t>PYCCA S.A.</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PYCCA S.A.</t>
+          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>QUIRIZUMBAY ROMERO PATRICIA DE JESUS</t>
+          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>RAMIREZ MOREIRA MAYRA JACQUELINE</t>
+          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>RODRIGUEZ BRAVO KAREN ANDREINA</t>
+          <t>ROSHANN</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ROSHANN</t>
+          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SAMPEDRO TOAQUIZA JUAN CARLOS</t>
+          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SAYAY AGUAYO SEGUNDO JUAN</t>
+          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SILVA YEPEZ CRISTIAN DAYAN</t>
+          <t>SOLIS SOLIS JUAN CARLOS</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SOLIS SOLIS JUAN CARLOS</t>
+          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SOLORZANO CHALEN JESSICA ELIZABETH</t>
+          <t>STOCKTIRE S.A.</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>STOCKTIRE S.A.</t>
+          <t>STROBEL CORDERO MARIA ELISABETH</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>STROBEL CORDERO MARIA ELISABETH</t>
+          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -5457,7 +5457,7 @@
         <v>0</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>0</v>
+        <v>150.37</v>
       </c>
       <c r="N83" s="2" t="n">
         <v>0</v>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>TIENDAS INDUSTRIALES ASOCIADAS TIA S. A.</t>
+          <t>TOCAGON PILA ANA ROSA</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -5517,7 +5517,7 @@
         <v>0</v>
       </c>
       <c r="M84" s="2" t="n">
-        <v>150.37</v>
+        <v>120.45</v>
       </c>
       <c r="N84" s="2" t="n">
         <v>0</v>
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>TOCAGON PILA ANA ROSA</t>
+          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -5577,7 +5577,7 @@
         <v>0</v>
       </c>
       <c r="M85" s="2" t="n">
-        <v>120.45</v>
+        <v>0</v>
       </c>
       <c r="N85" s="2" t="n">
         <v>0</v>
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>TOMALA GONZALEZ LUIS ALBERTO</t>
+          <t>TORRES CADENA JAVIER JOSUE</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>TORRES CADENA JAVIER JOSUE</t>
+          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TORRES ESPINOZA SEBASTIAN ALEXANDER</t>
+          <t>TRACTOMAQ S.A.</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TRACTOMAQ S.A.</t>
+          <t>TULCAN GELLIBERT MARIA ELENA</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TULCAN GELLIBERT MARIA ELENA</t>
+          <t>VACA PANCHI DORYS CAROLINA</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>VACA PANCHI DORYS CAROLINA</t>
+          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>VALLES RUBIO SEGUNDO MELCHOR</t>
+          <t>VARGAS OÑATE NORMA SUSANA</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>VARGAS OÑATE NORMA SUSANA</t>
+          <t>VEHINVER SA</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>VEHINVER SA</t>
+          <t>VERA TREJO JUAN CARLOS</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>VERA TREJO JUAN CARLOS</t>
+          <t>VILLACRES TORRES CLARA IVON</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>VILLACRES TORRES CLARA IVON</t>
+          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>VILLAMAR MANZABA MARGARITA ISABEL</t>
+          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>YANCHAGUANO AREQUIPA ERIKA YESENIA</t>
+          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ZAMBRANO VERDUGA RICARDO IVAN</t>
+          <t>ZAMBRANO ZAMBRANO FATIMA</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ZAMBRANO ZAMBRANO FATIMA</t>
+          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>ZAVALA MENOSCAL HOMERO MIGUEL</t>
+          <t>ZAZACORP S.A.</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ZAZACORP S.A.</t>
+          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -6616,144 +6616,84 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>OFICINA-CATAECSA</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>ZONA FRANCA DE POSORJA ZOFRAPORT S.A</t>
-        </is>
-      </c>
-      <c r="C103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q103" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R103" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="C104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
-        </is>
-      </c>
-      <c r="D104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
-        </is>
-      </c>
-      <c r="E104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
-        </is>
-      </c>
-      <c r="F104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
-        </is>
-      </c>
-      <c r="G104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
-        </is>
-      </c>
-      <c r="H104" s="3" t="inlineStr">
-        <is>
-          <t>1 de 102</t>
-        </is>
-      </c>
-      <c r="I104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
-        </is>
-      </c>
-      <c r="J104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
-        </is>
-      </c>
-      <c r="K104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
-        </is>
-      </c>
-      <c r="L104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
-        </is>
-      </c>
-      <c r="M104" s="3" t="inlineStr">
-        <is>
-          <t>7 de 102</t>
-        </is>
-      </c>
-      <c r="N104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
-        </is>
-      </c>
-      <c r="O104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
-        </is>
-      </c>
-      <c r="P104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
-        </is>
-      </c>
-      <c r="Q104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
-        </is>
-      </c>
-      <c r="R104" s="3" t="inlineStr">
-        <is>
-          <t>0 de 102</t>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
+        </is>
+      </c>
+      <c r="G103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
+        </is>
+      </c>
+      <c r="H103" s="3" t="inlineStr">
+        <is>
+          <t>1 de 101</t>
+        </is>
+      </c>
+      <c r="I103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
+        </is>
+      </c>
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
+        </is>
+      </c>
+      <c r="K103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
+        </is>
+      </c>
+      <c r="L103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
+        </is>
+      </c>
+      <c r="M103" s="3" t="inlineStr">
+        <is>
+          <t>7 de 101</t>
+        </is>
+      </c>
+      <c r="N103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
+        </is>
+      </c>
+      <c r="O103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
+        </is>
+      </c>
+      <c r="P103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
+        </is>
+      </c>
+      <c r="Q103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
+        </is>
+      </c>
+      <c r="R103" s="3" t="inlineStr">
+        <is>
+          <t>0 de 101</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-09-01 17:30:16
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -5457,7 +5457,7 @@
         <v>0</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>0</v>
+        <v>40.12</v>
       </c>
       <c r="N83" s="2" t="n">
         <v>0</v>
@@ -6668,7 +6668,7 @@
       </c>
       <c r="M103" s="3" t="inlineStr">
         <is>
-          <t>0 de 101</t>
+          <t>1 de 101</t>
         </is>
       </c>
       <c r="N103" s="3" t="inlineStr">
@@ -9991,7 +9991,7 @@
         <v>150.37</v>
       </c>
       <c r="F121" s="2" t="n">
-        <v>0</v>
+        <v>40.12</v>
       </c>
       <c r="G121" s="2" t="n">
         <v>0</v>
@@ -10521,7 +10521,7 @@
         <v>8971.120000000001</v>
       </c>
       <c r="F141" s="4" t="n">
-        <v>0</v>
+        <v>40.12</v>
       </c>
       <c r="G141" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-09-02 09:30:17
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -2994,7 +2994,7 @@
         <v>0</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>0</v>
+        <v>645.77</v>
       </c>
       <c r="M42" s="2" t="n">
         <v>0</v>
@@ -6663,7 +6663,7 @@
       </c>
       <c r="L103" s="3" t="inlineStr">
         <is>
-          <t>0 de 101</t>
+          <t>1 de 101</t>
         </is>
       </c>
       <c r="M103" s="3" t="inlineStr">
@@ -8263,7 +8263,7 @@
         <v>0</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0</v>
+        <v>645.77</v>
       </c>
       <c r="G57" s="2" t="n">
         <v>0</v>
@@ -10521,7 +10521,7 @@
         <v>8971.120000000001</v>
       </c>
       <c r="F141" s="4" t="n">
-        <v>40.12</v>
+        <v>685.89</v>
       </c>
       <c r="G141" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-09-02 11:30:19
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -1971,7 +1971,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>0</v>
+        <v>2.15</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>0</v>
@@ -6658,7 +6658,7 @@
       </c>
       <c r="K103" s="3" t="inlineStr">
         <is>
-          <t>0 de 101</t>
+          <t>1 de 101</t>
         </is>
       </c>
       <c r="L103" s="3" t="inlineStr">
@@ -7696,7 +7696,7 @@
         <v>0</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0</v>
+        <v>2.15</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>0</v>
@@ -10521,7 +10521,7 @@
         <v>8971.120000000001</v>
       </c>
       <c r="F141" s="4" t="n">
-        <v>685.89</v>
+        <v>688.04</v>
       </c>
       <c r="G141" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-09-04 15:30:15
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -2337,7 +2337,7 @@
         <v>0</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>0</v>
+        <v>136.39</v>
       </c>
       <c r="N31" s="2" t="n">
         <v>0</v>
@@ -6668,7 +6668,7 @@
       </c>
       <c r="M103" s="3" t="inlineStr">
         <is>
-          <t>1 de 101</t>
+          <t>2 de 101</t>
         </is>
       </c>
       <c r="N103" s="3" t="inlineStr">
@@ -7885,7 +7885,7 @@
         <v>0</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0</v>
+        <v>136.39</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>0</v>
@@ -10521,7 +10521,7 @@
         <v>8971.120000000001</v>
       </c>
       <c r="F141" s="4" t="n">
-        <v>688.04</v>
+        <v>824.4299999999999</v>
       </c>
       <c r="G141" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-09-11 12:30:18
</commit_message>
<xml_diff>
--- a/data/OFICINA-CATAECSA.xlsx
+++ b/data/OFICINA-CATAECSA.xlsx
@@ -2502,10 +2502,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>0</v>
+        <v>724.5</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0</v>
+        <v>637.01</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0</v>
@@ -6583,12 +6583,12 @@
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>1 de 100</t>
+          <t>2 de 100</t>
         </is>
       </c>
       <c r="I102" s="3" t="inlineStr">
         <is>
-          <t>1 de 100</t>
+          <t>2 de 100</t>
         </is>
       </c>
       <c r="J102" s="3" t="inlineStr">
@@ -7933,7 +7933,7 @@
         <v>5742.21</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0</v>
+        <v>1361.51</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>0</v>
@@ -10434,7 +10434,7 @@
         <v>8971.120000000001</v>
       </c>
       <c r="F140" s="4" t="n">
-        <v>1037.41</v>
+        <v>2398.92</v>
       </c>
       <c r="G140" s="4" t="n">
         <v>0</v>
@@ -10533,10 +10533,10 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-9.58</v>
+        <v>1351.93</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.58</v>
+        <v>-1351.93</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -10600,13 +10600,13 @@
         <v>37067</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1958.14</v>
+        <v>3319.650000000001</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>35108.86</v>
+        <v>33747.35</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.05282704292227588</v>
+        <v>0.08955809749912322</v>
       </c>
     </row>
   </sheetData>

</xml_diff>